<commit_message>
Label Grove Collaborative supplies separately from 827 N Grove.
User: “grove orders” means Grove Collaborative, not the 827 N Grove house.
Prime Grove Collaborative $791.21 stays on 524 Unit 2 SUPPLIES. The HD/Lowe’s/IKEA
1/3 ($604.12) stays on the 827 N Grove house tab as the Q5 split.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
+++ b/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
@@ -596,7 +596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -784,6 +784,18 @@
       <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Bundled home+auto (was Travelers home / Geico auto). HOME share $1105.46 on 524 INSURANCE 50/50 U1/U2 (yellow proxy from Feb $157.53/$145.25). AUTO share $1019.33 + Geico credit $540.89 EXCLUDED personal. No 2025 Travelers found. No Sep–Dec SF on Prime. Not tax advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>Grove Collaborative 2026-09-18</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>User: “grove orders” = Grove Collaborative, not 827 N Grove the house. Prime $791.21 already on 524 Unit 2 SUPPLIES (8 charges). HD/Lowe’s/IKEA 1/3 $604.12 stays on 827 N Grove the house (Q5), not mixed into Grove Collaborative. Betty’s Pizza / KS Grove is personal dining. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -3376,6 +3388,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -3485,10 +3498,11 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="51" t="inlineStr">
         <is>
-          <t>Prime HD / Lowe’s / IKEA — Grove 1/3 (user split 2026-09-18)</t>
+          <t>Prime HD / Lowe’s / IKEA — 827 N Grove the house 1/3 (NOT Grove Collaborative supplies)</t>
         </is>
       </c>
     </row>
@@ -3704,10 +3718,11 @@
         <v>604.12</v>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>CPA: this 1/3 is pre-close hardware/furniture (close 2025-12-18). Do NOT fold into locked TY2025 CapEx $53,660 (the 2025-12-19 contractor payments) until you say so. May be additional 827 basis / CapEx / personal — FLAG.</t>
+          <t>CPA: this 1/3 is pre-close hardware/furniture for 827 N Grove the house (close 2025-12-18). This is NOT Grove Collaborative. Do NOT fold into locked TY2025 CapEx $53,660 (the 2025-12-19 contractor payments) until you say so. May be additional 827 basis / CapEx / personal — FLAG.</t>
         </is>
       </c>
     </row>
@@ -6040,7 +6055,7 @@
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>Grove 8 orders</t>
+          <t>Jan/Mar/Apr/Jun/Jul/Aug/Sep</t>
         </is>
       </c>
       <c r="C55" s="11" t="inlineStr">
@@ -6068,7 +6083,7 @@
       </c>
       <c r="H55" s="11" t="inlineStr">
         <is>
-          <t>User example; Aug tagged Business in Monarch</t>
+          <t>User 2026-09-18: “grove orders” = Grove Collaborative, not 827 N Grove the house. 8 Prime charges → 524 Unit 2 SUPPLIES.</t>
         </is>
       </c>
     </row>
@@ -6808,7 +6823,7 @@
       </c>
       <c r="H74" s="11" t="inlineStr">
         <is>
-          <t>1/3 524 repairs / 1/3 personal / 1/3 827 Grove (by transaction) → U2 $5.67 / U1 $5.67</t>
+          <t>1/3 524 repairs / 1/3 personal / 1/3 827 N Grove the house (by transaction) → U2 $5.67 / U1 $5.67</t>
         </is>
       </c>
     </row>
@@ -6873,7 +6888,7 @@
       </c>
       <c r="E76" s="35" t="inlineStr">
         <is>
-          <t>827 Grove materials</t>
+          <t>827 N Grove the house (not Grove Collaborative)</t>
         </is>
       </c>
       <c r="F76" s="35" t="inlineStr">
@@ -6888,7 +6903,7 @@
       </c>
       <c r="H76" s="35" t="inlineStr">
         <is>
-          <t>1/3 of txn. Pre-close materials — NOT folded into locked TY2025 CapEx $53,660.</t>
+          <t>1/3 of txn for 827 N Grove the house. Pre-close materials — NOT Grove Collaborative supplies. NOT folded into locked TY2025 CapEx $53,660.</t>
         </is>
       </c>
     </row>
@@ -6928,7 +6943,7 @@
       </c>
       <c r="H77" s="11" t="inlineStr">
         <is>
-          <t>1/3 524 repairs / 1/3 personal / 1/3 827 Grove (by transaction) → U2 $49.90 / U1 $49.89</t>
+          <t>1/3 524 repairs / 1/3 personal / 1/3 827 N Grove the house (by transaction) → U2 $49.90 / U1 $49.89</t>
         </is>
       </c>
     </row>
@@ -6993,7 +7008,7 @@
       </c>
       <c r="E79" s="35" t="inlineStr">
         <is>
-          <t>827 Grove materials</t>
+          <t>827 N Grove the house (not Grove Collaborative)</t>
         </is>
       </c>
       <c r="F79" s="35" t="inlineStr">
@@ -7008,7 +7023,7 @@
       </c>
       <c r="H79" s="35" t="inlineStr">
         <is>
-          <t>1/3 of txn. Pre-close materials — NOT folded into locked TY2025 CapEx $53,660.</t>
+          <t>1/3 of txn for 827 N Grove the house. Pre-close materials — NOT Grove Collaborative supplies. NOT folded into locked TY2025 CapEx $53,660.</t>
         </is>
       </c>
     </row>
@@ -7048,7 +7063,7 @@
       </c>
       <c r="H80" s="11" t="inlineStr">
         <is>
-          <t>1/3 524 repairs / 1/3 personal / 1/3 827 Grove (by transaction) → U2 $11.00 / U1 $11.00</t>
+          <t>1/3 524 repairs / 1/3 personal / 1/3 827 N Grove the house (by transaction) → U2 $11.00 / U1 $11.00</t>
         </is>
       </c>
     </row>
@@ -7113,7 +7128,7 @@
       </c>
       <c r="E82" s="35" t="inlineStr">
         <is>
-          <t>827 Grove materials</t>
+          <t>827 N Grove the house (not Grove Collaborative)</t>
         </is>
       </c>
       <c r="F82" s="35" t="inlineStr">
@@ -7128,7 +7143,7 @@
       </c>
       <c r="H82" s="35" t="inlineStr">
         <is>
-          <t>1/3 of txn. Pre-close materials — NOT folded into locked TY2025 CapEx $53,660.</t>
+          <t>1/3 of txn for 827 N Grove the house. Pre-close materials — NOT Grove Collaborative supplies. NOT folded into locked TY2025 CapEx $53,660.</t>
         </is>
       </c>
     </row>
@@ -7168,7 +7183,7 @@
       </c>
       <c r="H83" s="11" t="inlineStr">
         <is>
-          <t>1/3 524 repairs / 1/3 personal / 1/3 827 Grove (by transaction) → U2 $9.29 / U1 $9.28</t>
+          <t>1/3 524 repairs / 1/3 personal / 1/3 827 N Grove the house (by transaction) → U2 $9.29 / U1 $9.28</t>
         </is>
       </c>
     </row>
@@ -7233,7 +7248,7 @@
       </c>
       <c r="E85" s="35" t="inlineStr">
         <is>
-          <t>827 Grove materials</t>
+          <t>827 N Grove the house (not Grove Collaborative)</t>
         </is>
       </c>
       <c r="F85" s="35" t="inlineStr">
@@ -7248,7 +7263,7 @@
       </c>
       <c r="H85" s="35" t="inlineStr">
         <is>
-          <t>1/3 of txn. Pre-close materials — NOT folded into locked TY2025 CapEx $53,660.</t>
+          <t>1/3 of txn for 827 N Grove the house. Pre-close materials — NOT Grove Collaborative supplies. NOT folded into locked TY2025 CapEx $53,660.</t>
         </is>
       </c>
     </row>
@@ -7288,7 +7303,7 @@
       </c>
       <c r="H86" s="11" t="inlineStr">
         <is>
-          <t>1/3 524 repairs / 1/3 personal / 1/3 827 Grove (by transaction) → U2 $39.40 / U1 $39.39</t>
+          <t>1/3 524 repairs / 1/3 personal / 1/3 827 N Grove the house (by transaction) → U2 $39.40 / U1 $39.39</t>
         </is>
       </c>
     </row>
@@ -7353,7 +7368,7 @@
       </c>
       <c r="E88" s="35" t="inlineStr">
         <is>
-          <t>827 Grove materials</t>
+          <t>827 N Grove the house (not Grove Collaborative)</t>
         </is>
       </c>
       <c r="F88" s="35" t="inlineStr">
@@ -7368,7 +7383,7 @@
       </c>
       <c r="H88" s="35" t="inlineStr">
         <is>
-          <t>1/3 of txn. Pre-close materials — NOT folded into locked TY2025 CapEx $53,660.</t>
+          <t>1/3 of txn for 827 N Grove the house. Pre-close materials — NOT Grove Collaborative supplies. NOT folded into locked TY2025 CapEx $53,660.</t>
         </is>
       </c>
     </row>
@@ -7408,7 +7423,7 @@
       </c>
       <c r="H89" s="11" t="inlineStr">
         <is>
-          <t>1/3 524 repairs / 1/3 personal / 1/3 827 Grove (by transaction) → U2 $0.18 / U1 $0.18</t>
+          <t>1/3 524 repairs / 1/3 personal / 1/3 827 N Grove the house (by transaction) → U2 $0.18 / U1 $0.18</t>
         </is>
       </c>
     </row>
@@ -7473,7 +7488,7 @@
       </c>
       <c r="E91" s="35" t="inlineStr">
         <is>
-          <t>827 Grove materials</t>
+          <t>827 N Grove the house (not Grove Collaborative)</t>
         </is>
       </c>
       <c r="F91" s="35" t="inlineStr">
@@ -7488,7 +7503,7 @@
       </c>
       <c r="H91" s="35" t="inlineStr">
         <is>
-          <t>1/3 of txn. Pre-close materials — NOT folded into locked TY2025 CapEx $53,660.</t>
+          <t>1/3 of txn for 827 N Grove the house. Pre-close materials — NOT Grove Collaborative supplies. NOT folded into locked TY2025 CapEx $53,660.</t>
         </is>
       </c>
     </row>
@@ -7528,7 +7543,7 @@
       </c>
       <c r="H92" s="11" t="inlineStr">
         <is>
-          <t>1/3 524 repairs / 1/3 personal / 1/3 827 Grove (by transaction) → U2 $50.99 / U1 $50.99</t>
+          <t>1/3 524 repairs / 1/3 personal / 1/3 827 N Grove the house (by transaction) → U2 $50.99 / U1 $50.99</t>
         </is>
       </c>
     </row>
@@ -7593,7 +7608,7 @@
       </c>
       <c r="E94" s="35" t="inlineStr">
         <is>
-          <t>827 Grove materials</t>
+          <t>827 N Grove the house (not Grove Collaborative)</t>
         </is>
       </c>
       <c r="F94" s="35" t="inlineStr">
@@ -7608,7 +7623,7 @@
       </c>
       <c r="H94" s="35" t="inlineStr">
         <is>
-          <t>1/3 of txn. Pre-close materials — NOT folded into locked TY2025 CapEx $53,660.</t>
+          <t>1/3 of txn for 827 N Grove the house. Pre-close materials — NOT Grove Collaborative supplies. NOT folded into locked TY2025 CapEx $53,660.</t>
         </is>
       </c>
     </row>
@@ -7648,7 +7663,7 @@
       </c>
       <c r="H95" s="11" t="inlineStr">
         <is>
-          <t>1/3 524 repairs / 1/3 personal / 1/3 827 Grove (by transaction) → U2 $34.87 / U1 $34.86</t>
+          <t>1/3 524 repairs / 1/3 personal / 1/3 827 N Grove the house (by transaction) → U2 $34.87 / U1 $34.86</t>
         </is>
       </c>
     </row>
@@ -7713,7 +7728,7 @@
       </c>
       <c r="E97" s="35" t="inlineStr">
         <is>
-          <t>827 Grove materials</t>
+          <t>827 N Grove the house (not Grove Collaborative)</t>
         </is>
       </c>
       <c r="F97" s="35" t="inlineStr">
@@ -7728,7 +7743,7 @@
       </c>
       <c r="H97" s="35" t="inlineStr">
         <is>
-          <t>1/3 of txn. Pre-close materials — NOT folded into locked TY2025 CapEx $53,660.</t>
+          <t>1/3 of txn for 827 N Grove the house. Pre-close materials — NOT Grove Collaborative supplies. NOT folded into locked TY2025 CapEx $53,660.</t>
         </is>
       </c>
     </row>
@@ -7768,7 +7783,7 @@
       </c>
       <c r="H98" s="11" t="inlineStr">
         <is>
-          <t>1/3 524 repairs / 1/3 personal / 1/3 827 Grove (by transaction) → U2 $68.48 / U1 $68.48</t>
+          <t>1/3 524 repairs / 1/3 personal / 1/3 827 N Grove the house (by transaction) → U2 $68.48 / U1 $68.48</t>
         </is>
       </c>
     </row>
@@ -7833,7 +7848,7 @@
       </c>
       <c r="E100" s="35" t="inlineStr">
         <is>
-          <t>827 Grove materials</t>
+          <t>827 N Grove the house (not Grove Collaborative)</t>
         </is>
       </c>
       <c r="F100" s="35" t="inlineStr">
@@ -7848,7 +7863,7 @@
       </c>
       <c r="H100" s="35" t="inlineStr">
         <is>
-          <t>1/3 of txn. Pre-close materials — NOT folded into locked TY2025 CapEx $53,660.</t>
+          <t>1/3 of txn for 827 N Grove the house. Pre-close materials — NOT Grove Collaborative supplies. NOT folded into locked TY2025 CapEx $53,660.</t>
         </is>
       </c>
     </row>
@@ -7888,7 +7903,7 @@
       </c>
       <c r="H101" s="11" t="inlineStr">
         <is>
-          <t>1/3 524 repairs / 1/3 personal / 1/3 827 Grove (by transaction) → U2 $32.33 / U1 $32.33</t>
+          <t>1/3 524 repairs / 1/3 personal / 1/3 827 N Grove the house (by transaction) → U2 $32.33 / U1 $32.33</t>
         </is>
       </c>
     </row>
@@ -7953,7 +7968,7 @@
       </c>
       <c r="E103" s="35" t="inlineStr">
         <is>
-          <t>827 Grove materials</t>
+          <t>827 N Grove the house (not Grove Collaborative)</t>
         </is>
       </c>
       <c r="F103" s="35" t="inlineStr">
@@ -7968,7 +7983,7 @@
       </c>
       <c r="H103" s="35" t="inlineStr">
         <is>
-          <t>1/3 of txn. Pre-close materials — NOT folded into locked TY2025 CapEx $53,660.</t>
+          <t>1/3 of txn for 827 N Grove the house. Pre-close materials — NOT Grove Collaborative supplies. NOT folded into locked TY2025 CapEx $53,660.</t>
         </is>
       </c>
     </row>
@@ -8015,7 +8030,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>STATUS: APPLIED = monthly P&amp;L. EXCLUDED = personal. HOLD = still confirm. INVENTORY = Art Sales (not P&amp;L, not Cost total yet). TBD-MEGAN = ComEd — remind Jacob to ask Megan. GROVE-SPLIT = 827 materials, not locked $53,660.</t>
+          <t>STATUS: APPLIED = monthly P&amp;L. EXCLUDED = personal. HOLD = still confirm. INVENTORY = Art Sales (not P&amp;L, not Cost total yet). TBD-MEGAN = ComEd — remind Jacob to ask Megan. GROVE-SPLIT = 827 N Grove the house materials (not Grove Collaborative), not locked $53,660.</t>
         </is>
       </c>
     </row>
@@ -8035,10 +8050,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="64" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="1" max="1"/>
     <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -8196,281 +8211,303 @@
       </c>
       <c r="B15" s="39" t="inlineStr">
         <is>
-          <t>CONFIRMED split by transaction 1/3 524 / 1/3 personal / 1/3 Grove. Remaining $1812.46. Extra Space $360 HOLD.</t>
+          <t>CONFIRMED split by transaction 1/3 524 repairs / 1/3 personal / 1/3 827 N Grove the house (NOT Grove Collaborative). Remaining $1812.46. Extra Space $360 HOLD.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="39" t="inlineStr">
         <is>
+          <t>Grove Collaborative orders</t>
+        </is>
+      </c>
+      <c r="B16" s="39" t="inlineStr">
+        <is>
+          <t>CONFIRMED. “Grove orders” = Grove Collaborative supplies, not 827 N Grove the house. Prime $791.21 → 524 Unit 2 SUPPLIES (8 charges). Betty’s Pizza / KS Grove is unrelated (personal dining).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="39" t="inlineStr">
+        <is>
           <t>State Farm bundled home + auto</t>
         </is>
       </c>
-      <c r="B16" s="39" t="inlineStr">
+      <c r="B17" s="39" t="inlineStr">
         <is>
           <t>CONFIRMED. Previously home=Travelers, car=Geico. Only the HOME share of Prime State Farm is on 524 INSURANCE (50/50 U1/U2, yellow). Auto share and Geico $540.89 credit are personal. Split uses Feb 11 unbundled $157.53 home / $145.25 auto as the ratio.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>STILL OPEN</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>What to confirm</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="52" customHeight="1">
-      <c r="A19" s="40" t="inlineStr">
+    <row r="20" ht="52" customHeight="1">
+      <c r="A20" s="40" t="inlineStr">
         <is>
           <t>REMIND JACOB — ComEd with Megan</t>
         </is>
       </c>
-      <c r="B19" s="40" t="inlineStr">
+      <c r="B20" s="40" t="inlineStr">
         <is>
           <t>ComEd is not on these cards. Monarch Adv Plus shows ACH: Jacob Coley $829.15 → Unit 2 ELECTRIC; Megan Gerrard $1,565.26 → Unit 1 ELECTRIC (yellow). User: must have been paid directly or with a check. Double-check with Megan: meters, whether Jake checking ACH is the full picture, and any extra check/direct payments.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="52" customHeight="1">
-      <c r="A20" s="17" t="inlineStr">
-        <is>
-          <t>Soldier Field East Parking $57</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>Coinbase 2025-11-01 same day as Field Museum. Not confirmed — HOLD.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="52" customHeight="1">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>Extra Space $360</t>
+          <t>Soldier Field East Parking $57</t>
         </is>
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>Prime 2025-12-10. Not part of the HD/Lowe’s/IKEA split — HOLD (storage vs moving vs personal).</t>
+          <t>Coinbase 2025-11-01 same day as Field Museum. Not confirmed — HOLD.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="52" customHeight="1">
       <c r="A22" s="17" t="inlineStr">
         <is>
-          <t>State Farm declarations / Sep–Dec</t>
+          <t>Extra Space $360</t>
         </is>
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>Home vs auto $ is a Feb-charge proxy ($157.53 home / $145.25 auto) until declarations pages. None on Prime Sep–Dec 2025 (524 sold 12/18 — those months may be another account). 2023–24 Excel booked all homeowners on U1; this packet 50/50’s the home share. No 2025 Travelers found on Prime/Sapphire/BoA/Monarch.</t>
+          <t>Prime 2025-12-10. Not part of the HD/Lowe’s/IKEA split — HOLD (storage vs moving vs personal).</t>
         </is>
       </c>
     </row>
     <row r="23" ht="52" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>Inventory object IDs</t>
+          <t>State Farm declarations / Sep–Dec</t>
         </is>
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>Frame Up $536.41 + LAMA $6,821.06 + Hindman $282.24 + $403.51 parked off Cost total until objects named (avoid Mercury double count).</t>
+          <t>Home vs auto $ is a Feb-charge proxy ($157.53 home / $145.25 auto) until declarations pages. None on Prime Sep–Dec 2025 (524 sold 12/18 — those months may be another account). 2023–24 Excel booked all homeowners on U1; this packet 50/50’s the home share. No 2025 Travelers found on Prime/Sapphire/BoA/Monarch.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="52" customHeight="1">
       <c r="A24" s="17" t="inlineStr">
         <is>
-          <t>827 Grove 1/3 hardware vs locked CapEx</t>
+          <t>Inventory object IDs</t>
         </is>
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>Grove share $604.12 is pre-close materials on the Grove tab. Do NOT fold into locked TY2025 CapEx $53,660 until CPA says so.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+          <t>Frame Up $536.41 + LAMA $6,821.06 + Hindman $282.24 + $403.51 parked off Cost total until objects named (avoid Mercury double count).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="52" customHeight="1">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>827 N Grove the house — HD 1/3 vs locked CapEx</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>HD/Lowe’s/IKEA 1/3 $604.12 is pre-close materials for 827 N Grove the house (Q5 split), not Grove Collaborative. Do NOT fold into locked TY2025 CapEx $53,660 until CPA says so.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Applied / split totals</t>
         </is>
       </c>
-      <c r="B26" s="18" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="19" t="inlineStr">
-        <is>
-          <t>EPGC Travel (Park Chicago $100 + Field Museum $53)</t>
-        </is>
-      </c>
-      <c r="B27" s="20" t="n">
-        <v>153</v>
-      </c>
+      <c r="B27" s="18" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="19" t="inlineStr">
         <is>
-          <t>March HD 100% 524 repairs</t>
+          <t>EPGC Travel (Park Chicago $100 + Field Museum $53)</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>1358.65</v>
+        <v>153</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="19" t="inlineStr">
         <is>
-          <t>Remaining HD/Lowe’s/IKEA (split pool)</t>
+          <t>March HD 100% 524 repairs</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
-        <v>1812.46</v>
+        <v>1358.65</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="19" t="inlineStr">
         <is>
-          <t>524 repairs from remaining 1/3 (then 50/50 U1/U2)</t>
+          <t>Remaining HD/Lowe’s/IKEA (split pool)</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
-        <v>604.1799999999999</v>
+        <v>1812.46</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="19" t="inlineStr">
         <is>
-          <t>Unit 2 EXTERIOR add (March 50% + remaining 524-share 50%)</t>
+          <t>524 repairs from remaining 1/3 (then 50/50 U1/U2)</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
-        <v>981.4400000000001</v>
+        <v>604.1799999999999</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="19" t="inlineStr">
         <is>
+          <t>Unit 2 EXTERIOR add (March 50% + remaining 524-share 50%)</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="n">
+        <v>981.4400000000001</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr">
+        <is>
           <t>Unit 1 EXTERIOR add (March 50% + remaining 524-share 50%)</t>
         </is>
       </c>
-      <c r="B32" s="20" t="n">
+      <c r="B33" s="20" t="n">
         <v>981.39</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="41" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="41" t="inlineStr">
         <is>
           <t>Personal 1/3 (excluded from P&amp;L)</t>
         </is>
       </c>
-      <c r="B33" s="42" t="n">
+      <c r="B34" s="42" t="n">
         <v>604.16</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="43" t="inlineStr">
-        <is>
-          <t>827 Grove 1/3 (not in locked $53,660)</t>
-        </is>
-      </c>
-      <c r="B34" s="44" t="n">
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>827 N Grove the house 1/3 HD/Lowe’s/IKEA (not Grove Collaborative; not locked $53,660)</t>
+        </is>
+      </c>
+      <c r="B35" s="20" t="n">
         <v>604.12</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="45" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>524 Unit 2 SUPPLIES (Grove Collaborative)</t>
+        </is>
+      </c>
+      <c r="B36" s="20" t="n">
+        <v>791.21</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="45" t="inlineStr">
         <is>
           <t>Unit 2 ELECTRIC ComEd Jacob (YELLOW — ask Megan)</t>
         </is>
       </c>
-      <c r="B35" s="46" t="n">
+      <c r="B37" s="46" t="n">
         <v>829.15</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="45" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="45" t="inlineStr">
         <is>
           <t>Unit 1 ELECTRIC ComEd Megan (YELLOW — ask Megan)</t>
         </is>
       </c>
-      <c r="B36" s="46" t="n">
+      <c r="B38" s="46" t="n">
         <v>1565.26</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>524 INSURANCE home share (Unit 2 50%, yellow proxy)</t>
         </is>
       </c>
-      <c r="B37" s="47" t="n">
+      <c r="B39" s="47" t="n">
         <v>552.76</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>524 INSURANCE home share (Unit 1 50%, yellow proxy)</t>
         </is>
       </c>
-      <c r="B38" s="47" t="n">
+      <c r="B40" s="47" t="n">
         <v>552.7</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="41" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="41" t="inlineStr">
         <is>
           <t>State Farm auto share (personal, excluded)</t>
         </is>
       </c>
-      <c r="B39" s="42" t="n">
+      <c r="B41" s="42" t="n">
         <v>1019.33</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="41" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="41" t="inlineStr">
         <is>
           <t>Geico auto credit (personal, excluded)</t>
         </is>
       </c>
-      <c r="B40" s="42" t="n">
+      <c r="B42" s="42" t="n">
         <v>-540.89</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="19" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="19" t="inlineStr">
         <is>
           <t>Inventory parked (Frame Up + LAMA + Hindman)</t>
         </is>
       </c>
-      <c r="B41" s="20" t="n">
+      <c r="B43" s="20" t="n">
         <v>8043.22</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Extra Space HOLD</t>
         </is>
       </c>
-      <c r="B42" s="47" t="n">
+      <c r="B44" s="47" t="n">
         <v>360</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>Soldier Field parking HOLD</t>
         </is>
       </c>
-      <c r="B43" s="47" t="n">
+      <c r="B45" s="47" t="n">
         <v>57</v>
       </c>
     </row>
@@ -8872,7 +8909,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="26" t="inlineStr">
         <is>
-          <t>March Home Depot 100% → 524 repairs, then 50/50 Unit 1 / Unit 2. Each remaining txn split 1/3 524 / 1/3 personal / 1/3 827 Grove; leftover pennies to 524 then personal. 524 third then 50/50 (extra penny to Unit 2). Not tax advice.</t>
+          <t>March Home Depot 100% → 524 repairs, then 50/50 Unit 1 / Unit 2. Each remaining txn split 1/3 524 / 1/3 personal / 1/3 827 N Grove the house (NOT Grove Collaborative); leftover pennies to 524 then personal. 524 third then 50/50 (extra penny to Unit 2). Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -9646,7 +9683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O40"/>
+  <dimension ref="B1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="2" max="2"/>
@@ -9889,7 +9926,6 @@
         <v/>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
@@ -10867,7 +10903,6 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
@@ -10927,24 +10962,13 @@
         <v/>
       </c>
     </row>
-    <row r="29"/>
-    <row r="30" ht="96" customHeight="1">
+    <row r="30" ht="108" customHeight="1">
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>CC answers 2026-09-18: Nicor small / Prime ATT / Grove / Schauer / yard CONFIRMED. March HD $1358.65 → 524 EXTERIOR REPAIRS 50/50 with Unit 1. Remaining Prime HD/Lowe’s/IKEA 1/3 524 (50/50), 1/3 personal, 1/3 Grove. ELECTRIC yellow — REMIND JACOB: double-check ComEd with Megan (checking ACH Jacob $829.15; any extra check?). Home Depot March read as 524 (not 534). Extra Space $360 HOLD. State Farm: bundled home+auto (was Travelers home / Geico auto). Only HOME share on this INSURANCE line (50/50 with Unit 1, yellow = Feb $157.53 home / $145.25 auto proxy). Auto share and Geico $540.89 credit EXCLUDED personal. No Sep–Dec on Prime. Not tax advice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
+          <t>CC answers 2026-09-18: Nicor small / Prime ATT / Grove Collaborative supplies / Schauer / yard CONFIRMED. March HD $1358.65 → 524 EXTERIOR REPAIRS 50/50 with Unit 1. Remaining Prime HD/Lowe’s/IKEA 1/3 524 (50/50), 1/3 personal, 1/3 827 N Grove the house (not Grove Collaborative). ELECTRIC yellow — REMIND JACOB: double-check ComEd with Megan (checking ACH Jacob $829.15; any extra check?). Home Depot March read as 524 (not 534). Extra Space $360 HOLD. State Farm: bundled home+auto (was Travelers home / Geico auto). Only HOME share on this INSURANCE line (50/50 with Unit 1, yellow = Feb $157.53 home / $145.25 auto proxy). Auto share and Geico $540.89 credit EXCLUDED personal. No Sep–Dec on Prime. Not tax advice.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10956,7 +10980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O40"/>
+  <dimension ref="B1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="2" max="2"/>
@@ -11199,7 +11223,6 @@
         <v/>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
@@ -12177,7 +12200,6 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
@@ -12237,7 +12259,6 @@
         <v/>
       </c>
     </row>
-    <row r="29"/>
     <row r="30" ht="96" customHeight="1">
       <c r="B30" s="23" t="inlineStr">
         <is>
@@ -12245,16 +12266,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Spell out Grove Collaborative on the SOURCE tab.
Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
+++ b/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
@@ -747,7 +747,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Q1–4 CONFIRMED. March HD → 524 repairs 50/50. Remaining HD/Lowe’s/IKEA 1/3 524 / 1/3 personal / 1/3 Grove. ComEd yellow — REMIND JACOB: double-check with Megan (checking ACH or extra check). Canva + Park Chicago + Field Museum $53 EPGC. Frame Up framing + LAMA/Hindman inventory. Soldier Field parking $57 and Extra Space $360 still HOLD. Not tax advice.</t>
+          <t>Q1–4 CONFIRMED. Grove Collaborative (not 827 N Grove) → 524 Unit 2 SUPPLIES $791.21. March HD → 524 repairs 50/50. Remaining HD/Lowe’s/IKEA 1/3 524 / 1/3 personal / 1/3 827 N Grove the house. ComEd yellow — REMIND JACOB: double-check with Megan (checking ACH or extra check). Canva + Park Chicago + Field Museum $53 EPGC. Frame Up framing + LAMA/Hindman inventory. Soldier Field parking $57 and Extra Space $360 still HOLD. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -3388,7 +3388,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -3498,7 +3497,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="51" t="inlineStr">
         <is>
@@ -3718,7 +3716,6 @@
         <v>604.12</v>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Apply checking-inflow answers: Ava rent, vacancy, Joan repair, GCM off Consultant.
Book 216 Oak Park cash $19,500 green (Ava co-tenant kept), vacant Oct + half Nov,
Joan Zelle $675 as December interior repair, and Freeman's Sale 6428 $11,000 on
Art Sales (check to Megan). Zero EPGC Consultant; GCM $21,500 stays personal 1099.
Bear Creek $38k is a parent gift to Jake. Half-Nov rent and 8507 wait on Megan.
Not tax advice.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
+++ b/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
@@ -29,7 +29,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CC_LEDGER'!$A$3:$H$104</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'INFLOW_LEDGER'!$A$4:$H$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'INFLOW_LEDGER'!$A$4:$H$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37,9 +37,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -160,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -233,6 +234,14 @@
     <xf numFmtId="165" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -598,7 +607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -807,9 +816,21 @@
           <t>Checking inflows 2026-09-18</t>
         </is>
       </c>
-      <c r="B22" s="23" t="inlineStr">
-        <is>
-          <t>JSC 9922 + joint 0203 full-year eStmts. GCM BOM $21500.00 → EPGC Consultant. Reimburse $5214.69 excluded. 216 Oak Park rent cash $19500.00 (Delach / Ava yellow / Joan yellow). Bear Creek $38000.00 + UTMA Thomas $10000.00 not income. Freeman’s CIBC $11,000 HOLD. Not tax advice.</t>
+      <c r="B22" s="56" t="inlineStr">
+        <is>
+          <t>JSC 9922 + joint 0203 full-year eStmts. GCM BOM $21500.00 → GCM tab + Income E7 only (NOT EPGC Consultant). Reimburse $5214.69 excluded (May 22 CONFIRMED). 216 Oak Park rent cash $19500.00 (Ava co-tenant CONFIRMED). Vacant Oct + half Nov. Joan repair $675 → INTERIOR Dec. Bear Creek $38000.00 gift to Jake from parents. UTMA Thomas $10000.00 not income. Freeman’s Sale 6428 $11,000 Art Sales (check to Megan). 8507 WAIT-MEGAN. Not tax advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>Checking answers 2026-09-18</t>
+        </is>
+      </c>
+      <c r="B23" s="56" t="inlineStr">
+        <is>
+          <t>Q1 Ava co-tenant keep. Q2 vacant Oct + half Nov. Q3 Joan half-Nov WAIT 8507; 12/1 Zelle OUT $675 repair. Q4 GCM off EPGC Consultant. Q5 May 22 reimbursement. Q6 Bear Creek $38k to Jake from parents. Q7 Freeman’s $11k art settlement to Megan. Q8 Megan sending 8507 statements.</t>
         </is>
       </c>
     </row>
@@ -920,40 +941,40 @@
           <t>STR / RENTAL INCOME</t>
         </is>
       </c>
-      <c r="C3" s="21" t="n">
+      <c r="C3" s="22" t="n">
         <v>1950</v>
       </c>
-      <c r="D3" s="21" t="n">
+      <c r="D3" s="22" t="n">
         <v>1950</v>
       </c>
-      <c r="E3" s="21" t="n">
+      <c r="E3" s="22" t="n">
         <v>1950</v>
       </c>
-      <c r="F3" s="21" t="n">
+      <c r="F3" s="22" t="n">
         <v>1950</v>
       </c>
-      <c r="G3" s="21" t="n">
+      <c r="G3" s="22" t="n">
         <v>1950</v>
       </c>
-      <c r="H3" s="21" t="n">
+      <c r="H3" s="22" t="n">
         <v>1950</v>
       </c>
-      <c r="I3" s="21" t="n">
+      <c r="I3" s="22" t="n">
         <v>1450</v>
       </c>
-      <c r="J3" s="21" t="n">
+      <c r="J3" s="22" t="n">
         <v>2450</v>
       </c>
-      <c r="K3" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="21" t="n">
+      <c r="K3" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="22" t="n">
         <v>3900</v>
       </c>
       <c r="O3">
@@ -1334,41 +1355,41 @@
           <t>INTERIOR MAINTENANCE</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="4" t="n">
-        <v>0</v>
+      <c r="C12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="22" t="n">
+        <v>675</v>
       </c>
       <c r="O12">
         <f>SUM(C12:N12)</f>
@@ -2106,10 +2127,10 @@
       </c>
     </row>
     <row r="29"/>
-    <row r="30" ht="90" customHeight="1">
+    <row r="30" ht="108" customHeight="1">
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>LTR rent 2026-09-18: joint 0203 Zelle — Delach $1,450 + Ava $500 (yellow, ASK roommate) Feb–Sep cash, then Joan $1,950 on 12/1 and 12/31 (yellow, ASK Dec vs Jan-2026 prepaid). TY2025 cash $19500.00. Oct–Nov no rent on 0203 (ASK vacancy). Jan 2025 occupancy was paid 12/31/2024 — not in this year. HOA + Rocket payment cash from Monarch (green). Deduct interest from Rocket 1098 only — not full P+I. Not tax advice.</t>
+          <t>LTR after answers 2026-09-18: Ava CONFIRMED Delach co-tenant — keep $500/mo. TY2025 cash $19500.00 (Delach $11,600 + Ava $4,000 + Joan $3,900). Occupancy vacant October and half of November (held for rent). Joan half-Nov $975 NOT booked — not on 0203, WAIT 8507. 12/1 $1,950 IN = December occupancy cash; 12/31 $1,950 = Jan 2026 prepaid cash in TY2025. 12/1 8507 Zelle OUT $675 to Joan → INTERIOR MAINTENANCE (repair). Jan 2025 occupancy was paid 12/31/2024 — not in this year. HOA + Rocket payment cash from Monarch (green). Deduct interest from Rocket 1098 only — not full P+I. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -2270,40 +2291,40 @@
           <t>Consultant</t>
         </is>
       </c>
-      <c r="B4" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" s="22" t="n">
-        <v>4100</v>
-      </c>
-      <c r="D4" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="22" t="n">
-        <v>9200</v>
-      </c>
-      <c r="F4" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="22" t="n">
-        <v>4100</v>
-      </c>
-      <c r="K4" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="22" t="n">
-        <v>4100</v>
-      </c>
-      <c r="M4" s="21" t="n">
+      <c r="B4" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="57" t="n">
         <v>0</v>
       </c>
       <c r="N4">
@@ -3388,9 +3409,9 @@
     </row>
     <row r="42"/>
     <row r="43">
-      <c r="A43" s="26" t="inlineStr">
-        <is>
-          <t>Checking inflows 2026-09-18: GCM BOM PAYMEN $21500.00 → Consultant (ties 1099-NEC). JAKE C / SEFOF reimbursements $5214.69 EXCLUDED. ASK: EPGC LLC vs personal 1099. Bear Creek / UTMA not on this tab. Not tax advice.</t>
+      <c r="A43" s="58" t="inlineStr">
+        <is>
+          <t>Checking answers 2026-09-18: GCM BOM PAYMEN $21,500 REMOVED from EPGC Consultant (personal 1099 / GCM tab + Income E7 only). Consultant row is $0. JAKE C / SEFOF reimbursements $5214.69 still EXCLUDED. Bear Creek / UTMA not on this tab. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -3410,7 +3431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4137,12 +4158,27 @@
       </c>
     </row>
     <row r="23">
-      <c r="C23" s="3">
-        <f>SUM(C51:C70)</f>
-        <v/>
-      </c>
-      <c r="F23" t="n">
-        <v>30000</v>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Sale 6428 Contract 303468 (object TBD)</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Cost TBD</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n"/>
+      <c r="E23" s="19" t="inlineStr">
+        <is>
+          <t>Freeman's LLC — check to Megan (joint 0203)</t>
+        </is>
+      </c>
+      <c r="F23" s="22" t="n">
+        <v>11000</v>
+      </c>
+      <c r="G23" s="59" t="n">
+        <v>46015</v>
       </c>
       <c r="H23">
         <f>IF(OR(F23="",C23=""),"",F23-C23)</f>
@@ -4175,7 +4211,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Yellow Sale Price = still need buyer invoices. Green Cost = COGS already entered.</t>
+          <t>Yellow Sale Price = still need Berk buyer invoices. Row 23 Freeman’s Sale 6428 $11,000 CONFIRMED (check to Megan 12/24); Cost / object yellow. Green Cost = COGS already entered. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -4273,8 +4309,17 @@
         </is>
       </c>
     </row>
+    <row r="35" ht="36" customHeight="1">
+      <c r="A35" s="23" t="inlineStr">
+        <is>
+          <t>User 2026-09-18: Freeman’s / CIBC $11,000 on joint 0203 is an art-sale settlement; the check went to Megan. Do not add Cost into the total until the object is named. 2026-01-08 Hindman Sale 6428 $937.83 is 2026.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
+    <mergeCell ref="A35:I35"/>
+    <mergeCell ref="A26:I26"/>
     <mergeCell ref="A33:I33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4293,7 +4338,7 @@
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="80" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -4309,14 +4354,14 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>GCM / Gates Capital 2025 — board fees vs reimbursements (not tax advice)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="36" customHeight="1">
+          <t>GCM / Gates Capital 2025 — personal 1099 (NOT EPGC Consultant) — not tax advice</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="26" t="inlineStr">
         <is>
-          <t>BOM PAYMEN $21500.00 = Form 1099-NEC $21,500 → EPGC Consultant + this tab. JAKE C / SEFOF reimbursements $5214.69 EXCLUDED. CPA: confirm EPGC LLC vs personal 1099/Sch C.</t>
+          <t>BOM PAYMEN $21500.00 = Form 1099-NEC $21,500 → this tab + Income E7 only. User 2026-09-18: remove GCM from the EPGC Consultant line (1099 is in Jacob’s name). JAKE C / SEFOF reimbursements $5214.69 EXCLUDED (May 22 $609.02 CONFIRMED reimbursement).</t>
         </is>
       </c>
     </row>
@@ -4395,7 +4440,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Board fee (BOM PAYMEN → Consultant)</t>
+          <t>Board fee (BOM PAYMEN → personal 1099 / GCM tab)</t>
         </is>
       </c>
       <c r="B5" s="49" t="n">
@@ -4541,7 +4586,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Consultant / 1099</t>
+          <t>Personal 1099 / GCM tab</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -4551,7 +4596,7 @@
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>BOM PAYMEN</t>
+          <t>BOM PAYMEN — not EPGC Consultant</t>
         </is>
       </c>
     </row>
@@ -4571,7 +4616,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Consultant / 1099</t>
+          <t>Personal 1099 / GCM tab</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
@@ -4581,7 +4626,7 @@
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>BOM PAYMEN</t>
+          <t>BOM PAYMEN — not EPGC Consultant</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4646,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Consultant / 1099</t>
+          <t>Personal 1099 / GCM tab</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -4611,7 +4656,7 @@
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>BOM PAYMEN</t>
+          <t>BOM PAYMEN — not EPGC Consultant</t>
         </is>
       </c>
     </row>
@@ -4631,7 +4676,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Consultant / 1099</t>
+          <t>Personal 1099 / GCM tab</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
@@ -4641,7 +4686,7 @@
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>BOM PAYMEN</t>
+          <t>BOM PAYMEN — not EPGC Consultant</t>
         </is>
       </c>
     </row>
@@ -4701,7 +4746,7 @@
       </c>
       <c r="F15" s="13" t="inlineStr">
         <is>
-          <t>JAKE C — no PMT INFO on statement; odd cents, not BOM — treated as reimburse</t>
+          <t>CONFIRMED reimbursement (JAKE C, not BOM)</t>
         </is>
       </c>
     </row>
@@ -4761,7 +4806,7 @@
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>SEFOF WHARTON EXPENSES — not on the two BoA folders</t>
+          <t>SEFOF WHARTON EXPENSES — WAIT 8507 statements</t>
         </is>
       </c>
     </row>
@@ -4791,7 +4836,7 @@
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>SEFOF ANNUAL CONFERENCE EXPENSES</t>
+          <t>SEFOF ANNUAL CONFERENCE EXPENSES — WAIT 8507 statements</t>
         </is>
       </c>
     </row>
@@ -4821,14 +4866,14 @@
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>SEFOF REIMBURSE EXPENSES FOR EDUCATION COMMITTEE</t>
+          <t>SEFOF EDUCATION COMMITTEE — WAIT 8507 statements</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="43" t="inlineStr">
         <is>
-          <t>1099-NEC Gates Capital Management LLC TIN 84-1331261 box 1 = $21,500. BOM sum ties. Reimbursements are not on the 1099.</t>
+          <t>1099-NEC Gates Capital Management LLC TIN 84-1331261 box 1 = $21,500. BOM sum ties. Reimbursements are not on the 1099. EPGC Consultant is $0.</t>
         </is>
       </c>
     </row>
@@ -10077,495 +10122,489 @@
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="39" t="inlineStr">
         <is>
-          <t>BoA checking folders = 9922 + 0203</t>
+          <t>Ava L Hernandez $500/mo rent</t>
         </is>
       </c>
       <c r="B18" s="39" t="inlineStr">
         <is>
-          <t>JSC Adv Plus 4830 6191 9922 (Jake) and joint Adv Plus 4830 7359 0203 (Megan+Jacob). 12 statements each for 2025. Monarch credits on those two accounts match the statement deposit sections sampled.</t>
+          <t>CONFIRMED Delach co-tenant. Keep eight $500 Zelle credits on 216 Oak Park STR / RENTAL INCOME. Delach $1,450 + Ava $500 = $1,950 unit rent (same as Joan later).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="36" customHeight="1">
       <c r="A19" s="39" t="inlineStr">
         <is>
-          <t>GCM board fee → Consultant</t>
+          <t>Oak Park vacant Oct + half Nov</t>
         </is>
       </c>
       <c r="B19" s="39" t="inlineStr">
         <is>
-          <t>Gates Capital BOM PAYMEN $21500.00: 2/12 $4,100 + 4/18 $9,200 + 9/13 $4,100 + 11/13 $4,100. Equals Form 1099-NEC $21,500. Booked EPGC Consultant (cash-basis month) and GCM tab. Income tab GCM actual was already $21,500.</t>
+          <t>CONFIRMED vacant October and the first half of November (held for rent). Occupancy: Delach/Ava through September; Joan from mid-November. Cash-basis months stay as deposited (Sep cash is $0 because September rent hit 8/29). Jan 2025 occupancy cash hit 12/31/2024 — still out of TY2025.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="39" t="inlineStr">
         <is>
-          <t>GCM reimbursements EXCLUDED</t>
+          <t>Joan 12/1 Zelle OUT $675 = repair</t>
         </is>
       </c>
       <c r="B20" s="39" t="inlineStr">
         <is>
-          <t>JAKE C / SEFOF on 9922 $3033.83 (board meeting $1,150.99; 5/22 $609.02 unlabeled; 11/05 $1,273.82). Plus Checking 8507 SEFOF $2180.86 (Wharton / annual conference / education committee) — that account is not in the two folders. Total reimbursement $5214.69 kept off Consultant.</t>
+          <t>CONFIRMED. Checking 8507 Zelle to Joan 12/1 $675 → 216 INTERIOR MAINTENANCE (December). CPA may reclass interior vs exterior. 12/1 $1,950 IN on joint 0203 stays December occupancy cash; 12/31 $1,950 “January rent” stays Jan 2026 prepaid cash in TY2025.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="36" customHeight="1">
       <c r="A21" s="39" t="inlineStr">
         <is>
-          <t>LTR rent → 216 Oak Park STR / RENTAL INCOME</t>
+          <t>GCM off EPGC Consultant</t>
         </is>
       </c>
       <c r="B21" s="39" t="inlineStr">
         <is>
-          <t>JOHN T DELACH 8×$1,450 ($11600.00) + Joan Friedberger 2×$1,950 ($3900.00) on joint 0203. Ava L Hernandez 8×$500 ($4000.00) same rent memo / $1,950 combined — included yellow (ASK). TY2025 cash total $19500.00. Oct–Nov 2025: no rent on 0203.</t>
+          <t>CONFIRMED. BOM PAYMEN $21,500 stays on the GCM tab + Income E7 (personal 1099-NEC, Jacob’s name). EPGC Consultant zeroed. JAKE C / SEFOF reimbursements $5,214.69 still excluded.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="39" t="inlineStr">
         <is>
-          <t>Bear Creek not income</t>
+          <t>May 22 Gates $609.02</t>
         </is>
       </c>
       <c r="B22" s="39" t="inlineStr">
         <is>
-          <t>Four wires $9,500 on Jake 9922 (1/9, 4/10, 7/10, 10/9) = $38000.00. Annual gift — excluded from Consultant / rental / Income tab.</t>
+          <t>CONFIRMED reimbursement (JAKE C, not BOM PAYMEN). Excluded from income.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="39" t="inlineStr">
         <is>
-          <t>UTMA not income</t>
+          <t>Bear Creek $38,000 to Jake from parents</t>
         </is>
       </c>
       <c r="B23" s="39" t="inlineStr">
         <is>
-          <t>Emma CMA 2T48 + sibling CMA 4729: Thomas wires $5,000 each Nov/Dec = $10000.00 (not ~$10k each). Treasury-note maturities $10,000 each 12/31 are principal, not gifts. Excluded from income.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+          <t>CONFIRMED annual gift to Jacob from parents — not income. User: UTMA was not ~$10k each; Thomas wires $5,000 each (Emma CMA 2T48 + Phoebe CMA 4729) = $10,000 excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="39" t="inlineStr">
+        <is>
+          <t>Freeman’s / CIBC $11,000 art-sale settlement</t>
+        </is>
+      </c>
+      <c r="B24" s="39" t="inlineStr">
+        <is>
+          <t>CONFIRMED Sale 6428 Contract 303468. Check went to Megan (joint 0203 2025-12-24). Booked Art Sales Sale Price $11,000; Cost and object name yellow TBD. Not Mercury, not W-2 payroll.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="39" t="inlineStr">
+        <is>
+          <t>Checking 8507 statements</t>
+        </is>
+      </c>
+      <c r="B25" s="39" t="inlineStr">
+        <is>
+          <t>WAIT-MEGAN. Jacob asked Megan to send 2025 NOW 8507 statements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>STILL OPEN</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>What to confirm</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="52" customHeight="1">
-      <c r="A26" s="40" t="inlineStr">
+    <row r="28" ht="52" customHeight="1">
+      <c r="A28" s="40" t="inlineStr">
         <is>
           <t>REMIND JACOB — ComEd with Megan</t>
         </is>
       </c>
-      <c r="B26" s="40" t="inlineStr">
+      <c r="B28" s="40" t="inlineStr">
         <is>
           <t>Joint 0203 statements show ComEd ACH (e.g. 1/21 Jacob $59.04 + Megan $132.94). ComEd is not on these cards. Monarch Adv Plus shows ACH: Jacob Coley $829.15 → Unit 2 ELECTRIC; Megan Gerrard $1,565.26 → Unit 1 ELECTRIC (yellow). User: must have been paid directly or with a check. Double-check with Megan: meters, whether Jake checking ACH is the full picture, and any extra check/direct payments.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="52" customHeight="1">
-      <c r="A27" s="17" t="inlineStr">
-        <is>
-          <t>Soldier Field East Parking $57</t>
-        </is>
-      </c>
-      <c r="B27" s="17" t="inlineStr">
-        <is>
-          <t>Coinbase 2025-11-01 same day as Field Museum. Not confirmed — HOLD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="52" customHeight="1">
-      <c r="A28" s="17" t="inlineStr">
-        <is>
-          <t>Extra Space $360</t>
-        </is>
-      </c>
-      <c r="B28" s="17" t="inlineStr">
-        <is>
-          <t>Prime 2025-12-10. Not part of the HD/Lowe’s/IKEA split — HOLD (storage vs moving vs personal).</t>
         </is>
       </c>
     </row>
     <row r="29" ht="52" customHeight="1">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>State Farm declarations / Sep–Dec</t>
+          <t>Soldier Field East Parking $57</t>
         </is>
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>Home vs auto $ is a Feb-charge proxy ($157.53 home / $145.25 auto) until declarations pages. None on Prime Sep–Dec 2025 (524 sold 12/18 — those months may be another account). 2023–24 Excel booked all homeowners on U1; this packet 50/50’s the home share. No 2025 Travelers found on Prime/Sapphire/BoA/Monarch.</t>
+          <t>Coinbase 2025-11-01 same day as Field Museum. Not confirmed — HOLD.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="52" customHeight="1">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>Inventory object IDs</t>
+          <t>Extra Space $360</t>
         </is>
       </c>
       <c r="B30" s="17" t="inlineStr">
         <is>
-          <t>Frame Up $536.41 + LAMA $6,821.06 + Hindman $282.24 + $403.51 parked off Cost total until objects named (avoid Mercury double count).</t>
+          <t>Prime 2025-12-10. Not part of the HD/Lowe’s/IKEA split — HOLD (storage vs moving vs personal).</t>
         </is>
       </c>
     </row>
     <row r="31" ht="52" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>827 N Grove the house — HD 1/3 vs locked CapEx</t>
+          <t>State Farm declarations / Sep–Dec</t>
         </is>
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>HD/Lowe’s/IKEA 1/3 $604.12 is pre-close materials for 827 N Grove the house (Q5 split), not Grove Collaborative. Do NOT fold into locked TY2025 CapEx $53,660 until CPA says so.</t>
+          <t>Home vs auto $ is a Feb-charge proxy ($157.53 home / $145.25 auto) until declarations pages. None on Prime Sep–Dec 2025 (524 sold 12/18 — those months may be another account). 2023–24 Excel booked all homeowners on U1; this packet 50/50’s the home share. No 2025 Travelers found on Prime/Sapphire/BoA/Monarch.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="52" customHeight="1">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>Ava L Hernandez $500/mo rent</t>
+          <t>Inventory object IDs</t>
         </is>
       </c>
       <c r="B32" s="17" t="inlineStr">
         <is>
-          <t>Eight Zelle credits on joint 0203, same days as Delach, memo “rent”. Delach $1,450 + Ava $500 = $1,950, which is Joan’s later rent. Is Ava Delach’s roommate/co-tenant at 216 Oak Park? I booked her on STR / RENTAL INCOME (yellow) so the $1,950 unit rent is complete. Say if she should be excluded.</t>
+          <t>Frame Up $536.41 + LAMA $6,821.06 + Hindman $282.24 + $403.51 parked off Cost total until objects named (avoid Mercury double count).</t>
         </is>
       </c>
     </row>
     <row r="33" ht="52" customHeight="1">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>Oak Park vacant Oct–Nov 2025?</t>
+          <t>827 N Grove the house — HD 1/3 vs locked CapEx</t>
         </is>
       </c>
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>No Delach / Ava / Joan rent on 0203 in October or November. Last Delach/Ava is 8/29 “September Rent”. Joan starts 12/1. Confirm those two months were vacant (and held for rent) for Sch E. Jan 2025 occupancy cash hit 12/31/2024 ($1,450+$500) — left out of TY2025 cash. Correct?</t>
+          <t>HD/Lowe’s/IKEA 1/3 $604.12 is pre-close materials for 827 N Grove the house (Q5 split), not Grove Collaborative. Do NOT fold into locked TY2025 CapEx $53,660 until CPA says so.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="52" customHeight="1">
       <c r="A34" s="17" t="inlineStr">
         <is>
-          <t>Joan Friedberger Dec cash</t>
+          <t>WAIT MEGAN — Checking 8507 (NOW) 2025 statements</t>
         </is>
       </c>
       <c r="B34" s="17" t="inlineStr">
         <is>
-          <t>12/1 $1,950 memo “rent” and 12/31 $1,950 memo “January rent” both in TY2025 cash. Is 12/1 December occupancy and 12/31 January 2026 prepaid? Also: Checking 8507 Zelle OUT $675 to Joan on 12/1 — deposit return / repair? Not on these two BoA folders.</t>
+          <t>Jacob asked Megan to send them. Needed to (a) book Joan’s half-November rent if the deposit is there, (b) keep reconciling Airbnb/VRBO vs platform, (c) keep the three SEFOF reimbursements tied. 11/30 Zelle FROM MEGAN $1,950 on 8507 is a Megan transfer, not Joan rent.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="52" customHeight="1">
       <c r="A35" s="17" t="inlineStr">
         <is>
-          <t>GCM on EPGC Consultant vs personal 1099</t>
+          <t>Joan half-November rent $975</t>
         </is>
       </c>
       <c r="B35" s="17" t="inlineStr">
         <is>
-          <t>You said board fee → consultant line, so I put BOM $21,500 on EPGC LLC Consultant. Historically GCM lived on its own tab + Income “GCM Boards”, and EPGC Consultant was empty. 1099-NEC is in Jacob’s name from Gates Capital. Confirm: EPGC LLC (this booking) vs personal Sch C / GCM tab only (then I will zero EPGC Consultant so LLC P&amp;L is not mixed).</t>
+          <t>User: Joan paid half of November. Not on joint 0203. Nov cash on 216 Oak Park stays $0 until 8507 (or another account) shows the deposit. Do not invent $975.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="52" customHeight="1">
       <c r="A36" s="17" t="inlineStr">
         <is>
-          <t>May 22 Gates $609.02</t>
+          <t>Sale 6428 object / Cost</t>
         </is>
       </c>
       <c r="B36" s="17" t="inlineStr">
         <is>
-          <t>Statement says GATES CAPITAL MA DES:JAKE C $609.02 — no PMT INFO. Same DES as reimbursements, not BOM PAYMEN. I excluded it from Consultant. Confirm it is reimbursement (or board fee if you say so).</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="52" customHeight="1">
-      <c r="A37" s="17" t="inlineStr">
-        <is>
-          <t>Bear Creek $38,000 vs kids’ UTMA ~$10k each</t>
-        </is>
-      </c>
-      <c r="B37" s="17" t="inlineStr">
-        <is>
-          <t>Bear Creek to Jake 9922 is $9,500×4 = $38,000 (not ~$10k). Thomas wires into the two CMA-Edge UTMAs are $5,000 each in late Nov. Are Bear Creek gifts to you (parents), and Thomas the kids’ UTMA? Is more UTMA cash coming that never hit these checkings (e.g. directly at Merrill)? 2/25 $36,000 9922→National Financial was reversed 2/27.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="52" customHeight="1">
-      <c r="A38" s="17" t="inlineStr">
-        <is>
-          <t>Freeman’s / CIBC $11,000 wire 12/24 on joint 0203</t>
-        </is>
-      </c>
-      <c r="B38" s="17" t="inlineStr">
-        <is>
-          <t>ORIG:FREEMAN'S LLC via CIBC Bank USA; PMT DET Sale 6428 Contract 303468. Not W-2 payroll (those are DIR DEP on 9922). Art sale? Consignment? Other? HOLD off income until you say.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="52" customHeight="1">
-      <c r="A39" s="17" t="inlineStr">
-        <is>
-          <t>Checking 8507 (NOW) 2025 statements?</t>
-        </is>
-      </c>
-      <c r="B39" s="17" t="inlineStr">
-        <is>
-          <t>Third checking in Monarch — Airbnb/VRBO STR, Megan Zelle, and the three GCM SEFOF reimbursements. Not in the two folders you just added. Upload 2025 statements if you want that account reconciled the same way.</t>
-        </is>
+          <t>Freeman’s $11,000 is Art Sales Sale Price (check to Megan 12/24). Cost and object blank yellow — Income E8 net stays $0 until Cost is filled. 2026-01-08 Hindman SETTLEMENT SALE 6428 $937.83 is 2026, not TY2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Applied / split totals</t>
+        </is>
+      </c>
+      <c r="B38" s="18" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
+          <t>EPGC Travel (Park Chicago $100 + Field Museum $53)</t>
+        </is>
+      </c>
+      <c r="B39" s="20" t="n">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="19" t="inlineStr">
+        <is>
+          <t>March HD 100% 524 repairs</t>
+        </is>
+      </c>
+      <c r="B40" s="20" t="n">
+        <v>1358.65</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>Applied / split totals</t>
-        </is>
-      </c>
-      <c r="B41" s="18" t="n"/>
+      <c r="A41" s="19" t="inlineStr">
+        <is>
+          <t>Remaining HD/Lowe’s/IKEA (split pool)</t>
+        </is>
+      </c>
+      <c r="B41" s="20" t="n">
+        <v>1812.46</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="19" t="inlineStr">
         <is>
-          <t>EPGC Travel (Park Chicago $100 + Field Museum $53)</t>
+          <t>524 repairs from remaining 1/3 (then 50/50 U1/U2)</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
-        <v>153</v>
+        <v>604.1799999999999</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="19" t="inlineStr">
         <is>
-          <t>March HD 100% 524 repairs</t>
+          <t>Unit 2 EXTERIOR add (March 50% + remaining 524-share 50%)</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
-        <v>1358.65</v>
+        <v>981.4400000000001</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="19" t="inlineStr">
         <is>
-          <t>Remaining HD/Lowe’s/IKEA (split pool)</t>
+          <t>Unit 1 EXTERIOR add (March 50% + remaining 524-share 50%)</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
-        <v>1812.46</v>
+        <v>981.39</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="19" t="inlineStr">
-        <is>
-          <t>524 repairs from remaining 1/3 (then 50/50 U1/U2)</t>
-        </is>
-      </c>
-      <c r="B45" s="20" t="n">
-        <v>604.1799999999999</v>
+      <c r="A45" s="41" t="inlineStr">
+        <is>
+          <t>Personal 1/3 (excluded from P&amp;L)</t>
+        </is>
+      </c>
+      <c r="B45" s="42" t="n">
+        <v>604.16</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="19" t="inlineStr">
         <is>
-          <t>Unit 2 EXTERIOR add (March 50% + remaining 524-share 50%)</t>
+          <t>827 N Grove the house 1/3 HD/Lowe’s/IKEA (not Grove Collaborative; not locked $53,660)</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
-        <v>981.4400000000001</v>
+        <v>604.12</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="19" t="inlineStr">
         <is>
-          <t>Unit 1 EXTERIOR add (March 50% + remaining 524-share 50%)</t>
+          <t>524 Unit 2 SUPPLIES (Grove Collaborative)</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
-        <v>981.39</v>
+        <v>791.21</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="41" t="inlineStr">
-        <is>
-          <t>Personal 1/3 (excluded from P&amp;L)</t>
-        </is>
-      </c>
-      <c r="B48" s="42" t="n">
-        <v>604.16</v>
+      <c r="A48" s="45" t="inlineStr">
+        <is>
+          <t>Unit 2 ELECTRIC ComEd Jacob (YELLOW — ask Megan)</t>
+        </is>
+      </c>
+      <c r="B48" s="46" t="n">
+        <v>829.15</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="19" t="inlineStr">
-        <is>
-          <t>827 N Grove the house 1/3 HD/Lowe’s/IKEA (not Grove Collaborative; not locked $53,660)</t>
-        </is>
-      </c>
-      <c r="B49" s="20" t="n">
-        <v>604.12</v>
+      <c r="A49" s="45" t="inlineStr">
+        <is>
+          <t>Unit 1 ELECTRIC ComEd Megan (YELLOW — ask Megan)</t>
+        </is>
+      </c>
+      <c r="B49" s="46" t="n">
+        <v>1565.26</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="19" t="inlineStr">
-        <is>
-          <t>524 Unit 2 SUPPLIES (Grove Collaborative)</t>
-        </is>
-      </c>
-      <c r="B50" s="20" t="n">
-        <v>791.21</v>
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>524 INSURANCE home share (Unit 2 50%, yellow proxy)</t>
+        </is>
+      </c>
+      <c r="B50" s="47" t="n">
+        <v>552.76</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="45" t="inlineStr">
-        <is>
-          <t>Unit 2 ELECTRIC ComEd Jacob (YELLOW — ask Megan)</t>
-        </is>
-      </c>
-      <c r="B51" s="46" t="n">
-        <v>829.15</v>
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>524 INSURANCE home share (Unit 1 50%, yellow proxy)</t>
+        </is>
+      </c>
+      <c r="B51" s="47" t="n">
+        <v>552.7</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="45" t="inlineStr">
-        <is>
-          <t>Unit 1 ELECTRIC ComEd Megan (YELLOW — ask Megan)</t>
-        </is>
-      </c>
-      <c r="B52" s="46" t="n">
-        <v>1565.26</v>
+      <c r="A52" s="41" t="inlineStr">
+        <is>
+          <t>State Farm auto share (personal, excluded)</t>
+        </is>
+      </c>
+      <c r="B52" s="42" t="n">
+        <v>1019.33</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>524 INSURANCE home share (Unit 2 50%, yellow proxy)</t>
-        </is>
-      </c>
-      <c r="B53" s="47" t="n">
-        <v>552.76</v>
+      <c r="A53" s="41" t="inlineStr">
+        <is>
+          <t>Geico auto credit (personal, excluded)</t>
+        </is>
+      </c>
+      <c r="B53" s="42" t="n">
+        <v>-540.89</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>524 INSURANCE home share (Unit 1 50%, yellow proxy)</t>
-        </is>
-      </c>
-      <c r="B54" s="47" t="n">
-        <v>552.7</v>
+      <c r="A54" s="19" t="inlineStr">
+        <is>
+          <t>Inventory parked (Frame Up + LAMA + Hindman)</t>
+        </is>
+      </c>
+      <c r="B54" s="20" t="n">
+        <v>8043.22</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="41" t="inlineStr">
-        <is>
-          <t>State Farm auto share (personal, excluded)</t>
-        </is>
-      </c>
-      <c r="B55" s="42" t="n">
-        <v>1019.33</v>
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Extra Space HOLD</t>
+        </is>
+      </c>
+      <c r="B55" s="47" t="n">
+        <v>360</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="41" t="inlineStr">
-        <is>
-          <t>Geico auto credit (personal, excluded)</t>
-        </is>
-      </c>
-      <c r="B56" s="42" t="n">
-        <v>-540.89</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="19" t="inlineStr">
-        <is>
-          <t>Inventory parked (Frame Up + LAMA + Hindman)</t>
-        </is>
-      </c>
-      <c r="B57" s="20" t="n">
-        <v>8043.22</v>
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Soldier Field parking HOLD</t>
+        </is>
+      </c>
+      <c r="B56" s="47" t="n">
+        <v>57</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>Extra Space HOLD</t>
-        </is>
-      </c>
-      <c r="B58" s="47" t="n">
-        <v>360</v>
-      </c>
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Checking inflows after answers 2026-09-18</t>
+        </is>
+      </c>
+      <c r="B58" s="18" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>Soldier Field parking HOLD</t>
-        </is>
-      </c>
-      <c r="B59" s="47" t="n">
-        <v>57</v>
+      <c r="A59" s="19" t="inlineStr">
+        <is>
+          <t>216 Oak Park STR / RENTAL INCOME (cash, Ava CONFIRMED co-tenant)</t>
+        </is>
+      </c>
+      <c r="B59" s="20" t="n">
+        <v>19500</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Delach 8 × $1,450</t>
+        </is>
+      </c>
+      <c r="B60" s="20" t="n">
+        <v>11600</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="5" t="inlineStr">
-        <is>
-          <t>Checking inflows 2026-09-18</t>
-        </is>
-      </c>
-      <c r="B61" s="18" t="n"/>
+      <c r="A61" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ava Hernandez 8 × $500 (co-tenant CONFIRMED)</t>
+        </is>
+      </c>
+      <c r="B61" s="20" t="n">
+        <v>4000</v>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="4" t="inlineStr">
-        <is>
-          <t>216 Oak Park STR / RENTAL INCOME (cash, incl. Ava yellow)</t>
-        </is>
-      </c>
-      <c r="B62" s="47" t="n">
-        <v>19500</v>
+      <c r="A62" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Joan Friedberger 2 × $1,950 (Dec cash + Jan 2026 prepaid)</t>
+        </is>
+      </c>
+      <c r="B62" s="20" t="n">
+        <v>3900</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Delach 8 × $1,450</t>
-        </is>
-      </c>
-      <c r="B63" s="20" t="n">
-        <v>11600</v>
+      <c r="A63" s="45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Joan half-Nov $975 NOT booked (WAIT 8507)</t>
+        </is>
+      </c>
+      <c r="B63" s="46" t="n">
+        <v>975</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Ava Hernandez 8 × $500 (ASK roommate)</t>
-        </is>
-      </c>
-      <c r="B64" s="47" t="n">
-        <v>4000</v>
+      <c r="A64" s="19" t="inlineStr">
+        <is>
+          <t>216 INTERIOR MAINTENANCE Dec (Joan Zelle OUT repair)</t>
+        </is>
+      </c>
+      <c r="B64" s="20" t="n">
+        <v>675</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Joan Friedberger 2 × $1,950 (ASK Dec vs Jan prepaid)</t>
-        </is>
-      </c>
-      <c r="B65" s="47" t="n">
-        <v>3900</v>
+      <c r="A65" s="41" t="inlineStr">
+        <is>
+          <t>EPGC Consultant (GCM removed)</t>
+        </is>
+      </c>
+      <c r="B65" s="42" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="19" t="inlineStr">
         <is>
-          <t>EPGC Consultant = GCM BOM = 1099-NEC</t>
+          <t>GCM personal 1099-NEC (tab + Income E7)</t>
         </is>
       </c>
       <c r="B66" s="20" t="n">
@@ -10575,7 +10614,7 @@
     <row r="67">
       <c r="A67" s="41" t="inlineStr">
         <is>
-          <t>GCM reimbursements EXCLUDED (9922 + 8507)</t>
+          <t>GCM reimbursements EXCLUDED (9922 + 8507; May 22 CONFIRMED)</t>
         </is>
       </c>
       <c r="B67" s="42" t="n">
@@ -10585,7 +10624,7 @@
     <row r="68">
       <c r="A68" s="41" t="inlineStr">
         <is>
-          <t>Bear Creek gift EXCLUDED (4 × $9,500)</t>
+          <t>Bear Creek gift to Jake from parents EXCLUDED</t>
         </is>
       </c>
       <c r="B68" s="42" t="n">
@@ -10595,7 +10634,7 @@
     <row r="69">
       <c r="A69" s="41" t="inlineStr">
         <is>
-          <t>UTMA Thomas wires EXCLUDED (2 × $5,000)</t>
+          <t>UTMA Thomas wires EXCLUDED (2 × $5,000, not ~$10k each)</t>
         </is>
       </c>
       <c r="B69" s="42" t="n">
@@ -10605,7 +10644,7 @@
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>Freeman’s CIBC $11,000 12/24 HOLD</t>
+          <t>Art Sales Sale 6428 Sale Price (Cost TBD)</t>
         </is>
       </c>
       <c r="B70" s="47" t="n">
@@ -10627,30 +10666,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="78" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>2025 checking inflows — JSC 9922 + joint 0203 (folder 07) — not tax advice</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="40" customHeight="1">
+          <t>2025 checking inflows after 2026-09-18 answers — JSC 9922 + joint 0203 — not tax advice</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="52" customHeight="1">
       <c r="A2" s="26" t="inlineStr">
         <is>
-          <t>Cash-basis by deposit date. BOM → Consultant. JAKE C / SEFOF → reimbursement EXCLUDED. Delach / Ava / Joan → 216 Oak Park STR / RENTAL INCOME. Bear Creek + UTMA Thomas wires → not income. Hindman/Freeman payroll stays on the W-2 tab. EPGC Mercury ACH into 9922 is a transfer, not income.</t>
+          <t>Cash-basis by deposit date. GCM BOM → personal 1099 / GCM tab (NOT EPGC Consultant). JAKE C / SEFOF → reimbursement EXCLUDED (May 22 CONFIRMED). Delach + Ava (co-tenant CONFIRMED) + Joan → 216 Oak Park STR / RENTAL INCOME. Bear Creek = gift to Jake from parents. UTMA Thomas $5k each excluded. Freeman’s Sale 6428 $11,000 → Art Sales (check to Megan). 8507 Zelle OUT Joan $675 → 216 INTERIOR MAINTENANCE.</t>
         </is>
       </c>
     </row>
@@ -10737,42 +10776,42 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>0203 joint</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>2025-01-31</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>AVA L HERNANDEZ</t>
         </is>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="12" t="n">
         <v>500</v>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>STR / RENTAL INCOME</t>
         </is>
       </c>
-      <c r="F6" s="14" t="inlineStr">
+      <c r="F6" s="11" t="inlineStr">
         <is>
           <t>216 N. Oak Park Ave</t>
         </is>
       </c>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>APPLIED-YELLOW</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>Rent (same day as Delach). Roommate/co-tenant? ASK</t>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>Rent (same day as Delach). Delach co-tenant CONFIRMED.</t>
         </is>
       </c>
     </row>
@@ -10817,42 +10856,42 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>0203 joint</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>2025-02-28</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>AVA L HERNANDEZ</t>
         </is>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="12" t="n">
         <v>500</v>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>STR / RENTAL INCOME</t>
         </is>
       </c>
-      <c r="F8" s="14" t="inlineStr">
+      <c r="F8" s="11" t="inlineStr">
         <is>
           <t>216 N. Oak Park Ave</t>
         </is>
       </c>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>APPLIED-YELLOW</t>
-        </is>
-      </c>
-      <c r="H8" s="14" t="inlineStr">
-        <is>
-          <t>Rent. Roommate/co-tenant? ASK</t>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>Rent. Delach co-tenant CONFIRMED.</t>
         </is>
       </c>
     </row>
@@ -10897,82 +10936,82 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>0203 joint</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>2025-03-31</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>AVA L HERNANDEZ</t>
         </is>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="12" t="n">
         <v>500</v>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>STR / RENTAL INCOME</t>
         </is>
       </c>
-      <c r="F10" s="14" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>216 N. Oak Park Ave</t>
         </is>
       </c>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>APPLIED-YELLOW</t>
-        </is>
-      </c>
-      <c r="H10" s="14" t="inlineStr">
-        <is>
-          <t>April Rent. Roommate/co-tenant? ASK</t>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>April Rent. Delach co-tenant CONFIRMED.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>0203 joint</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>2025-04-28</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>AVA L HERNANDEZ</t>
         </is>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="12" t="n">
         <v>500</v>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>STR / RENTAL INCOME</t>
         </is>
       </c>
-      <c r="F11" s="14" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>216 N. Oak Park Ave</t>
         </is>
       </c>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>APPLIED-YELLOW</t>
-        </is>
-      </c>
-      <c r="H11" s="14" t="inlineStr">
-        <is>
-          <t>May Rent. Roommate/co-tenant? ASK</t>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>May Rent. Delach co-tenant CONFIRMED.</t>
         </is>
       </c>
     </row>
@@ -11057,82 +11096,82 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>0203 joint</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>2025-05-30</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>AVA L HERNANDEZ</t>
         </is>
       </c>
-      <c r="D14" s="15" t="n">
+      <c r="D14" s="12" t="n">
         <v>500</v>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>STR / RENTAL INCOME</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
+      <c r="F14" s="11" t="inlineStr">
         <is>
           <t>216 N. Oak Park Ave</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>APPLIED-YELLOW</t>
-        </is>
-      </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>June rent. Roommate/co-tenant? ASK</t>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t>June rent. Delach co-tenant CONFIRMED.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>0203 joint</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>2025-06-23</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>AVA L HERNANDEZ</t>
         </is>
       </c>
-      <c r="D15" s="15" t="n">
+      <c r="D15" s="12" t="n">
         <v>500</v>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>STR / RENTAL INCOME</t>
         </is>
       </c>
-      <c r="F15" s="14" t="inlineStr">
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>216 N. Oak Park Ave</t>
         </is>
       </c>
-      <c r="G15" s="14" t="inlineStr">
-        <is>
-          <t>APPLIED-YELLOW</t>
-        </is>
-      </c>
-      <c r="H15" s="14" t="inlineStr">
-        <is>
-          <t>july rent. Roommate/co-tenant? ASK</t>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>july rent. Delach co-tenant CONFIRMED.</t>
         </is>
       </c>
     </row>
@@ -11217,42 +11256,42 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>0203 joint</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>2025-08-01</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>AVA L HERNANDEZ</t>
         </is>
       </c>
-      <c r="D18" s="15" t="n">
+      <c r="D18" s="12" t="n">
         <v>500</v>
       </c>
-      <c r="E18" s="14" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>STR / RENTAL INCOME</t>
         </is>
       </c>
-      <c r="F18" s="14" t="inlineStr">
+      <c r="F18" s="11" t="inlineStr">
         <is>
           <t>216 N. Oak Park Ave</t>
         </is>
       </c>
-      <c r="G18" s="14" t="inlineStr">
-        <is>
-          <t>APPLIED-YELLOW</t>
-        </is>
-      </c>
-      <c r="H18" s="14" t="inlineStr">
-        <is>
-          <t>August rent. Roommate/co-tenant? ASK</t>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t>August rent. Delach co-tenant CONFIRMED.</t>
         </is>
       </c>
     </row>
@@ -11297,122 +11336,122 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>0203 joint</t>
         </is>
       </c>
-      <c r="B20" s="14" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>2025-08-29</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>AVA L HERNANDEZ</t>
         </is>
       </c>
-      <c r="D20" s="15" t="n">
+      <c r="D20" s="12" t="n">
         <v>500</v>
       </c>
-      <c r="E20" s="14" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>STR / RENTAL INCOME</t>
         </is>
       </c>
-      <c r="F20" s="14" t="inlineStr">
+      <c r="F20" s="11" t="inlineStr">
         <is>
           <t>216 N. Oak Park Ave</t>
         </is>
       </c>
-      <c r="G20" s="14" t="inlineStr">
-        <is>
-          <t>APPLIED-YELLOW</t>
-        </is>
-      </c>
-      <c r="H20" s="14" t="inlineStr">
-        <is>
-          <t>september rent. Roommate/co-tenant? ASK</t>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>september rent. Delach co-tenant CONFIRMED.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>0203 joint</t>
         </is>
       </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>2025-12-01</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>JOAN FRIEDBERGER</t>
         </is>
       </c>
-      <c r="D21" s="15" t="n">
+      <c r="D21" s="12" t="n">
         <v>1950</v>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>STR / RENTAL INCOME</t>
         </is>
       </c>
-      <c r="F21" s="14" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <t>216 N. Oak Park Ave</t>
         </is>
       </c>
-      <c r="G21" s="14" t="inlineStr">
-        <is>
-          <t>APPLIED-YELLOW</t>
-        </is>
-      </c>
-      <c r="H21" s="14" t="inlineStr">
-        <is>
-          <t>rent. Dec occupancy vs prepaid? ASK</t>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+      <c r="H21" s="11" t="inlineStr">
+        <is>
+          <t>rent. December occupancy cash. (Half-Nov $975 not on 0203 — WAIT 8507.)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="inlineStr">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>0203 joint</t>
         </is>
       </c>
-      <c r="B22" s="14" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>2025-12-31</t>
         </is>
       </c>
-      <c r="C22" s="14" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>JOAN FRIEDBERGER</t>
         </is>
       </c>
-      <c r="D22" s="15" t="n">
+      <c r="D22" s="12" t="n">
         <v>1950</v>
       </c>
-      <c r="E22" s="14" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>STR / RENTAL INCOME</t>
         </is>
       </c>
-      <c r="F22" s="14" t="inlineStr">
+      <c r="F22" s="11" t="inlineStr">
         <is>
           <t>216 N. Oak Park Ave</t>
         </is>
       </c>
-      <c r="G22" s="14" t="inlineStr">
-        <is>
-          <t>APPLIED-YELLOW</t>
-        </is>
-      </c>
-      <c r="H22" s="14" t="inlineStr">
-        <is>
-          <t>January rent. Jan 2026 prepaid cash in TY2025. ASK</t>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>January rent. Jan 2026 prepaid cash in TY2025.</t>
         </is>
       </c>
     </row>
@@ -11437,12 +11476,12 @@
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>Consultant</t>
+          <t>Personal 1099</t>
         </is>
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>EPGC LLC + GCM</t>
+          <t>GCM tab + Income E7</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr">
@@ -11452,7 +11491,7 @@
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>BOM PAYMEN</t>
+          <t>BOM PAYMEN — personal 1099, not EPGC</t>
         </is>
       </c>
     </row>
@@ -11477,12 +11516,12 @@
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>Consultant</t>
+          <t>Personal 1099</t>
         </is>
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>EPGC LLC + GCM</t>
+          <t>GCM tab + Income E7</t>
         </is>
       </c>
       <c r="G24" s="11" t="inlineStr">
@@ -11492,7 +11531,7 @@
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>BOM PAYMEN</t>
+          <t>BOM PAYMEN — personal 1099, not EPGC</t>
         </is>
       </c>
     </row>
@@ -11517,12 +11556,12 @@
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>Consultant</t>
+          <t>Personal 1099</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>EPGC LLC + GCM</t>
+          <t>GCM tab + Income E7</t>
         </is>
       </c>
       <c r="G25" s="11" t="inlineStr">
@@ -11532,7 +11571,7 @@
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>BOM PAYMEN</t>
+          <t>BOM PAYMEN — personal 1099, not EPGC</t>
         </is>
       </c>
     </row>
@@ -11557,12 +11596,12 @@
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>Consultant</t>
+          <t>Personal 1099</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>EPGC LLC + GCM</t>
+          <t>GCM tab + Income E7</t>
         </is>
       </c>
       <c r="G26" s="11" t="inlineStr">
@@ -11572,7 +11611,7 @@
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>BOM PAYMEN</t>
+          <t>BOM PAYMEN — personal 1099, not EPGC</t>
         </is>
       </c>
     </row>
@@ -11652,7 +11691,7 @@
       </c>
       <c r="H28" s="13" t="inlineStr">
         <is>
-          <t>JAKE C — no PMT INFO on statement; odd cents, not BOM — treated as reimburse</t>
+          <t>CONFIRMED reimbursement (JAKE C, not BOM)</t>
         </is>
       </c>
     </row>
@@ -11699,7 +11738,7 @@
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>8507 NOW (not in folders)</t>
+          <t>8507 NOW (WAIT-MEGAN statements)</t>
         </is>
       </c>
       <c r="B30" s="13" t="inlineStr">
@@ -11739,7 +11778,7 @@
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>8507 NOW (not in folders)</t>
+          <t>8507 NOW (WAIT-MEGAN statements)</t>
         </is>
       </c>
       <c r="B31" s="13" t="inlineStr">
@@ -11779,7 +11818,7 @@
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>8507 NOW (not in folders)</t>
+          <t>8507 NOW (WAIT-MEGAN statements)</t>
         </is>
       </c>
       <c r="B32" s="13" t="inlineStr">
@@ -11837,7 +11876,7 @@
       </c>
       <c r="E33" s="13" t="inlineStr">
         <is>
-          <t>Annual gift</t>
+          <t>Annual gift to Jake from parents</t>
         </is>
       </c>
       <c r="F33" s="13" t="inlineStr">
@@ -11877,7 +11916,7 @@
       </c>
       <c r="E34" s="13" t="inlineStr">
         <is>
-          <t>Annual gift</t>
+          <t>Annual gift to Jake from parents</t>
         </is>
       </c>
       <c r="F34" s="13" t="inlineStr">
@@ -11917,7 +11956,7 @@
       </c>
       <c r="E35" s="13" t="inlineStr">
         <is>
-          <t>Annual gift</t>
+          <t>Annual gift to Jake from parents</t>
         </is>
       </c>
       <c r="F35" s="13" t="inlineStr">
@@ -11957,7 +11996,7 @@
       </c>
       <c r="E36" s="13" t="inlineStr">
         <is>
-          <t>Annual gift</t>
+          <t>Annual gift to Jake from parents</t>
         </is>
       </c>
       <c r="F36" s="13" t="inlineStr">
@@ -12057,96 +12096,136 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="14" t="inlineStr">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>0203 joint</t>
         </is>
       </c>
-      <c r="B39" s="14" t="inlineStr">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>2025-12-24</t>
         </is>
       </c>
-      <c r="C39" s="14" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr">
         <is>
           <t>Freeman's LLC / CIBC</t>
         </is>
       </c>
-      <c r="D39" s="15" t="n">
+      <c r="D39" s="12" t="n">
         <v>11000</v>
       </c>
-      <c r="E39" s="14" t="inlineStr">
-        <is>
-          <t>Unknown — Sale 6428 Contract</t>
-        </is>
-      </c>
-      <c r="F39" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G39" s="14" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="H39" s="14" t="inlineStr">
-        <is>
-          <t>Not payroll. ASK: art sale vs other.</t>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>Art-sale settlement Sale 6428</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>Art Sales</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+      <c r="H39" s="11" t="inlineStr">
+        <is>
+          <t>Check to Megan. Sale Price $11,000; Cost / object TBD.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="14" t="inlineStr">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t>8507 NOW</t>
         </is>
       </c>
-      <c r="B40" s="14" t="inlineStr">
+      <c r="B40" s="11" t="inlineStr">
         <is>
           <t>2025-12-01</t>
         </is>
       </c>
-      <c r="C40" s="14" t="inlineStr">
+      <c r="C40" s="11" t="inlineStr">
         <is>
           <t>JOAN FRIEDBERGER</t>
         </is>
       </c>
-      <c r="D40" s="15" t="n">
+      <c r="D40" s="12" t="n">
         <v>-675</v>
       </c>
-      <c r="E40" s="14" t="inlineStr">
-        <is>
-          <t>Zelle OUT</t>
-        </is>
-      </c>
-      <c r="F40" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G40" s="14" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="H40" s="14" t="inlineStr">
-        <is>
-          <t>Same day as Joan rent in. Deposit/repair? ASK.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>STATUS: APPLIED = in monthly P&amp;L (green). APPLIED-YELLOW = in P&amp;L pending your yes/no. EXCLUDED = not income. HOLD = parked.</t>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>Repair (Zelle OUT)</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>216 INTERIOR MAINTENANCE</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+      <c r="H40" s="11" t="inlineStr">
+        <is>
+          <t>User: towards a repair. Booked December INTERIOR. Interior vs exterior not specified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="33" t="inlineStr">
+        <is>
+          <t>8507 NOW</t>
+        </is>
+      </c>
+      <c r="B41" s="33" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C41" s="33" t="inlineStr">
+        <is>
+          <t>JOAN FRIEDBERGER</t>
+        </is>
+      </c>
+      <c r="D41" s="34" t="n">
+        <v>975</v>
+      </c>
+      <c r="E41" s="33" t="inlineStr">
+        <is>
+          <t>Half-November rent</t>
+        </is>
+      </c>
+      <c r="F41" s="33" t="inlineStr">
+        <is>
+          <t>216 N. Oak Park Ave</t>
+        </is>
+      </c>
+      <c r="G41" s="33" t="inlineStr">
+        <is>
+          <t>WAIT-MEGAN</t>
+        </is>
+      </c>
+      <c r="H41" s="33" t="inlineStr">
+        <is>
+          <t>User: Joan paid half of November. Not on 0203. Do not book until 8507 shows the deposit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>STATUS: APPLIED = in the workbook. EXCLUDED = not income. WAIT-MEGAN = parked until 8507 statements.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H40"/>
+  <autoFilter ref="A4:H41"/>
   <mergeCells count="3">
-    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A43:H43"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -13208,7 +13287,7 @@
       <c r="D5" t="n">
         <v>1500</v>
       </c>
-      <c r="E5" s="21" t="n">
+      <c r="E5" s="22" t="n">
         <v>19500</v>
       </c>
     </row>
@@ -13240,7 +13319,7 @@
       <c r="D7" t="n">
         <v>21500</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E7" s="22" t="n">
         <v>21500</v>
       </c>
     </row>
@@ -13256,7 +13335,7 @@
       <c r="D8" t="n">
         <v>20000</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13299,10 +13378,10 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="48" customHeight="1">
+    <row r="12" ht="64" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>Notes: E4 Monarch paycheck cash ≠ W-2 Box 1. E5 216 Oak Park LTR cash $19500.00 (Delach+Ava+Joan; Ava/Joan yellow ASK; Oct–Nov vacant ASK). E6 PLATFORM STR net LOCKED. E7 GCM 1099-NEC $21,500 = BOM on Consultant (reimbursements excluded). E8 Art net yellow until Sale Prices filled (COGS on Art Sales). Not tax advice.</t>
+          <t>Notes: E4 Monarch paycheck cash ≠ W-2 Box 1. E5 216 Oak Park LTR cash $19500.00 (Delach + Ava co-tenant CONFIRMED + Joan; vacant Oct + half Nov; half-Nov $975 WAIT 8507). E6 PLATFORM STR net LOCKED. E7 GCM 1099-NEC $21,500 on GCM tab only — NOT EPGC Consultant (reimbursements excluded; May 22 CONFIRMED). E8 Art net $0 until Sale 6428 Cost is filled (Sale Price $11,000 on Art Sales, check to Megan). Not tax advice.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lock Mercury Q6 David Aaron as consultant and Q8 as pass-through.
David Aaron Limited $13,595 (6/24) is EPGC Consultant June, not an art sale.
Koziol/Ariadne $150,000 is a locked pass-through and stays off P&L.
Art Sales MATCHED cash and Income I8 art net are unchanged.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
+++ b/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
@@ -648,7 +648,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="206">
+  <cellXfs count="209">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1077,6 +1077,15 @@
     <xf numFmtId="164" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="27" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="24" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2200,7 +2209,7 @@
     <row r="12" ht="48" customHeight="1" s="137">
       <c r="A12" s="191" t="inlineStr">
         <is>
-          <t>2025 Actual: I4 Monarch paycheck cash ≠ W-2 Box 1. I5 216 LTR cash $19,500. I6 524 #2 STR platform net LOCKED. I7 GCM 1099-NEC $21,500. I8 Art net $23,055.06 = MATCHED Mercury deals only (Berk lots $30,000 − $22,944.94 Cost) + seals $1,000 + mosaics $15,000. Excludes Sale 6428 $11,000 until Cost, David Aaron $13,595 (proposed), Erdal/Aysel/EOEB/L5 ASK. Not tax advice.</t>
+          <t>2025 Actual: I4 Monarch paycheck cash ≠ W-2 Box 1. I5 216 LTR cash $19,500. I6 524 #2 STR platform net LOCKED. I7 GCM 1099-NEC $21,500. I8 Art net $23,055.06 = MATCHED Mercury deals only (Berk lots $30,000 − $22,944.94 Cost) + seals $1,000 + mosaics $15,000. Excludes Sale 6428 $11,000 until Cost. David Aaron $13,595 is EPGC Consultant June (not I8). Erdal/Aysel/EOEB/L5 ASK. Not tax advice.</t>
         </is>
       </c>
       <c r="B12" s="88" t="n"/>
@@ -9932,7 +9941,7 @@
     <row r="1" ht="48" customHeight="1" s="137">
       <c r="A1" s="176" t="inlineStr">
         <is>
-          <t>Mercury Checking 8291 — EPGC LLC (Choice Financial) 2025. 64 unique cash transactions. Coinbase ACH = investment. Newstar = jewelry COGS on intaglios/gems/scarabs. Do not treat BoA 9922 draws or Koziol/Ariadne $150k as P&amp;L until confirmed. Not tax advice.</t>
+          <t>Mercury Checking 8291 — EPGC LLC (Choice Financial) 2025. 64 unique cash transactions. Coinbase ACH = investment. Newstar = jewelry COGS on intaglios/gems/scarabs. BoA 9922 draws and Koziol/Ariadne $150k are LOCKED not-P&amp;L (pass-through / owner transfer). David Aaron $13,595 is LOCKED EPGC Consultant (June). Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -11209,7 +11218,7 @@
           <t>DAVID AARON LIMITED</t>
         </is>
       </c>
-      <c r="C24" s="139" t="n">
+      <c r="C24" s="183" t="n">
         <v>13595</v>
       </c>
       <c r="D24" s="178" t="inlineStr">
@@ -11217,19 +11226,19 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="E24" s="184" t="inlineStr">
-        <is>
-          <t>ART_SALE</t>
-        </is>
-      </c>
-      <c r="F24" s="185" t="inlineStr">
-        <is>
-          <t>PROPOSED</t>
+      <c r="E24" s="181" t="inlineStr">
+        <is>
+          <t>ADVISORY</t>
+        </is>
+      </c>
+      <c r="F24" s="181" t="inlineStr">
+        <is>
+          <t>LOCKED</t>
         </is>
       </c>
       <c r="G24" s="178" t="inlineStr">
         <is>
-          <t>David Aaron Limited — proposed art sale</t>
+          <t>David Aaron Limited — consultant fee</t>
         </is>
       </c>
       <c r="H24" s="178" t="inlineStr">
@@ -11239,7 +11248,7 @@
       </c>
       <c r="I24" s="178" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="J24" s="178" t="inlineStr">
@@ -11254,7 +11263,7 @@
       </c>
       <c r="L24" s="182" t="inlineStr">
         <is>
-          <t>London antiquities dealer; Request or Invoice Payment $13,595. Booked as a proposed sale (yellow) — confirm object / whether this is a purchase refund.</t>
+          <t>User 2026-09-20: consultant fee, not a sale. Hits EPGC Consultant June $13,595. Not Art Sales.</t>
         </is>
       </c>
     </row>
@@ -12769,7 +12778,7 @@
           <t>JACK EDWARD KOZIOL &amp; TRACY HOFFMAN</t>
         </is>
       </c>
-      <c r="C50" s="139" t="n">
+      <c r="C50" s="179" t="n">
         <v>150000</v>
       </c>
       <c r="D50" s="178" t="inlineStr">
@@ -12782,9 +12791,9 @@
           <t>PASS_THROUGH</t>
         </is>
       </c>
-      <c r="F50" s="187" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F50" s="181" t="inlineStr">
+        <is>
+          <t>LOCKED</t>
         </is>
       </c>
       <c r="G50" s="178" t="inlineStr">
@@ -12814,7 +12823,7 @@
       </c>
       <c r="L50" s="182" t="inlineStr">
         <is>
-          <t>Incoming wire /BNF/Per your request. Next-day $150,000 OUT to Ariadne Demirjian LLC. Proposed pass-through — not income unless you say it is a sale.</t>
+          <t>User 2026-09-20: pass-through, not a sale. Incoming wire /BNF/Per your request. Next-day $150,000 OUT to Ariadne Demirjian LLC. Not P&amp;L.</t>
         </is>
       </c>
     </row>
@@ -12829,7 +12838,7 @@
           <t>Ariadne Demirjian LLC</t>
         </is>
       </c>
-      <c r="C51" s="139" t="n">
+      <c r="C51" s="179" t="n">
         <v>-150000</v>
       </c>
       <c r="D51" s="178" t="inlineStr">
@@ -12842,9 +12851,9 @@
           <t>PASS_THROUGH</t>
         </is>
       </c>
-      <c r="F51" s="187" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F51" s="181" t="inlineStr">
+        <is>
+          <t>LOCKED</t>
         </is>
       </c>
       <c r="G51" s="178" t="inlineStr">
@@ -12874,7 +12883,7 @@
       </c>
       <c r="L51" s="182" t="inlineStr">
         <is>
-          <t>Same window as Koziol $150,000 IN. Proposed pass-through — not COGS/expense unless you say it is a purchase.</t>
+          <t>User 2026-09-20: pass-through, not a purchase. Same window as Koziol $150,000 IN. Not P&amp;L.</t>
         </is>
       </c>
     </row>
@@ -13854,7 +13863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" style="137" min="1" max="1"/>
@@ -13865,7 +13874,7 @@
     <row r="1">
       <c r="A1" s="156" t="inlineStr">
         <is>
-          <t>ASK — Mercury 8291 (answer these so EPGC Consultant / remaining sales can be booked). Not tax advice.</t>
+          <t>ASK — remaining Mercury 8291 questions. Q6 David Aaron consultant fee and Q8 Koziol/Ariadne pass-through LOCKED 2026-09-20. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -13942,14 +13951,14 @@
       </c>
     </row>
     <row r="9" ht="48" customHeight="1" s="137">
-      <c r="A9" s="189" t="inlineStr">
-        <is>
-          <t>6. David Aaron Limited $13,595 IN (6/24)</t>
-        </is>
-      </c>
-      <c r="B9" s="190" t="inlineStr">
-        <is>
-          <t>Proposed art sale (London antiquities dealer invoice). Confirm object. If it is a purchase you paid and they refunded, say so.</t>
+      <c r="A9" s="207" t="inlineStr">
+        <is>
+          <t>6. David Aaron Limited $13,595 IN (6/24) — LOCKED consultant fee</t>
+        </is>
+      </c>
+      <c r="B9" s="208" t="inlineStr">
+        <is>
+          <t>CONFIRMED 2026-09-20: consultant fee, not a sale. Booked EPGC Consultant June $13,595 (peach). Not Art Sales. Not Income I8.</t>
         </is>
       </c>
     </row>
@@ -13966,14 +13975,14 @@
       </c>
     </row>
     <row r="11" ht="48" customHeight="1" s="137">
-      <c r="A11" s="189" t="inlineStr">
-        <is>
-          <t>8. Jack Koziol &amp; Tracy Hoffman $150,000 IN (10/20) / Ariadne Demirjian $150,000 OUT (10/21)</t>
-        </is>
-      </c>
-      <c r="B11" s="190" t="inlineStr">
-        <is>
-          <t>Proposed pass-through (not P&amp;L). If this was a real purchase/sale, name the object.</t>
+      <c r="A11" s="207" t="inlineStr">
+        <is>
+          <t>8. Jack Koziol &amp; Tracy Hoffman $150,000 IN (10/20) / Ariadne Demirjian $150,000 OUT (10/21) — LOCKED pass-through</t>
+        </is>
+      </c>
+      <c r="B11" s="208" t="inlineStr">
+        <is>
+          <t>CONFIRMED 2026-09-20: pass-through, not P&amp;L. Not a sale, not a purchase, not COGS, not Consultant.</t>
         </is>
       </c>
     </row>
@@ -14089,6 +14098,30 @@
       <c r="B22" s="181" t="inlineStr">
         <is>
           <t>Jamal Rifai / EPGC / Plutus tests — not P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="181" t="inlineStr">
+        <is>
+          <t>David Aaron Limited</t>
+        </is>
+      </c>
+      <c r="B23" s="181" t="inlineStr">
+        <is>
+          <t>$13,595 (6/24) consultant fee → EPGC Consultant June. Not a sale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="181" t="inlineStr">
+        <is>
+          <t>Koziol / Ariadne</t>
+        </is>
+      </c>
+      <c r="B24" s="181" t="inlineStr">
+        <is>
+          <t>$150,000 IN 10/20 + $150,000 OUT 10/21 LOCKED pass-through — not P&amp;L</t>
         </is>
       </c>
     </row>
@@ -27716,8 +27749,8 @@
       <c r="F54" s="179" t="n">
         <v>0</v>
       </c>
-      <c r="G54" s="179" t="n">
-        <v>0</v>
+      <c r="G54" s="192" t="n">
+        <v>13595</v>
       </c>
       <c r="H54" s="179" t="n">
         <v>0</v>
@@ -28452,7 +28485,7 @@
     <row r="75" ht="72" customHeight="1" s="137">
       <c r="A75" s="182" t="inlineStr">
         <is>
-          <t>2025 Mercury unbundled 2026-09-20: Art Sales = MATCHED cash only (Berk $14,000 Jan + Berk $30,000 / mosaics $105,000 Feb = $149,000). Prior mixed Mercury dump removed. Consultant $0 until EOEB remainder $130,270.00 and L5 $87,396.32 are answered. Coinbase is Investments, not this tab. Newstar $23,581 is Art Sales COGS, not operating expense. 2024 leftover supplies/furniture/consultant-fee numbers on this 2025 block were zeroed. GCM 1099 is personal. Not tax advice.</t>
+          <t>2025 Mercury 2026-09-20: Art Sales = MATCHED cash only (Berk $14,000 Jan + Berk $30,000 / mosaics $105,000 Feb = $149,000). Consultant June $13,595 = David Aaron Limited LOCKED (user: consultant fee, not a sale). EOEB remainder $130,270.00 and L5 $87,396.32 still ASK — not on Consultant. Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments, not this tab. Newstar $23,581 is Art Sales COGS, not operating expense. 2024 leftover supplies/furniture/consultant-fee numbers on this 2025 block were zeroed. GCM 1099 is personal. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -34697,7 +34730,7 @@
     <row r="78" ht="48" customHeight="1" s="137">
       <c r="A78" s="199" t="inlineStr">
         <is>
-          <t>Mercury 8291 MATCHED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics). Fortuna $13,000 (1/8 seals Cost). Plutus $50,000 of mosaics $90,000 Cost — $40,000 of Cost not on 8291 (ASK). Newstar $23,581 is jewelry fabrication COGS, parked below — not in sold-lot Cost (Berk gem/scarab lots already sold in February). Not tax advice.</t>
+          <t>Mercury 8291 MATCHED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics). Fortuna $13,000 (1/8 seals Cost). Plutus $50,000 of mosaics $90,000 Cost — $40,000 of Cost not on 8291 (ASK). Newstar $23,581 is jewelry fabrication COGS, parked below — not in sold-lot Cost (Berk gem/scarab lots already sold in February). David Aaron $13,595 (6/24) is LOCKED consultant fee — not a sale (EPGC Consultant June). Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -35358,43 +35391,32 @@
     </row>
     <row r="118" ht="14.25" customHeight="1" s="137"/>
     <row r="119" ht="14.25" customHeight="1" s="137">
-      <c r="A119" s="156" t="inlineStr">
-        <is>
-          <t>2025 Mercury 8291 — proposed sale / ASK cash (not in EPGC Art Sales until confirmed)</t>
+      <c r="A119" s="201" t="inlineStr">
+        <is>
+          <t>2025 Mercury 8291 — David Aaron Limited is LOCKED consultant fee (not Art Sales)</t>
         </is>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1" s="137">
-      <c r="A120" s="200" t="inlineStr">
-        <is>
-          <t>Proposed: object TBD (David Aaron Limited invoice)</t>
-        </is>
-      </c>
-      <c r="B120" s="200" t="inlineStr">
+      <c r="A120" s="181" t="inlineStr">
+        <is>
+          <t>NOT a 2025 art sale — David Aaron Limited consultant fee (EPGC Consultant June)</t>
+        </is>
+      </c>
+      <c r="B120" s="181" t="inlineStr">
         <is>
           <t>David Aaron Limited</t>
         </is>
       </c>
-      <c r="E120" s="200" t="inlineStr">
-        <is>
-          <t>David Aaron Limited (London)</t>
-        </is>
-      </c>
-      <c r="F120" s="157" t="n">
-        <v>13595</v>
-      </c>
-      <c r="G120" s="0" t="inlineStr">
-        <is>
-          <t>2025-06-24</t>
-        </is>
-      </c>
-      <c r="H120" s="0">
-        <f>IF(OR(F120="",C120=""),"",F120-C120)</f>
-        <v/>
-      </c>
-      <c r="I120" s="200" t="inlineStr">
-        <is>
-          <t>PROPOSED art sale — confirm object. Mercury Request or Invoice Payment.</t>
+      <c r="C120" s="181" t="n"/>
+      <c r="D120" s="181" t="n"/>
+      <c r="E120" s="181" t="n"/>
+      <c r="F120" s="183" t="n"/>
+      <c r="G120" s="206" t="n"/>
+      <c r="H120" s="206" t="n"/>
+      <c r="I120" s="181" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-09-20: consultant fee, not a sale. $13,595 is on EPGC Consultant June. Not tax advice.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lock Mercury Q7 Wise payments as EPGC expertise write-up expenses.
Wise $334.17 (7/9) and $658.63 (10/30) are Consultant Fees, not COGS.
December Wise $565.75 stays reimbursed and off P&L.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
+++ b/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
@@ -9941,7 +9941,7 @@
     <row r="1" ht="48" customHeight="1" s="137">
       <c r="A1" s="176" t="inlineStr">
         <is>
-          <t>Mercury Checking 8291 — EPGC LLC (Choice Financial) 2025. 64 unique cash transactions. Coinbase ACH = investment. Newstar = jewelry COGS on intaglios/gems/scarabs. BoA 9922 draws and Koziol/Ariadne $150k are LOCKED not-P&amp;L (pass-through / owner transfer). David Aaron $13,595 is LOCKED EPGC Consultant (June). Not tax advice.</t>
+          <t>Mercury Checking 8291 — EPGC LLC (Choice Financial) 2025. 64 unique cash transactions. Coinbase ACH = investment. Newstar = jewelry COGS on intaglios/gems/scarabs. BoA 9922 draws and Koziol/Ariadne $150k are LOCKED not-P&amp;L (pass-through / owner transfer). David Aaron $13,595 is LOCKED EPGC Consultant (June). Wise $334.17 + $658.63 are LOCKED EPGC Consultant Fees (expertise write-ups). Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -11398,7 +11398,7 @@
           <t>Wise Inc</t>
         </is>
       </c>
-      <c r="C27" s="139" t="n">
+      <c r="C27" s="183" t="n">
         <v>-334.17</v>
       </c>
       <c r="D27" s="178" t="inlineStr">
@@ -11406,19 +11406,19 @@
           <t>OUT</t>
         </is>
       </c>
-      <c r="E27" s="185" t="inlineStr">
-        <is>
-          <t>ASK</t>
-        </is>
-      </c>
-      <c r="F27" s="185" t="inlineStr">
-        <is>
-          <t>ASK</t>
+      <c r="E27" s="184" t="inlineStr">
+        <is>
+          <t>EPGC_EXPENSE</t>
+        </is>
+      </c>
+      <c r="F27" s="181" t="inlineStr">
+        <is>
+          <t>LOCKED</t>
         </is>
       </c>
       <c r="G27" s="178" t="inlineStr">
         <is>
-          <t>Wise — vendor / COGS / other</t>
+          <t>Wise — expertise write-ups (Consultant Fees)</t>
         </is>
       </c>
       <c r="H27" s="178" t="inlineStr">
@@ -11443,7 +11443,7 @@
       </c>
       <c r="L27" s="182" t="inlineStr">
         <is>
-          <t>International payment from EPGC. Not reimbursed. COGS, advisory cost, or personal?</t>
+          <t>User 2026-09-20: business expense (expertise write-ups). Hits EPGC Consultant Fees July $334.17. Not COGS, not reimbursed. Distinct from Dec Wise $565.75 (EOEB reimburse).</t>
         </is>
       </c>
     </row>
@@ -13018,7 +13018,7 @@
           <t>Wise Inc</t>
         </is>
       </c>
-      <c r="C54" s="139" t="n">
+      <c r="C54" s="183" t="n">
         <v>-658.63</v>
       </c>
       <c r="D54" s="178" t="inlineStr">
@@ -13026,19 +13026,19 @@
           <t>OUT</t>
         </is>
       </c>
-      <c r="E54" s="185" t="inlineStr">
-        <is>
-          <t>ASK</t>
-        </is>
-      </c>
-      <c r="F54" s="185" t="inlineStr">
-        <is>
-          <t>ASK</t>
+      <c r="E54" s="184" t="inlineStr">
+        <is>
+          <t>EPGC_EXPENSE</t>
+        </is>
+      </c>
+      <c r="F54" s="181" t="inlineStr">
+        <is>
+          <t>LOCKED</t>
         </is>
       </c>
       <c r="G54" s="178" t="inlineStr">
         <is>
-          <t>Wise — vendor / COGS / other</t>
+          <t>Wise — expertise write-ups (Consultant Fees)</t>
         </is>
       </c>
       <c r="H54" s="178" t="inlineStr">
@@ -13063,7 +13063,7 @@
       </c>
       <c r="L54" s="182" t="inlineStr">
         <is>
-          <t>International payment from EPGC. Not reimbursed. COGS, advisory cost, or personal?</t>
+          <t>User 2026-09-20: business expense (expertise write-ups). Hits EPGC Consultant Fees October $658.63. Not COGS, not reimbursed. Distinct from Dec Wise $565.75 (EOEB reimburse).</t>
         </is>
       </c>
     </row>
@@ -13863,7 +13863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" style="137" min="1" max="1"/>
@@ -13874,7 +13874,7 @@
     <row r="1">
       <c r="A1" s="156" t="inlineStr">
         <is>
-          <t>ASK — remaining Mercury 8291 questions. Q6 David Aaron consultant fee and Q8 Koziol/Ariadne pass-through LOCKED 2026-09-20. Not tax advice.</t>
+          <t>ASK — remaining Mercury 8291 questions. Q6 consultant, Q7 Wise expertise write-ups, Q8 pass-through LOCKED 2026-09-20. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -13963,14 +13963,14 @@
       </c>
     </row>
     <row r="10" ht="48" customHeight="1" s="137">
-      <c r="A10" s="189" t="inlineStr">
-        <is>
-          <t>7. Wise $334.17 (7/9) and $658.63 (10/30)</t>
-        </is>
-      </c>
-      <c r="B10" s="190" t="inlineStr">
-        <is>
-          <t>Who / what? Dec $565.75 was reimbursed by EOEB (locked net $0). These two were not.</t>
+      <c r="A10" s="207" t="inlineStr">
+        <is>
+          <t>7. Wise $334.17 (7/9) and $658.63 (10/30) — LOCKED expertise write-ups</t>
+        </is>
+      </c>
+      <c r="B10" s="208" t="inlineStr">
+        <is>
+          <t>CONFIRMED 2026-09-20: business expenses (expertise write-ups). Booked EPGC Consultant Fees July $334.17 + October $658.63 = $992.80. Not COGS. Distinct from Dec Wise $565.75 reimbursed by EOEB (still not P&amp;L).</t>
         </is>
       </c>
     </row>
@@ -14122,6 +14122,18 @@
       <c r="B24" s="181" t="inlineStr">
         <is>
           <t>$150,000 IN 10/20 + $150,000 OUT 10/21 LOCKED pass-through — not P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="181" t="inlineStr">
+        <is>
+          <t>Wise expertise write-ups</t>
+        </is>
+      </c>
+      <c r="B25" s="181" t="inlineStr">
+        <is>
+          <t>$334.17 (7/9) + $658.63 (10/30) = $992.80 → EPGC Consultant Fees expense. Dec $565.75 still reimbursed / not P&amp;L.</t>
         </is>
       </c>
     </row>
@@ -28310,20 +28322,42 @@
           <t>Consultant Fees</t>
         </is>
       </c>
-      <c r="B69" s="88" t="n"/>
-      <c r="C69" s="88" t="n"/>
-      <c r="D69" s="88" t="n"/>
-      <c r="E69" s="88" t="n"/>
-      <c r="F69" s="88" t="n"/>
-      <c r="G69" s="88" t="n"/>
-      <c r="H69" s="88" t="n"/>
-      <c r="I69" s="88" t="n"/>
-      <c r="J69" s="194" t="n">
-        <v>0</v>
-      </c>
-      <c r="K69" s="88" t="n"/>
-      <c r="L69" s="88" t="n"/>
-      <c r="M69" s="88" t="n"/>
+      <c r="B69" s="179" t="n">
+        <v>0</v>
+      </c>
+      <c r="C69" s="179" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="179" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" s="179" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" s="179" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" s="179" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" s="192" t="n">
+        <v>334.17</v>
+      </c>
+      <c r="I69" s="179" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" s="179" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" s="192" t="n">
+        <v>658.63</v>
+      </c>
+      <c r="L69" s="179" t="n">
+        <v>0</v>
+      </c>
+      <c r="M69" s="179" t="n">
+        <v>0</v>
+      </c>
       <c r="N69" s="88">
         <f>SUM(B69:M69)</f>
         <v/>
@@ -28485,7 +28519,7 @@
     <row r="75" ht="72" customHeight="1" s="137">
       <c r="A75" s="182" t="inlineStr">
         <is>
-          <t>2025 Mercury 2026-09-20: Art Sales = MATCHED cash only (Berk $14,000 Jan + Berk $30,000 / mosaics $105,000 Feb = $149,000). Consultant June $13,595 = David Aaron Limited LOCKED (user: consultant fee, not a sale). EOEB remainder $130,270.00 and L5 $87,396.32 still ASK — not on Consultant. Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments, not this tab. Newstar $23,581 is Art Sales COGS, not operating expense. 2024 leftover supplies/furniture/consultant-fee numbers on this 2025 block were zeroed. GCM 1099 is personal. Not tax advice.</t>
+          <t>2025 Mercury 2026-09-20: Art Sales = MATCHED cash only (Berk $14,000 Jan + Berk $30,000 / mosaics $105,000 Feb = $149,000). Consultant June $13,595 = David Aaron Limited LOCKED (user: consultant fee, not a sale). Consultant Fees July $334.17 + October $658.63 = Wise expertise write-ups LOCKED ($992.80). EOEB remainder $130,270.00 and L5 $87,396.32 still ASK — not on Consultant income. Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments, not this tab. Newstar $23,581 is Art Sales COGS, not operating expense. Dec Wise $565.75 reimbursed — not on Consultant Fees. GCM 1099 is personal. Not tax advice.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lock Mercury Q9 Aquinas $1,000 as books sold.
Aquinas Hobor 2/4 is EPGC Art Sales February ($150,000 cash). Cost and titles stay TBD so Income I8 net is unchanged.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
+++ b/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
@@ -36,7 +36,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
@@ -44,6 +44,7 @@
     <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="169" formatCode="_([$CAD]\ * #,##0.00_);_([$CAD]\ * \(#,##0.00\);_([$CAD]\ * &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="170" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="171" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="34">
     <font>
@@ -648,7 +649,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="209">
+  <cellXfs count="210">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1086,6 +1087,7 @@
     <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="170" fontId="24" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2209,7 +2211,7 @@
     <row r="12" ht="48" customHeight="1" s="137">
       <c r="A12" s="191" t="inlineStr">
         <is>
-          <t>2025 Actual: I4 Monarch paycheck cash ≠ W-2 Box 1. I5 216 LTR cash $19,500. I6 524 #2 STR platform net LOCKED. I7 GCM 1099-NEC $21,500. I8 Art net $23,055.06 = MATCHED Mercury deals only (Berk lots $30,000 − $22,944.94 Cost) + seals $1,000 + mosaics $15,000. Excludes Sale 6428 $11,000 until Cost. David Aaron $13,595 is EPGC Consultant June (not I8). Erdal/Aysel/EOEB/L5 ASK. Not tax advice.</t>
+          <t>2025 Actual: I4 Monarch paycheck cash ≠ W-2 Box 1. I5 216 LTR cash $19,500. I6 524 #2 STR platform net LOCKED. I7 GCM 1099-NEC $21,500. I8 Art net $23,055.06 = MATCHED Mercury deals only (Berk lots $30,000 − $22,944.94 Cost) + seals $1,000 + mosaics $15,000. Excludes Sale 6428 $11,000 until Cost. Excludes Aquinas books $1,000 until Cost. David Aaron $13,595 is EPGC Consultant June (not I8). Erdal/Aysel/EOEB/L5 ASK. Not tax advice.</t>
         </is>
       </c>
       <c r="B12" s="88" t="n"/>
@@ -9941,7 +9943,7 @@
     <row r="1" ht="48" customHeight="1" s="137">
       <c r="A1" s="176" t="inlineStr">
         <is>
-          <t>Mercury Checking 8291 — EPGC LLC (Choice Financial) 2025. 64 unique cash transactions. Coinbase ACH = investment. Newstar = jewelry COGS on intaglios/gems/scarabs. BoA 9922 draws and Koziol/Ariadne $150k are LOCKED not-P&amp;L (pass-through / owner transfer). David Aaron $13,595 is LOCKED EPGC Consultant (June). Wise $334.17 + $658.63 are LOCKED EPGC Consultant Fees (expertise write-ups). Not tax advice.</t>
+          <t>Mercury Checking 8291 — EPGC LLC (Choice Financial) 2025. 64 unique cash transactions. Coinbase ACH = investment. Newstar = jewelry COGS on intaglios/gems/scarabs. BoA 9922 draws and Koziol/Ariadne $150k are LOCKED not-P&amp;L (pass-through / owner transfer). David Aaron $13,595 is LOCKED EPGC Consultant (June). Wise $334.17 + $658.63 are LOCKED EPGC Consultant Fees (expertise write-ups). Aquinas Hobor $1,000 (2/4) is LOCKED books sold (EPGC Art Sales February; Cost TBD). Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -10258,7 +10260,7 @@
           <t>AQUINAS HOBOR</t>
         </is>
       </c>
-      <c r="C8" s="139" t="n">
+      <c r="C8" s="183" t="n">
         <v>1000</v>
       </c>
       <c r="D8" s="178" t="inlineStr">
@@ -10266,31 +10268,31 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="E8" s="185" t="inlineStr">
-        <is>
-          <t>ASK</t>
-        </is>
-      </c>
-      <c r="F8" s="185" t="inlineStr">
-        <is>
-          <t>ASK</t>
+      <c r="E8" s="184" t="inlineStr">
+        <is>
+          <t>ART_SALE</t>
+        </is>
+      </c>
+      <c r="F8" s="181" t="inlineStr">
+        <is>
+          <t>LOCKED</t>
         </is>
       </c>
       <c r="G8" s="178" t="inlineStr">
         <is>
-          <t>Aquinas Hobor $1,000</t>
+          <t>Books sold to Aquinas Hobor — Sale Price</t>
         </is>
       </c>
       <c r="H8" s="178" t="inlineStr">
         <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I8" s="178" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
-      <c r="I8" s="178" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
       <c r="J8" s="178" t="inlineStr">
         <is>
           <t>Transfer</t>
@@ -10303,7 +10305,7 @@
       </c>
       <c r="L8" s="182" t="inlineStr">
         <is>
-          <t>Prior-year buyer (Saharan bracelets 2022). 2025 sale, leftover, or something else?</t>
+          <t>User 2026-09-20: books sold to Aquinas. Hits EPGC Art Sales February $1,000. Cost / titles TBD (not in I8 net until Cost). Distinct from 2022 Saharan bracelets sale.</t>
         </is>
       </c>
     </row>
@@ -13863,7 +13865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" style="137" min="1" max="1"/>
@@ -13874,7 +13876,7 @@
     <row r="1">
       <c r="A1" s="156" t="inlineStr">
         <is>
-          <t>ASK — remaining Mercury 8291 questions. Q6 consultant, Q7 Wise expertise write-ups, Q8 pass-through LOCKED 2026-09-20. Not tax advice.</t>
+          <t>ASK — remaining Mercury 8291 questions. Q6 consultant, Q7 Wise expertise write-ups, Q8 pass-through, Q9 Aquinas books LOCKED 2026-09-20. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -13987,14 +13989,14 @@
       </c>
     </row>
     <row r="12" ht="48" customHeight="1" s="137">
-      <c r="A12" s="189" t="inlineStr">
-        <is>
-          <t>9. Aquinas Hobor $1,000 IN (2/4)</t>
-        </is>
-      </c>
-      <c r="B12" s="190" t="inlineStr">
-        <is>
-          <t>Sale, leftover, or other? Aquinas bought Saharan bracelets in 2022.</t>
+      <c r="A12" s="207" t="inlineStr">
+        <is>
+          <t>9. Aquinas Hobor $1,000 IN (2/4) — LOCKED books sold</t>
+        </is>
+      </c>
+      <c r="B12" s="208" t="inlineStr">
+        <is>
+          <t>CONFIRMED 2026-09-20: books sold to Aquinas. Booked EPGC Art Sales February $1,000 (peach). Cost / titles TBD — not in Income I8 until Cost. Distinct from 2022 Saharan bracelets.</t>
         </is>
       </c>
     </row>
@@ -14134,6 +14136,18 @@
       <c r="B25" s="181" t="inlineStr">
         <is>
           <t>$334.17 (7/9) + $658.63 (10/30) = $992.80 → EPGC Consultant Fees expense. Dec $565.75 still reimbursed / not P&amp;L.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="181" t="inlineStr">
+        <is>
+          <t>Aquinas Hobor books</t>
+        </is>
+      </c>
+      <c r="B26" s="181" t="inlineStr">
+        <is>
+          <t>$1,000 IN 2/4 LOCKED books sold → EPGC Art Sales February. Cost / titles TBD (not in I8 until Cost).</t>
         </is>
       </c>
     </row>
@@ -27703,7 +27717,7 @@
         <v>14000</v>
       </c>
       <c r="C53" s="192" t="n">
-        <v>135000</v>
+        <v>136000</v>
       </c>
       <c r="D53" s="179" t="n">
         <v>0</v>
@@ -28519,7 +28533,7 @@
     <row r="75" ht="72" customHeight="1" s="137">
       <c r="A75" s="182" t="inlineStr">
         <is>
-          <t>2025 Mercury 2026-09-20: Art Sales = MATCHED cash only (Berk $14,000 Jan + Berk $30,000 / mosaics $105,000 Feb = $149,000). Consultant June $13,595 = David Aaron Limited LOCKED (user: consultant fee, not a sale). Consultant Fees July $334.17 + October $658.63 = Wise expertise write-ups LOCKED ($992.80). EOEB remainder $130,270.00 and L5 $87,396.32 still ASK — not on Consultant income. Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments, not this tab. Newstar $23,581 is Art Sales COGS, not operating expense. Dec Wise $565.75 reimbursed — not on Consultant Fees. GCM 1099 is personal. Not tax advice.</t>
+          <t>2025 Mercury 2026-09-20: Art Sales = MATCHED/LOCKED cash (Berk $14,000 Jan + Berk $30,000 / mosaics $105,000 / Aquinas books $1,000 Feb = $150,000). Consultant June $13,595 = David Aaron Limited LOCKED (user: consultant fee, not a sale). Consultant Fees July $334.17 + October $658.63 = Wise expertise write-ups LOCKED ($992.80). EOEB remainder $130,270.00 and L5 $87,396.32 still ASK — not on Consultant income. Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments, not this tab. Newstar $23,581 is Art Sales COGS, not operating expense. Dec Wise $565.75 reimbursed — not on Consultant Fees. Aquinas books Cost TBD — cash on Art Sales, not in I8. GCM 1099 is personal. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -32069,7 +32083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z132"/>
+  <dimension ref="A1:Z135"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="47.86" customWidth="1" style="137" min="1" max="1"/>
@@ -34764,7 +34778,7 @@
     <row r="78" ht="48" customHeight="1" s="137">
       <c r="A78" s="199" t="inlineStr">
         <is>
-          <t>Mercury 8291 MATCHED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics). Fortuna $13,000 (1/8 seals Cost). Plutus $50,000 of mosaics $90,000 Cost — $40,000 of Cost not on 8291 (ASK). Newstar $23,581 is jewelry fabrication COGS, parked below — not in sold-lot Cost (Berk gem/scarab lots already sold in February). David Aaron $13,595 (6/24) is LOCKED consultant fee — not a sale (EPGC Consultant June). Not tax advice.</t>
+          <t>Mercury 8291 MATCHED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics). Fortuna $13,000 (1/8 seals Cost). Plutus $50,000 of mosaics $90,000 Cost — $40,000 of Cost not on 8291 (ASK). Newstar $23,581 is jewelry fabrication COGS, parked below — not in sold-lot Cost (Berk gem/scarab lots already sold in February). David Aaron $13,595 (6/24) is LOCKED consultant fee — not a sale (EPGC Consultant June). Aquinas Hobor $1,000 (2/4) is LOCKED books sold — EPGC Art Sales February; Cost TBD (not in I8). Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -35642,8 +35656,47 @@
       </c>
     </row>
     <row r="133" ht="14.25" customHeight="1" s="137"/>
-    <row r="134" ht="14.25" customHeight="1" s="137"/>
-    <row r="135" ht="14.25" customHeight="1" s="137"/>
+    <row r="134" ht="14.25" customHeight="1" s="137">
+      <c r="A134" s="201" t="inlineStr">
+        <is>
+          <t>2025 Mercury 8291 — Books sold to Aquinas Hobor (LOCKED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="14.25" customHeight="1" s="137">
+      <c r="A135" s="181" t="inlineStr">
+        <is>
+          <t>Books sold to Aquinas Hobor (titles TBD)</t>
+        </is>
+      </c>
+      <c r="B135" s="181" t="inlineStr">
+        <is>
+          <t>Aquinas Hobor</t>
+        </is>
+      </c>
+      <c r="C135" s="181" t="n"/>
+      <c r="D135" s="181" t="n"/>
+      <c r="E135" s="181" t="inlineStr">
+        <is>
+          <t>Aquinas Hobor</t>
+        </is>
+      </c>
+      <c r="F135" s="183" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G135" s="209" t="n">
+        <v>45692</v>
+      </c>
+      <c r="H135" s="181">
+        <f>IF(C135="","",F135-C135)</f>
+        <v/>
+      </c>
+      <c r="I135" s="181" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-09-20: books sold to Aquinas. $1,000 cash on EPGC Art Sales February. Cost / titles TBD — not in Income I8 until Cost. Distinct from 2022 Saharan bracelets. Not tax advice.</t>
+        </is>
+      </c>
+    </row>
     <row r="136" ht="14.25" customHeight="1" s="137"/>
     <row r="137" ht="14.25" customHeight="1" s="137"/>
     <row r="138" ht="14.25" customHeight="1" s="137"/>
@@ -36510,7 +36563,8 @@
     <row r="999" ht="14.25" customHeight="1" s="137"/>
     <row r="1000" ht="14.25" customHeight="1" s="137"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="A134:I134"/>
     <mergeCell ref="A78:I78"/>
     <mergeCell ref="A119:I119"/>
     <mergeCell ref="A122:I122"/>

</xml_diff>

<commit_message>
Point Drive packet at Q9 Aquinas books sale.
Aquinas $1,000 is EPGC Art Sales February ($150,000 cash). Cost TBD so I8 stays $23,055.06. EOEB/L5 mixed pattern is noted; remainder stays unallocated.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
+++ b/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
@@ -36,7 +36,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
@@ -44,7 +44,6 @@
     <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="169" formatCode="_([$CAD]\ * #,##0.00_);_([$CAD]\ * \(#,##0.00\);_([$CAD]\ * &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="170" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="171" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="34">
     <font>
@@ -649,7 +648,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="210">
+  <cellXfs count="211">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1088,6 +1087,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="170" fontId="24" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1542,7 +1544,7 @@
 Finders Fee</t>
       </text>
     </comment>
-    <comment ref="C80" authorId="0" shapeId="0">
+    <comment ref="C81" authorId="0" shapeId="0">
       <text>
         <t>======
 ID#AAABsxbhmK0
@@ -1551,7 +1553,7 @@
 to Amyas for mount making</t>
       </text>
     </comment>
-    <comment ref="C98" authorId="0" shapeId="0">
+    <comment ref="C99" authorId="0" shapeId="0">
       <text>
         <t>======
 ID#AAABfvHoPDk
@@ -10160,7 +10162,7 @@
       </c>
       <c r="G6" s="178" t="inlineStr">
         <is>
-          <t>EOEB $1,000 — Canosan horse vs advisory</t>
+          <t>EOEB $1,000 — Canosan horse vs advisory (STILL OPEN)</t>
         </is>
       </c>
       <c r="H6" s="178" t="inlineStr">
@@ -10185,7 +10187,7 @@
       </c>
       <c r="L6" s="182" t="inlineStr">
         <is>
-          <t>Art Sales has Canosan Terracotta Horse to Erdal $1,000. This cash is EOEB, not Erdal. Sale or advisory invoice?</t>
+          <t>STILL OPEN after mixed-pattern confirm. Art Sales has Canosan Terracotta Horse to Erdal $1,000. This cash is EOEB, not Erdal. Sale of the horse, advisory invoice, or other? Not allocated.</t>
         </is>
       </c>
     </row>
@@ -10280,7 +10282,7 @@
       </c>
       <c r="G8" s="178" t="inlineStr">
         <is>
-          <t>Books sold to Aquinas Hobor — Sale Price</t>
+          <t>Books (titles TBD) — Sale Price</t>
         </is>
       </c>
       <c r="H8" s="178" t="inlineStr">
@@ -10305,7 +10307,7 @@
       </c>
       <c r="L8" s="182" t="inlineStr">
         <is>
-          <t>User 2026-09-20: books sold to Aquinas. Hits EPGC Art Sales February $1,000. Cost / titles TBD (not in I8 net until Cost). Distinct from 2022 Saharan bracelets sale.</t>
+          <t>User 2026-09-20: book SALE to Aquinas Hobor. Hits EPGC Art Sales February +$1,000. Art Sales register: Books (titles TBD), Cost TBD. Not in Income I8 until Cost is known (same as Sale 6428).</t>
         </is>
       </c>
     </row>
@@ -10880,7 +10882,7 @@
       </c>
       <c r="G18" s="178" t="inlineStr">
         <is>
-          <t>EOEB — sale vs art advisory</t>
+          <t>EOEB — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H18" s="178" t="inlineStr">
@@ -10905,7 +10907,7 @@
       </c>
       <c r="L18" s="182" t="inlineStr">
         <is>
-          <t>Invoice / MAKE A PAYMENT. Not matched to an Art Sales object. Proposed advisory (Consultant) until you say otherwise.</t>
+          <t>User 2026-09-20: EOEB LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump EOEB remainder $130,270 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -10940,7 +10942,7 @@
       </c>
       <c r="G19" s="178" t="inlineStr">
         <is>
-          <t>EOEB — sale vs art advisory</t>
+          <t>EOEB — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H19" s="178" t="inlineStr">
@@ -10965,7 +10967,7 @@
       </c>
       <c r="L19" s="182" t="inlineStr">
         <is>
-          <t>Invoice / MAKE A PAYMENT. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: EOEB LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump EOEB remainder $130,270 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -11060,7 +11062,7 @@
       </c>
       <c r="G21" s="178" t="inlineStr">
         <is>
-          <t>EOEB — sale vs art advisory</t>
+          <t>EOEB — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H21" s="178" t="inlineStr">
@@ -11085,7 +11087,7 @@
       </c>
       <c r="L21" s="182" t="inlineStr">
         <is>
-          <t>Invoice / MAKE A PAYMENT. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: EOEB LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump EOEB remainder $130,270 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -11120,7 +11122,7 @@
       </c>
       <c r="G22" s="178" t="inlineStr">
         <is>
-          <t>EOEB — sale vs art advisory</t>
+          <t>EOEB — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H22" s="178" t="inlineStr">
@@ -11145,7 +11147,7 @@
       </c>
       <c r="L22" s="182" t="inlineStr">
         <is>
-          <t>Invoice / MAKE A PAYMENT. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: EOEB LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump EOEB remainder $130,270 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -11180,7 +11182,7 @@
       </c>
       <c r="G23" s="178" t="inlineStr">
         <is>
-          <t>EOEB — sale vs art advisory</t>
+          <t>EOEB — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H23" s="178" t="inlineStr">
@@ -11205,7 +11207,7 @@
       </c>
       <c r="L23" s="182" t="inlineStr">
         <is>
-          <t>Invoice / MAKE A PAYMENT. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: EOEB LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump EOEB remainder $130,270 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -11360,7 +11362,7 @@
       </c>
       <c r="G26" s="178" t="inlineStr">
         <is>
-          <t>EOEB — sale vs art advisory</t>
+          <t>EOEB — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H26" s="178" t="inlineStr">
@@ -11385,7 +11387,7 @@
       </c>
       <c r="L26" s="182" t="inlineStr">
         <is>
-          <t>Auto-Routing Request or Invoice Payment. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: EOEB LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump EOEB remainder $130,270 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -11480,7 +11482,7 @@
       </c>
       <c r="G28" s="178" t="inlineStr">
         <is>
-          <t>L5 — sale vs art advisory</t>
+          <t>L5 — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H28" s="178" t="inlineStr">
@@ -11505,7 +11507,7 @@
       </c>
       <c r="L28" s="182" t="inlineStr">
         <is>
-          <t>Auto-Routing Request or Invoice Payment. Same invoice pattern as EOEB. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: L5 LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump L5 remainder $87,396.32 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -11540,7 +11542,7 @@
       </c>
       <c r="G29" s="178" t="inlineStr">
         <is>
-          <t>L5 — sale vs art advisory</t>
+          <t>L5 — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H29" s="178" t="inlineStr">
@@ -11565,7 +11567,7 @@
       </c>
       <c r="L29" s="182" t="inlineStr">
         <is>
-          <t>Auto-Routing Request or Invoice Payment. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: L5 LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump L5 remainder $87,396.32 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -11600,7 +11602,7 @@
       </c>
       <c r="G30" s="178" t="inlineStr">
         <is>
-          <t>L5 $50,000 — sale vs art advisory vs pass-through</t>
+          <t>L5 $50,000 — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H30" s="178" t="inlineStr">
@@ -11625,7 +11627,7 @@
       </c>
       <c r="L30" s="182" t="inlineStr">
         <is>
-          <t>Largest L5 invoice. Sale of an object, advisory, or pass-through? Same week as Aysel $50k IN and Fortuna $45k OUT.</t>
+          <t>User 2026-09-20: L5 LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump L5 remainder $87,396.32 onto Consultant or Art Sales. Invoice-level split still ASK. Same week as Aysel $50k IN and Fortuna $45k OUT.</t>
         </is>
       </c>
     </row>
@@ -11960,7 +11962,7 @@
       </c>
       <c r="G36" s="178" t="inlineStr">
         <is>
-          <t>EOEB — sale vs art advisory</t>
+          <t>EOEB — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H36" s="178" t="inlineStr">
@@ -11985,7 +11987,7 @@
       </c>
       <c r="L36" s="182" t="inlineStr">
         <is>
-          <t>Auto-Routing. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: EOEB LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump EOEB remainder $130,270 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -12020,7 +12022,7 @@
       </c>
       <c r="G37" s="178" t="inlineStr">
         <is>
-          <t>L5 — sale vs art advisory</t>
+          <t>L5 — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H37" s="178" t="inlineStr">
@@ -12045,7 +12047,7 @@
       </c>
       <c r="L37" s="182" t="inlineStr">
         <is>
-          <t>Auto-Routing. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: L5 LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump L5 remainder $87,396.32 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -12140,7 +12142,7 @@
       </c>
       <c r="G39" s="178" t="inlineStr">
         <is>
-          <t>EOEB — sale vs art advisory</t>
+          <t>EOEB — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H39" s="178" t="inlineStr">
@@ -12165,7 +12167,7 @@
       </c>
       <c r="L39" s="182" t="inlineStr">
         <is>
-          <t>Auto-Routing. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: EOEB LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump EOEB remainder $130,270 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -12200,7 +12202,7 @@
       </c>
       <c r="G40" s="178" t="inlineStr">
         <is>
-          <t>L5 — sale vs art advisory</t>
+          <t>L5 — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H40" s="178" t="inlineStr">
@@ -12225,7 +12227,7 @@
       </c>
       <c r="L40" s="182" t="inlineStr">
         <is>
-          <t>Auto-Routing. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: L5 LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump L5 remainder $87,396.32 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -12320,7 +12322,7 @@
       </c>
       <c r="G42" s="178" t="inlineStr">
         <is>
-          <t>EOEB — sale vs art advisory</t>
+          <t>EOEB — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H42" s="178" t="inlineStr">
@@ -12345,7 +12347,7 @@
       </c>
       <c r="L42" s="182" t="inlineStr">
         <is>
-          <t>Auto-Routing. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: EOEB LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump EOEB remainder $130,270 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -12500,7 +12502,7 @@
       </c>
       <c r="G45" s="178" t="inlineStr">
         <is>
-          <t>EOEB — sale vs art advisory</t>
+          <t>EOEB — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H45" s="178" t="inlineStr">
@@ -12525,7 +12527,7 @@
       </c>
       <c r="L45" s="182" t="inlineStr">
         <is>
-          <t>Auto-Routing. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: EOEB LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump EOEB remainder $130,270 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -12740,7 +12742,7 @@
       </c>
       <c r="G49" s="178" t="inlineStr">
         <is>
-          <t>EOEB — sale vs art advisory</t>
+          <t>EOEB — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H49" s="178" t="inlineStr">
@@ -12765,7 +12767,7 @@
       </c>
       <c r="L49" s="182" t="inlineStr">
         <is>
-          <t>Auto-Routing. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: EOEB LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump EOEB remainder $130,270 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -12920,7 +12922,7 @@
       </c>
       <c r="G52" s="178" t="inlineStr">
         <is>
-          <t>L5 — sale vs art advisory</t>
+          <t>L5 — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H52" s="178" t="inlineStr">
@@ -12945,7 +12947,7 @@
       </c>
       <c r="L52" s="182" t="inlineStr">
         <is>
-          <t>Auto-Routing. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: L5 LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump L5 remainder $87,396.32 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -12980,7 +12982,7 @@
       </c>
       <c r="G53" s="178" t="inlineStr">
         <is>
-          <t>EOEB — sale vs art advisory</t>
+          <t>EOEB — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H53" s="178" t="inlineStr">
@@ -13005,7 +13007,7 @@
       </c>
       <c r="L53" s="182" t="inlineStr">
         <is>
-          <t>Auto-Routing. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: EOEB LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump EOEB remainder $130,270 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -13100,7 +13102,7 @@
       </c>
       <c r="G55" s="178" t="inlineStr">
         <is>
-          <t>EOEB — sale vs art advisory</t>
+          <t>EOEB — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H55" s="178" t="inlineStr">
@@ -13125,7 +13127,7 @@
       </c>
       <c r="L55" s="182" t="inlineStr">
         <is>
-          <t>Auto-Routing. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: EOEB LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump EOEB remainder $130,270 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -13640,7 +13642,7 @@
       </c>
       <c r="G64" s="178" t="inlineStr">
         <is>
-          <t>L5 — sale vs art advisory</t>
+          <t>L5 — mixed unallocated (sale vs advisory)</t>
         </is>
       </c>
       <c r="H64" s="178" t="inlineStr">
@@ -13665,7 +13667,7 @@
       </c>
       <c r="L64" s="182" t="inlineStr">
         <is>
-          <t>Auto-Routing. Proposed advisory until confirmed.</t>
+          <t>User 2026-09-20: L5 LLC mixed art sales AND advisory/consultant fees. Pattern confirmed; this invoice still unallocated. Do NOT dump L5 remainder $87,396.32 onto Consultant or Art Sales. Invoice-level split still ASK.</t>
         </is>
       </c>
     </row>
@@ -13876,7 +13878,7 @@
     <row r="1">
       <c r="A1" s="156" t="inlineStr">
         <is>
-          <t>ASK — remaining Mercury 8291 questions. Q6 consultant, Q7 Wise expertise write-ups, Q8 pass-through, Q9 Aquinas books LOCKED 2026-09-20. Not tax advice.</t>
+          <t>ASK — remaining Mercury 8291 questions. Q6 consultant, Q7 Wise expertise, Q8 pass-through, Q9 Aquinas books LOCKED (green). Q1/Q2 mixed pattern CONFIRMED, dollars unallocated (yellow). Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -13895,24 +13897,24 @@
     <row r="4" ht="48" customHeight="1" s="137">
       <c r="A4" s="189" t="inlineStr">
         <is>
-          <t>1. EOEB LLC remainder after mosaics</t>
+          <t>1. EOEB LLC remainder after mosaics — MIXED PATTERN CONFIRMED, dollars unallocated</t>
         </is>
       </c>
       <c r="B4" s="190" t="inlineStr">
         <is>
-          <t>$130,270.00 of EOEB IN is not the $105,000 mosaics sale and not the $565.75 Wise reimbursement. Invoice / MAKE A PAYMENT pattern. Book as art advisory (EPGC Consultant) or as more art sales? Jan 16 $1,000 might be the Canosan horse (sold to Erdal $1,000 on Art Sales) — yes/no?</t>
+          <t>$130,270.00 of EOEB IN is not mosaics $105,000 and not Wise reimburse $565.75. User 2026-09-20: EOEB is mixed art sales AND advisory/consultant fees. Do NOT dump this remainder onto Consultant or Art Sales. Invoice-level split still ASK. Jan 16 $1,000 Canosan-horse question STILL OPEN (Art Sales horse is to Erdal; this cash is EOEB).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" s="137">
       <c r="A5" s="189" t="inlineStr">
         <is>
-          <t>2. L5 (all seven invoices)</t>
+          <t>2. L5 (all seven invoices) — MIXED PATTERN CONFIRMED, dollars unallocated</t>
         </is>
       </c>
       <c r="B5" s="190" t="inlineStr">
         <is>
-          <t>$87,396.32. Same Auto-Routing Request or Invoice Payment pattern as EOEB. Advisory fees, art sales, or mixed? The 7/15 $50,000 lands the same week as Aysel $50k and Fortuna $45k.</t>
+          <t>$87,396.32. User 2026-09-20: L5 is mixed art sales AND advisory/consultant fees. Do NOT dump onto Consultant or Art Sales. Invoice-level split still ASK. The 7/15 $50,000 still sits in the Aysel $50k / Fortuna $45k week.</t>
         </is>
       </c>
     </row>
@@ -13991,12 +13993,12 @@
     <row r="12" ht="48" customHeight="1" s="137">
       <c r="A12" s="207" t="inlineStr">
         <is>
-          <t>9. Aquinas Hobor $1,000 IN (2/4) — LOCKED books sold</t>
+          <t>9. Aquinas Hobor $1,000 IN (2/4) — LOCKED book sale</t>
         </is>
       </c>
       <c r="B12" s="208" t="inlineStr">
         <is>
-          <t>CONFIRMED 2026-09-20: books sold to Aquinas. Booked EPGC Art Sales February $1,000 (peach). Cost / titles TBD — not in Income I8 until Cost. Distinct from 2022 Saharan bracelets.</t>
+          <t>CONFIRMED 2026-09-20: book SALE. Hits EPGC Art Sales February +$1,000 (Feb $136,000; matched cash $150,000). Art Sales register: Books (titles TBD) to Aquinas Hobor, Sale Price $1,000, Sale Date 2025-02-04, Cost TBD. Not in Income I8 until Cost (same as Sale 6428).</t>
         </is>
       </c>
     </row>
@@ -14147,7 +14149,7 @@
       </c>
       <c r="B26" s="181" t="inlineStr">
         <is>
-          <t>$1,000 IN 2/4 LOCKED books sold → EPGC Art Sales February. Cost / titles TBD (not in I8 until Cost).</t>
+          <t>$1,000 IN 2/4 LOCKED book sale → EPGC Art Sales February +$1,000 (Feb $136,000; matched cash $150,000). Cost / titles TBD (not in I8 until Cost, same as Sale 6428).</t>
         </is>
       </c>
     </row>
@@ -28533,7 +28535,7 @@
     <row r="75" ht="72" customHeight="1" s="137">
       <c r="A75" s="182" t="inlineStr">
         <is>
-          <t>2025 Mercury 2026-09-20: Art Sales = MATCHED/LOCKED cash (Berk $14,000 Jan + Berk $30,000 / mosaics $105,000 / Aquinas books $1,000 Feb = $150,000). Consultant June $13,595 = David Aaron Limited LOCKED (user: consultant fee, not a sale). Consultant Fees July $334.17 + October $658.63 = Wise expertise write-ups LOCKED ($992.80). EOEB remainder $130,270.00 and L5 $87,396.32 still ASK — not on Consultant income. Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments, not this tab. Newstar $23,581 is Art Sales COGS, not operating expense. Dec Wise $565.75 reimbursed — not on Consultant Fees. Aquinas books Cost TBD — cash on Art Sales, not in I8. GCM 1099 is personal. Not tax advice.</t>
+          <t>2025 Mercury 2026-09-20: Art Sales = MATCHED/LOCKED cash (Berk $14,000 Jan + Berk $30,000 / mosaics $105,000 / Aquinas books $1,000 Feb = $150,000). Consultant June $13,595 = David Aaron Limited LOCKED (user: consultant fee, not a sale). Consultant Fees July $334.17 + October $658.63 = Wise expertise write-ups LOCKED ($992.80). EOEB remainder $130,270.00 and L5 $87,396.32 MIXED PATTERN CONFIRMED (art sales + advisory/consultant) — invoice-level split still ASK; not dumped onto Consultant or Art Sales. Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments, not this tab. Newstar $23,581 is Art Sales COGS, not operating expense. Dec Wise $565.75 reimbursed — not on Consultant Fees. Aquinas books Cost TBD — cash on Art Sales, not in I8. GCM 1099 is personal. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -32083,7 +32085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z135"/>
+  <dimension ref="A1:Z134"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="47.86" customWidth="1" style="137" min="1" max="1"/>
@@ -34758,94 +34760,97 @@
       <c r="I76" s="105" t="n"/>
     </row>
     <row r="77" ht="14.25" customHeight="1" s="137">
-      <c r="A77" s="89" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B77" s="104" t="n"/>
-      <c r="C77" s="114" t="n"/>
-      <c r="D77" s="113" t="n"/>
-      <c r="E77" s="113" t="n"/>
-      <c r="F77" s="114" t="n"/>
-      <c r="G77" s="113" t="n"/>
-      <c r="H77" s="114">
-        <f>SUM(H51:H75)</f>
-        <v/>
-      </c>
-      <c r="I77" s="105" t="n"/>
+      <c r="A77" s="181" t="inlineStr">
+        <is>
+          <t>Books (titles TBD)</t>
+        </is>
+      </c>
+      <c r="B77" s="185" t="inlineStr">
+        <is>
+          <t>Cost TBD</t>
+        </is>
+      </c>
+      <c r="C77" s="200" t="n"/>
+      <c r="E77" s="181" t="inlineStr">
+        <is>
+          <t>Aquinas Hobor</t>
+        </is>
+      </c>
+      <c r="F77" s="183" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G77" s="209" t="n">
+        <v>45692</v>
+      </c>
+      <c r="H77" s="178">
+        <f>IF(OR(F77="",C77=""),"",F77-C77)</f>
+        <v/>
+      </c>
+      <c r="I77" s="190" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-09-20: book SALE $1,000 on Mercury 8291. Cost TBD — not in Income I8 yet (same as Sale 6428). Titles TBD. Not tax advice.</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="48" customHeight="1" s="137">
-      <c r="A78" s="199" t="inlineStr">
+      <c r="A78" s="210" t="inlineStr">
         <is>
           <t>Mercury 8291 MATCHED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics). Fortuna $13,000 (1/8 seals Cost). Plutus $50,000 of mosaics $90,000 Cost — $40,000 of Cost not on 8291 (ASK). Newstar $23,581 is jewelry fabrication COGS, parked below — not in sold-lot Cost (Berk gem/scarab lots already sold in February). David Aaron $13,595 (6/24) is LOCKED consultant fee — not a sale (EPGC Consultant June). Aquinas Hobor $1,000 (2/4) is LOCKED books sold — EPGC Art Sales February; Cost TBD (not in I8). Not tax advice.</t>
         </is>
       </c>
     </row>
     <row r="79" ht="14.25" customHeight="1" s="137">
-      <c r="A79" s="119" t="inlineStr">
+      <c r="A79" s="199" t="inlineStr">
+        <is>
+          <t>Mercury 8291 MATCHED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics). Fortuna $13,000 (1/8 seals Cost). Plutus $50,000 of mosaics $90,000 Cost — $40,000 of Cost not on 8291 (ASK). Newstar $23,581 is jewelry fabrication COGS, parked below — not in sold-lot Cost (Berk gem/scarab lots already sold in February). David Aaron $13,595 (6/24) is LOCKED consultant fee — not a sale (EPGC Consultant June). Aquinas Hobor $1,000 (2/4) is LOCKED books sold — EPGC Art Sales February; Cost TBD (not in I8). Not tax advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="14.25" customHeight="1" s="137">
+      <c r="A80" s="119" t="inlineStr">
         <is>
           <t>Art Purchases/Inventory</t>
         </is>
       </c>
-      <c r="B79" s="120" t="n"/>
-      <c r="C79" s="100" t="n"/>
-      <c r="D79" s="101" t="n"/>
-      <c r="E79" s="99" t="n"/>
-      <c r="F79" s="100" t="n"/>
-      <c r="G79" s="101" t="n"/>
-      <c r="H79" s="99" t="n"/>
-      <c r="I79" s="121" t="n"/>
-      <c r="J79" s="99" t="n"/>
-      <c r="K79" s="99" t="n"/>
-      <c r="L79" s="99" t="n"/>
-      <c r="M79" s="99" t="n"/>
-      <c r="N79" s="99" t="n"/>
-      <c r="O79" s="99" t="n"/>
-      <c r="P79" s="99" t="n"/>
-      <c r="Q79" s="99" t="n"/>
-      <c r="R79" s="99" t="n"/>
-      <c r="S79" s="99" t="n"/>
-      <c r="T79" s="99" t="n"/>
-      <c r="U79" s="99" t="n"/>
-      <c r="V79" s="99" t="n"/>
-      <c r="W79" s="99" t="n"/>
-      <c r="X79" s="99" t="n"/>
-      <c r="Y79" s="99" t="n"/>
-      <c r="Z79" s="99" t="n"/>
-    </row>
-    <row r="80" ht="14.25" customHeight="1" s="137">
-      <c r="A80" s="122" t="inlineStr">
-        <is>
-          <t>30 Paleothic and Neolithic Stone Tools</t>
-        </is>
-      </c>
-      <c r="B80" s="116" t="inlineStr">
-        <is>
-          <t>Holestein</t>
-        </is>
-      </c>
-      <c r="C80" s="88" t="n">
-        <v>4000</v>
-      </c>
-      <c r="E80" s="105" t="n"/>
+      <c r="B80" s="120" t="n"/>
+      <c r="C80" s="100" t="n"/>
+      <c r="D80" s="101" t="n"/>
+      <c r="E80" s="99" t="n"/>
+      <c r="F80" s="100" t="n"/>
+      <c r="G80" s="101" t="n"/>
+      <c r="H80" s="99" t="n"/>
+      <c r="I80" s="121" t="n"/>
+      <c r="J80" s="99" t="n"/>
+      <c r="K80" s="99" t="n"/>
+      <c r="L80" s="99" t="n"/>
+      <c r="M80" s="99" t="n"/>
+      <c r="N80" s="99" t="n"/>
+      <c r="O80" s="99" t="n"/>
+      <c r="P80" s="99" t="n"/>
+      <c r="Q80" s="99" t="n"/>
+      <c r="R80" s="99" t="n"/>
+      <c r="S80" s="99" t="n"/>
+      <c r="T80" s="99" t="n"/>
+      <c r="U80" s="99" t="n"/>
+      <c r="V80" s="99" t="n"/>
+      <c r="W80" s="99" t="n"/>
+      <c r="X80" s="99" t="n"/>
+      <c r="Y80" s="99" t="n"/>
+      <c r="Z80" s="99" t="n"/>
     </row>
     <row r="81" ht="14.25" customHeight="1" s="137">
       <c r="A81" s="122" t="inlineStr">
         <is>
-          <t>A Tairona Figure</t>
+          <t>30 Paleothic and Neolithic Stone Tools</t>
         </is>
       </c>
       <c r="B81" s="116" t="inlineStr">
         <is>
-          <t>Live Auctioneers</t>
+          <t>Holestein</t>
         </is>
       </c>
       <c r="C81" s="88" t="n">
-        <v>250</v>
-      </c>
-      <c r="D81" s="92" t="n">
-        <v>45119</v>
+        <v>4000</v>
       </c>
       <c r="E81" s="105" t="n"/>
     </row>
@@ -34861,7 +34866,7 @@
         </is>
       </c>
       <c r="C82" s="88" t="n">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="D82" s="92" t="n">
         <v>45119</v>
@@ -34871,26 +34876,26 @@
     <row r="83" ht="14.25" customHeight="1" s="137">
       <c r="A83" s="122" t="inlineStr">
         <is>
-          <t>A Pair of Greek Bronze Greeves</t>
+          <t>A Tairona Figure</t>
         </is>
       </c>
       <c r="B83" s="116" t="inlineStr">
         <is>
-          <t>ebay</t>
+          <t>Live Auctioneers</t>
         </is>
       </c>
       <c r="C83" s="88" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D83" s="92" t="n">
-        <v>45145</v>
+        <v>45119</v>
       </c>
       <c r="E83" s="105" t="n"/>
     </row>
     <row r="84" ht="14.25" customHeight="1" s="137">
       <c r="A84" s="122" t="inlineStr">
         <is>
-          <t>An Illyrian Bronze Helmet</t>
+          <t>A Pair of Greek Bronze Greeves</t>
         </is>
       </c>
       <c r="B84" s="116" t="inlineStr">
@@ -34899,58 +34904,57 @@
         </is>
       </c>
       <c r="C84" s="88" t="n">
-        <v>551.25</v>
+        <v>200</v>
       </c>
       <c r="D84" s="92" t="n">
-        <v>45114</v>
+        <v>45145</v>
       </c>
       <c r="E84" s="105" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1" s="137">
       <c r="A85" s="122" t="inlineStr">
         <is>
-          <t>An Egyptian Faience Ibis</t>
-        </is>
-      </c>
-      <c r="B85" s="104" t="inlineStr">
-        <is>
-          <t>Hindman</t>
+          <t>An Illyrian Bronze Helmet</t>
+        </is>
+      </c>
+      <c r="B85" s="116" t="inlineStr">
+        <is>
+          <t>ebay</t>
         </is>
       </c>
       <c r="C85" s="88" t="n">
-        <v>375</v>
+        <v>551.25</v>
       </c>
       <c r="D85" s="92" t="n">
-        <v>44343</v>
-      </c>
-      <c r="E85" s="92" t="n"/>
-      <c r="F85" s="88" t="n"/>
-      <c r="I85" s="105" t="n"/>
+        <v>45114</v>
+      </c>
+      <c r="E85" s="105" t="n"/>
     </row>
     <row r="86" ht="14.25" customHeight="1" s="137">
       <c r="A86" s="122" t="inlineStr">
         <is>
-          <t>African Stone Bracelet Upper Volta River 1 0f 4</t>
+          <t>An Egyptian Faience Ibis</t>
         </is>
       </c>
       <c r="B86" s="104" t="inlineStr">
         <is>
-          <t>Live Auctioneers</t>
+          <t>Hindman</t>
         </is>
       </c>
       <c r="C86" s="88" t="n">
-        <v>293</v>
+        <v>375</v>
       </c>
       <c r="D86" s="92" t="n">
-        <v>44548</v>
-      </c>
+        <v>44343</v>
+      </c>
+      <c r="E86" s="92" t="n"/>
       <c r="F86" s="88" t="n"/>
       <c r="I86" s="105" t="n"/>
     </row>
     <row r="87" ht="14.25" customHeight="1" s="137">
       <c r="A87" s="122" t="inlineStr">
         <is>
-          <t>African Stone Bracelet Upper Volta River 2 0f 4</t>
+          <t>African Stone Bracelet Upper Volta River 1 0f 4</t>
         </is>
       </c>
       <c r="B87" s="104" t="inlineStr">
@@ -34970,7 +34974,7 @@
     <row r="88" ht="14.25" customHeight="1" s="137">
       <c r="A88" s="122" t="inlineStr">
         <is>
-          <t>African Stone Bracelet Upper Volta River 4 0f 4</t>
+          <t>African Stone Bracelet Upper Volta River 2 0f 4</t>
         </is>
       </c>
       <c r="B88" s="104" t="inlineStr">
@@ -34990,19 +34994,19 @@
     <row r="89" ht="14.25" customHeight="1" s="137">
       <c r="A89" s="122" t="inlineStr">
         <is>
-          <t>A Saharan Stone Discoidal</t>
+          <t>African Stone Bracelet Upper Volta River 4 0f 4</t>
         </is>
       </c>
       <c r="B89" s="104" t="inlineStr">
         <is>
-          <t>Pace African Art</t>
+          <t>Live Auctioneers</t>
         </is>
       </c>
       <c r="C89" s="88" t="n">
-        <v>1000</v>
+        <v>293</v>
       </c>
       <c r="D89" s="92" t="n">
-        <v>44562</v>
+        <v>44548</v>
       </c>
       <c r="F89" s="88" t="n"/>
       <c r="I89" s="105" t="n"/>
@@ -35010,16 +35014,19 @@
     <row r="90" ht="14.25" customHeight="1" s="137">
       <c r="A90" s="122" t="inlineStr">
         <is>
-          <t>Carved Ostrish Egg</t>
+          <t>A Saharan Stone Discoidal</t>
         </is>
       </c>
       <c r="B90" s="104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Etsy </t>
+          <t>Pace African Art</t>
         </is>
       </c>
       <c r="C90" s="88" t="n">
-        <v>90</v>
+        <v>1000</v>
+      </c>
+      <c r="D90" s="92" t="n">
+        <v>44562</v>
       </c>
       <c r="F90" s="88" t="n"/>
       <c r="I90" s="105" t="n"/>
@@ -35027,16 +35034,16 @@
     <row r="91" ht="14.25" customHeight="1" s="137">
       <c r="A91" s="122" t="inlineStr">
         <is>
-          <t>Carved Goose Egg</t>
+          <t>Carved Ostrish Egg</t>
         </is>
       </c>
       <c r="B91" s="104" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t xml:space="preserve">Etsy </t>
         </is>
       </c>
       <c r="C91" s="88" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="F91" s="88" t="n"/>
       <c r="I91" s="105" t="n"/>
@@ -35053,7 +35060,7 @@
         </is>
       </c>
       <c r="C92" s="88" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F92" s="88" t="n"/>
       <c r="I92" s="105" t="n"/>
@@ -35061,31 +35068,29 @@
     <row r="93" ht="14.25" customHeight="1" s="137">
       <c r="A93" s="122" t="inlineStr">
         <is>
-          <t>Quimbaya Figure (Gift)</t>
+          <t>Carved Goose Egg</t>
         </is>
       </c>
       <c r="B93" s="104" t="inlineStr">
         <is>
-          <t>Jeffrey Norris</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C93" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="D93" s="92" t="n">
-        <v>45079</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="F93" s="88" t="n"/>
       <c r="I93" s="105" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1" s="137">
       <c r="A94" s="122" t="inlineStr">
         <is>
-          <t>A Saharan Stone Discoidal (Gift)</t>
+          <t>Quimbaya Figure (Gift)</t>
         </is>
       </c>
       <c r="B94" s="104" t="inlineStr">
         <is>
-          <t>Aquinas Hobor</t>
+          <t>Jeffrey Norris</t>
         </is>
       </c>
       <c r="C94" s="88" t="n">
@@ -35099,7 +35104,7 @@
     <row r="95" ht="14.25" customHeight="1" s="137">
       <c r="A95" s="122" t="inlineStr">
         <is>
-          <t>A Saharan Stone Discoidal</t>
+          <t>A Saharan Stone Discoidal (Gift)</t>
         </is>
       </c>
       <c r="B95" s="104" t="inlineStr">
@@ -35107,31 +35112,30 @@
           <t>Aquinas Hobor</t>
         </is>
       </c>
-      <c r="C95" s="103" t="n">
-        <v>500</v>
+      <c r="C95" s="88" t="n">
+        <v>10</v>
       </c>
       <c r="D95" s="92" t="n">
         <v>45079</v>
       </c>
-      <c r="F95" s="88" t="n"/>
       <c r="I95" s="105" t="n"/>
     </row>
     <row r="96" ht="14.25" customHeight="1" s="137">
       <c r="A96" s="122" t="inlineStr">
         <is>
-          <t>Two Songye and Bozo Vessels</t>
+          <t>A Saharan Stone Discoidal</t>
         </is>
       </c>
       <c r="B96" s="104" t="inlineStr">
         <is>
-          <t>Hindman</t>
+          <t>Aquinas Hobor</t>
         </is>
       </c>
       <c r="C96" s="103" t="n">
-        <v>138.91</v>
+        <v>500</v>
       </c>
       <c r="D96" s="92" t="n">
-        <v>45211</v>
+        <v>45079</v>
       </c>
       <c r="F96" s="88" t="n"/>
       <c r="I96" s="105" t="n"/>
@@ -35139,19 +35143,19 @@
     <row r="97" ht="14.25" customHeight="1" s="137">
       <c r="A97" s="122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sword 9th Century </t>
+          <t>Two Songye and Bozo Vessels</t>
         </is>
       </c>
       <c r="B97" s="104" t="inlineStr">
         <is>
-          <t>Zevantiques</t>
+          <t>Hindman</t>
         </is>
       </c>
       <c r="C97" s="103" t="n">
-        <v>3000</v>
+        <v>138.91</v>
       </c>
       <c r="D97" s="92" t="n">
-        <v>45311</v>
+        <v>45211</v>
       </c>
       <c r="F97" s="88" t="n"/>
       <c r="I97" s="105" t="n"/>
@@ -35159,19 +35163,19 @@
     <row r="98" ht="14.25" customHeight="1" s="137">
       <c r="A98" s="122" t="inlineStr">
         <is>
-          <t>A Roman Marble Plaque with Insciption</t>
+          <t xml:space="preserve">Sword 9th Century </t>
         </is>
       </c>
       <c r="B98" s="104" t="inlineStr">
         <is>
-          <t>ebay</t>
+          <t>Zevantiques</t>
         </is>
       </c>
       <c r="C98" s="103" t="n">
-        <v>1331.41</v>
+        <v>3000</v>
       </c>
       <c r="D98" s="92" t="n">
-        <v>45546</v>
+        <v>45311</v>
       </c>
       <c r="F98" s="88" t="n"/>
       <c r="I98" s="105" t="n"/>
@@ -35179,7 +35183,7 @@
     <row r="99" ht="14.25" customHeight="1" s="137">
       <c r="A99" s="122" t="inlineStr">
         <is>
-          <t>Erotic Intaglio Finger Ring</t>
+          <t>A Roman Marble Plaque with Insciption</t>
         </is>
       </c>
       <c r="B99" s="104" t="inlineStr">
@@ -35188,85 +35192,94 @@
         </is>
       </c>
       <c r="C99" s="103" t="n">
-        <v>205.07</v>
+        <v>1331.41</v>
       </c>
       <c r="D99" s="92" t="n">
-        <v>45446</v>
+        <v>45546</v>
       </c>
       <c r="F99" s="88" t="n"/>
       <c r="I99" s="105" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1" s="137">
-      <c r="B100" s="104" t="n"/>
-      <c r="C100" s="103" t="n"/>
-      <c r="D100" s="92" t="n"/>
+      <c r="A100" s="122" t="inlineStr">
+        <is>
+          <t>Erotic Intaglio Finger Ring</t>
+        </is>
+      </c>
+      <c r="B100" s="104" t="inlineStr">
+        <is>
+          <t>ebay</t>
+        </is>
+      </c>
+      <c r="C100" s="103" t="n">
+        <v>205.07</v>
+      </c>
+      <c r="D100" s="92" t="n">
+        <v>45446</v>
+      </c>
       <c r="F100" s="88" t="n"/>
       <c r="I100" s="105" t="n"/>
     </row>
     <row r="101" ht="14.25" customHeight="1" s="137">
-      <c r="A101" s="5" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
       <c r="B101" s="104" t="n"/>
-      <c r="C101" s="86" t="n"/>
+      <c r="C101" s="103" t="n"/>
+      <c r="D101" s="92" t="n"/>
       <c r="F101" s="88" t="n"/>
       <c r="I101" s="105" t="n"/>
     </row>
     <row r="102" ht="14.25" customHeight="1" s="137">
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
       <c r="B102" s="104" t="n"/>
-      <c r="C102" s="88" t="n"/>
+      <c r="C102" s="86" t="n"/>
       <c r="F102" s="88" t="n"/>
       <c r="I102" s="105" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1" s="137">
-      <c r="A103" s="119" t="inlineStr">
+      <c r="B103" s="104" t="n"/>
+      <c r="C103" s="88" t="n"/>
+      <c r="F103" s="88" t="n"/>
+      <c r="I103" s="105" t="n"/>
+    </row>
+    <row r="104" ht="14.25" customHeight="1" s="137">
+      <c r="A104" s="119" t="inlineStr">
         <is>
           <t>Office/Business Inventory</t>
         </is>
       </c>
-      <c r="B103" s="120" t="n"/>
-      <c r="C103" s="100" t="n"/>
-      <c r="D103" s="99" t="n"/>
-      <c r="E103" s="99" t="n"/>
-      <c r="F103" s="100" t="n"/>
-      <c r="G103" s="99" t="n"/>
-      <c r="H103" s="99" t="n"/>
-      <c r="I103" s="121" t="n"/>
-      <c r="J103" s="99" t="n"/>
-      <c r="K103" s="99" t="n"/>
-      <c r="L103" s="99" t="n"/>
-      <c r="M103" s="99" t="n"/>
-      <c r="N103" s="99" t="n"/>
-      <c r="O103" s="99" t="n"/>
-      <c r="P103" s="99" t="n"/>
-      <c r="Q103" s="99" t="n"/>
-      <c r="R103" s="99" t="n"/>
-      <c r="S103" s="99" t="n"/>
-      <c r="T103" s="99" t="n"/>
-      <c r="U103" s="99" t="n"/>
-      <c r="V103" s="99" t="n"/>
-      <c r="W103" s="99" t="n"/>
-      <c r="X103" s="99" t="n"/>
-      <c r="Y103" s="99" t="n"/>
-      <c r="Z103" s="99" t="n"/>
-    </row>
-    <row r="104" ht="14.25" customHeight="1" s="137">
-      <c r="A104" s="122" t="inlineStr">
-        <is>
-          <t>Sofa</t>
-        </is>
-      </c>
-      <c r="B104" s="104" t="n"/>
-      <c r="C104" s="88" t="n"/>
-      <c r="F104" s="88" t="n"/>
-      <c r="I104" s="105" t="n"/>
+      <c r="B104" s="120" t="n"/>
+      <c r="C104" s="100" t="n"/>
+      <c r="D104" s="99" t="n"/>
+      <c r="E104" s="99" t="n"/>
+      <c r="F104" s="100" t="n"/>
+      <c r="G104" s="99" t="n"/>
+      <c r="H104" s="99" t="n"/>
+      <c r="I104" s="121" t="n"/>
+      <c r="J104" s="99" t="n"/>
+      <c r="K104" s="99" t="n"/>
+      <c r="L104" s="99" t="n"/>
+      <c r="M104" s="99" t="n"/>
+      <c r="N104" s="99" t="n"/>
+      <c r="O104" s="99" t="n"/>
+      <c r="P104" s="99" t="n"/>
+      <c r="Q104" s="99" t="n"/>
+      <c r="R104" s="99" t="n"/>
+      <c r="S104" s="99" t="n"/>
+      <c r="T104" s="99" t="n"/>
+      <c r="U104" s="99" t="n"/>
+      <c r="V104" s="99" t="n"/>
+      <c r="W104" s="99" t="n"/>
+      <c r="X104" s="99" t="n"/>
+      <c r="Y104" s="99" t="n"/>
+      <c r="Z104" s="99" t="n"/>
     </row>
     <row r="105" ht="14.25" customHeight="1" s="137">
       <c r="A105" s="122" t="inlineStr">
         <is>
-          <t>Space Heater</t>
+          <t>Sofa</t>
         </is>
       </c>
       <c r="B105" s="104" t="n"/>
@@ -35277,7 +35290,7 @@
     <row r="106" ht="14.25" customHeight="1" s="137">
       <c r="A106" s="122" t="inlineStr">
         <is>
-          <t>Shelving</t>
+          <t>Space Heater</t>
         </is>
       </c>
       <c r="B106" s="104" t="n"/>
@@ -35288,7 +35301,7 @@
     <row r="107" ht="14.25" customHeight="1" s="137">
       <c r="A107" s="122" t="inlineStr">
         <is>
-          <t>Storage Bins</t>
+          <t>Shelving</t>
         </is>
       </c>
       <c r="B107" s="104" t="n"/>
@@ -35299,7 +35312,7 @@
     <row r="108" ht="14.25" customHeight="1" s="137">
       <c r="A108" s="122" t="inlineStr">
         <is>
-          <t>Table</t>
+          <t>Storage Bins</t>
         </is>
       </c>
       <c r="B108" s="104" t="n"/>
@@ -35310,7 +35323,7 @@
     <row r="109" ht="14.25" customHeight="1" s="137">
       <c r="A109" s="122" t="inlineStr">
         <is>
-          <t>Computer</t>
+          <t>Table</t>
         </is>
       </c>
       <c r="B109" s="104" t="n"/>
@@ -35321,7 +35334,7 @@
     <row r="110" ht="14.25" customHeight="1" s="137">
       <c r="A110" s="122" t="inlineStr">
         <is>
-          <t>Art Library</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="B110" s="104" t="n"/>
@@ -35332,7 +35345,7 @@
     <row r="111" ht="14.25" customHeight="1" s="137">
       <c r="A111" s="122" t="inlineStr">
         <is>
-          <t>Standing Desk</t>
+          <t>Art Library</t>
         </is>
       </c>
       <c r="B111" s="104" t="n"/>
@@ -35341,46 +35354,37 @@
       <c r="I111" s="105" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1" s="137">
+      <c r="A112" s="122" t="inlineStr">
+        <is>
+          <t>Standing Desk</t>
+        </is>
+      </c>
       <c r="B112" s="104" t="n"/>
       <c r="C112" s="88" t="n"/>
       <c r="F112" s="88" t="n"/>
       <c r="I112" s="105" t="n"/>
     </row>
     <row r="113" ht="14.25" customHeight="1" s="137">
-      <c r="A113" s="156" t="inlineStr">
-        <is>
-          <t>2025 CC inventory (not in Cost total until object is named)</t>
-        </is>
-      </c>
       <c r="B113" s="104" t="n"/>
       <c r="C113" s="88" t="n"/>
       <c r="F113" s="88" t="n"/>
       <c r="I113" s="105" t="n"/>
     </row>
     <row r="114" ht="14.25" customHeight="1" s="137">
-      <c r="A114" s="0" t="inlineStr">
-        <is>
-          <t>Los Angeles Modern Auctions (inventory purchase)</t>
-        </is>
-      </c>
-      <c r="B114" s="0" t="inlineStr">
-        <is>
-          <t>Sapphire 5423</t>
-        </is>
-      </c>
-      <c r="C114" s="157" t="n">
-        <v>6821.06</v>
-      </c>
-      <c r="D114" s="0" t="inlineStr">
-        <is>
-          <t>2025-07-24</t>
-        </is>
-      </c>
+      <c r="A114" s="156" t="inlineStr">
+        <is>
+          <t>2025 CC inventory (not in Cost total until object is named)</t>
+        </is>
+      </c>
+      <c r="B114" s="104" t="n"/>
+      <c r="C114" s="88" t="n"/>
+      <c r="F114" s="88" t="n"/>
+      <c r="I114" s="105" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1" s="137">
       <c r="A115" s="0" t="inlineStr">
         <is>
-          <t>Hindman LLC (inventory purchase)</t>
+          <t>Los Angeles Modern Auctions (inventory purchase)</t>
         </is>
       </c>
       <c r="B115" s="0" t="inlineStr">
@@ -35389,11 +35393,11 @@
         </is>
       </c>
       <c r="C115" s="157" t="n">
-        <v>282.24</v>
+        <v>6821.06</v>
       </c>
       <c r="D115" s="0" t="inlineStr">
         <is>
-          <t>2025-04-03</t>
+          <t>2025-07-24</t>
         </is>
       </c>
     </row>
@@ -35409,95 +35413,90 @@
         </is>
       </c>
       <c r="C116" s="157" t="n">
-        <v>403.51</v>
+        <v>282.24</v>
       </c>
       <c r="D116" s="0" t="inlineStr">
         <is>
-          <t>2025-07-29</t>
+          <t>2025-04-03</t>
         </is>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1" s="137">
       <c r="A117" s="0" t="inlineStr">
         <is>
+          <t>Hindman LLC (inventory purchase)</t>
+        </is>
+      </c>
+      <c r="B117" s="0" t="inlineStr">
+        <is>
+          <t>Sapphire 5423</t>
+        </is>
+      </c>
+      <c r="C117" s="157" t="n">
+        <v>403.51</v>
+      </c>
+      <c r="D117" s="0" t="inlineStr">
+        <is>
+          <t>2025-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="14.25" customHeight="1" s="137">
+      <c r="A118" s="0" t="inlineStr">
+        <is>
           <t>The Great Frame Up (inventory framing)</t>
         </is>
       </c>
-      <c r="B117" s="0" t="inlineStr">
+      <c r="B118" s="0" t="inlineStr">
         <is>
           <t>Sapphire 5423</t>
         </is>
       </c>
-      <c r="C117" s="157" t="n">
+      <c r="C118" s="157" t="n">
         <v>536.41</v>
       </c>
-      <c r="D117" s="0" t="inlineStr">
+      <c r="D118" s="0" t="inlineStr">
         <is>
           <t>2025-02-16</t>
         </is>
       </c>
     </row>
-    <row r="118" ht="14.25" customHeight="1" s="137"/>
-    <row r="119" ht="14.25" customHeight="1" s="137">
-      <c r="A119" s="201" t="inlineStr">
+    <row r="119" ht="14.25" customHeight="1" s="137"/>
+    <row r="120" ht="14.25" customHeight="1" s="137">
+      <c r="A120" s="201" t="inlineStr">
         <is>
           <t>2025 Mercury 8291 — David Aaron Limited is LOCKED consultant fee (not Art Sales)</t>
         </is>
       </c>
     </row>
-    <row r="120" ht="14.25" customHeight="1" s="137">
-      <c r="A120" s="181" t="inlineStr">
+    <row r="121" ht="14.25" customHeight="1" s="137">
+      <c r="A121" s="181" t="inlineStr">
         <is>
           <t>NOT a 2025 art sale — David Aaron Limited consultant fee (EPGC Consultant June)</t>
         </is>
       </c>
-      <c r="B120" s="181" t="inlineStr">
+      <c r="B121" s="181" t="inlineStr">
         <is>
           <t>David Aaron Limited</t>
         </is>
       </c>
-      <c r="C120" s="181" t="n"/>
-      <c r="D120" s="181" t="n"/>
-      <c r="E120" s="181" t="n"/>
-      <c r="F120" s="183" t="n"/>
-      <c r="G120" s="206" t="n"/>
-      <c r="H120" s="206" t="n"/>
-      <c r="I120" s="181" t="inlineStr">
+      <c r="C121" s="181" t="n"/>
+      <c r="D121" s="181" t="n"/>
+      <c r="E121" s="181" t="n"/>
+      <c r="F121" s="183" t="n"/>
+      <c r="G121" s="206" t="n"/>
+      <c r="H121" s="206" t="n"/>
+      <c r="I121" s="181" t="inlineStr">
         <is>
           <t>LOCKED 2026-09-20: consultant fee, not a sale. $13,595 is on EPGC Consultant June. Not tax advice.</t>
         </is>
       </c>
     </row>
-    <row r="121" ht="14.25" customHeight="1" s="137"/>
-    <row r="122" ht="14.25" customHeight="1" s="137">
-      <c r="A122" s="201" t="inlineStr">
+    <row r="122" ht="14.25" customHeight="1" s="137"/>
+    <row r="123" ht="14.25" customHeight="1" s="137">
+      <c r="A123" s="201" t="inlineStr">
         <is>
           <t>2025 Mercury COGS — Newstar Jewelers (LOCKED jewelry fabrication)</t>
-        </is>
-      </c>
-    </row>
-    <row r="123" ht="14.25" customHeight="1" s="137">
-      <c r="A123" s="202" t="inlineStr">
-        <is>
-          <t>Newstar Jewelers — jewelry from intaglios / engraved gems / scarabs</t>
-        </is>
-      </c>
-      <c r="B123" s="202" t="inlineStr">
-        <is>
-          <t>Mercury 8291</t>
-        </is>
-      </c>
-      <c r="C123" s="203" t="n">
-        <v>8000</v>
-      </c>
-      <c r="D123" s="202" t="inlineStr">
-        <is>
-          <t>2025-10-14</t>
-        </is>
-      </c>
-      <c r="I123" s="0" t="inlineStr">
-        <is>
-          <t>LOCKED COGS fabrication. Not in sold-lot Cost total (Feb Berk lots already sold). Identify which gems/intaglios/scarabs.</t>
         </is>
       </c>
     </row>
@@ -35517,7 +35516,7 @@
       </c>
       <c r="D124" s="202" t="inlineStr">
         <is>
-          <t>2025-11-12</t>
+          <t>2025-10-14</t>
         </is>
       </c>
       <c r="I124" s="0" t="inlineStr">
@@ -35529,69 +35528,69 @@
     <row r="125" ht="14.25" customHeight="1" s="137">
       <c r="A125" s="202" t="inlineStr">
         <is>
+          <t>Newstar Jewelers — jewelry from intaglios / engraved gems / scarabs</t>
+        </is>
+      </c>
+      <c r="B125" s="202" t="inlineStr">
+        <is>
+          <t>Mercury 8291</t>
+        </is>
+      </c>
+      <c r="C125" s="203" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D125" s="202" t="inlineStr">
+        <is>
+          <t>2025-11-12</t>
+        </is>
+      </c>
+      <c r="I125" s="0" t="inlineStr">
+        <is>
+          <t>LOCKED COGS fabrication. Not in sold-lot Cost total (Feb Berk lots already sold). Identify which gems/intaglios/scarabs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="14.25" customHeight="1" s="137">
+      <c r="A126" s="202" t="inlineStr">
+        <is>
           <t>Newstar Jewelers — jewelry from intaglios / engraved gems / scarabs (3 of 3)</t>
         </is>
       </c>
-      <c r="B125" s="202" t="inlineStr">
+      <c r="B126" s="202" t="inlineStr">
         <is>
           <t>Mercury 8291</t>
         </is>
       </c>
-      <c r="C125" s="203" t="n">
+      <c r="C126" s="203" t="n">
         <v>7581</v>
       </c>
-      <c r="D125" s="202" t="inlineStr">
+      <c r="D126" s="202" t="inlineStr">
         <is>
           <t>2025-12-24</t>
         </is>
       </c>
-      <c r="I125" s="0" t="inlineStr">
+      <c r="I126" s="0" t="inlineStr">
         <is>
           <t>LOCKED COGS fabrication. Not in sold-lot Cost total (Feb Berk lots already sold). Identify which gems/intaglios/scarabs.</t>
         </is>
       </c>
     </row>
-    <row r="126" ht="14.25" customHeight="1" s="137">
-      <c r="A126" s="0" t="inlineStr">
+    <row r="127" ht="14.25" customHeight="1" s="137">
+      <c r="A127" s="0" t="inlineStr">
         <is>
           <t>Newstar 2025 total</t>
         </is>
       </c>
-      <c r="C126" s="203">
+      <c r="C127" s="203">
         <f>SUM(C123:C125)</f>
         <v/>
       </c>
     </row>
-    <row r="127" ht="14.25" customHeight="1" s="137"/>
-    <row r="128" ht="14.25" customHeight="1" s="137">
-      <c r="A128" s="204" t="inlineStr">
+    <row r="128" ht="14.25" customHeight="1" s="137"/>
+    <row r="129" ht="14.25" customHeight="1" s="137">
+      <c r="A129" s="204" t="inlineStr">
         <is>
           <t>2025 Mercury ASK — Fortuna inventory remaining (not in Cost total until object is named)</t>
-        </is>
-      </c>
-    </row>
-    <row r="129" ht="14.25" customHeight="1" s="137">
-      <c r="A129" s="200" t="inlineStr">
-        <is>
-          <t>Fortuna / Erdal Dere — object TBD</t>
-        </is>
-      </c>
-      <c r="B129" s="200" t="inlineStr">
-        <is>
-          <t>Mercury 8291</t>
-        </is>
-      </c>
-      <c r="C129" s="157" t="n">
-        <v>20000</v>
-      </c>
-      <c r="D129" s="200" t="inlineStr">
-        <is>
-          <t>2025-05-09</t>
-        </is>
-      </c>
-      <c r="I129" s="0" t="inlineStr">
-        <is>
-          <t>ASK: inventory purchase vs other. Do not add to sold Cost until named (avoid double count).</t>
         </is>
       </c>
     </row>
@@ -35607,11 +35606,11 @@
         </is>
       </c>
       <c r="C130" s="157" t="n">
-        <v>45000</v>
+        <v>20000</v>
       </c>
       <c r="D130" s="200" t="inlineStr">
         <is>
-          <t>2025-07-21</t>
+          <t>2025-05-09</t>
         </is>
       </c>
       <c r="I130" s="0" t="inlineStr">
@@ -35632,71 +35631,56 @@
         </is>
       </c>
       <c r="C131" s="157" t="n">
+        <v>45000</v>
+      </c>
+      <c r="D131" s="200" t="inlineStr">
+        <is>
+          <t>2025-07-21</t>
+        </is>
+      </c>
+      <c r="I131" s="0" t="inlineStr">
+        <is>
+          <t>ASK: inventory purchase vs other. Do not add to sold Cost until named (avoid double count).</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="14.25" customHeight="1" s="137">
+      <c r="A132" s="200" t="inlineStr">
+        <is>
+          <t>Fortuna / Erdal Dere — object TBD</t>
+        </is>
+      </c>
+      <c r="B132" s="200" t="inlineStr">
+        <is>
+          <t>Mercury 8291</t>
+        </is>
+      </c>
+      <c r="C132" s="157" t="n">
         <v>20000</v>
       </c>
-      <c r="D131" s="200" t="inlineStr">
+      <c r="D132" s="200" t="inlineStr">
         <is>
           <t>2025-08-15</t>
         </is>
       </c>
-      <c r="I131" s="0" t="inlineStr">
+      <c r="I132" s="0" t="inlineStr">
         <is>
           <t>ASK: inventory purchase vs other. Do not add to sold Cost until named (avoid double count).</t>
         </is>
       </c>
     </row>
-    <row r="132" ht="14.25" customHeight="1" s="137">
-      <c r="A132" s="0" t="inlineStr">
+    <row r="133" ht="14.25" customHeight="1" s="137">
+      <c r="A133" s="0" t="inlineStr">
         <is>
           <t>Fortuna remaining 2025 (excl. seals $13,000 already on row 73)</t>
         </is>
       </c>
-      <c r="C132" s="157" t="n">
+      <c r="C133" s="157" t="n">
         <v>85000</v>
       </c>
     </row>
-    <row r="133" ht="14.25" customHeight="1" s="137"/>
-    <row r="134" ht="14.25" customHeight="1" s="137">
-      <c r="A134" s="201" t="inlineStr">
-        <is>
-          <t>2025 Mercury 8291 — Books sold to Aquinas Hobor (LOCKED)</t>
-        </is>
-      </c>
-    </row>
-    <row r="135" ht="14.25" customHeight="1" s="137">
-      <c r="A135" s="181" t="inlineStr">
-        <is>
-          <t>Books sold to Aquinas Hobor (titles TBD)</t>
-        </is>
-      </c>
-      <c r="B135" s="181" t="inlineStr">
-        <is>
-          <t>Aquinas Hobor</t>
-        </is>
-      </c>
-      <c r="C135" s="181" t="n"/>
-      <c r="D135" s="181" t="n"/>
-      <c r="E135" s="181" t="inlineStr">
-        <is>
-          <t>Aquinas Hobor</t>
-        </is>
-      </c>
-      <c r="F135" s="183" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G135" s="209" t="n">
-        <v>45692</v>
-      </c>
-      <c r="H135" s="181">
-        <f>IF(C135="","",F135-C135)</f>
-        <v/>
-      </c>
-      <c r="I135" s="181" t="inlineStr">
-        <is>
-          <t>LOCKED 2026-09-20: books sold to Aquinas. $1,000 cash on EPGC Art Sales February. Cost / titles TBD — not in Income I8 until Cost. Distinct from 2022 Saharan bracelets. Not tax advice.</t>
-        </is>
-      </c>
-    </row>
+    <row r="134" ht="14.25" customHeight="1" s="137"/>
+    <row r="135" ht="14.25" customHeight="1" s="137"/>
     <row r="136" ht="14.25" customHeight="1" s="137"/>
     <row r="137" ht="14.25" customHeight="1" s="137"/>
     <row r="138" ht="14.25" customHeight="1" s="137"/>

</xml_diff>

<commit_message>
Confirm EOEB and L5 mixed sales plus advisory, keep remainder off P&L.
Pattern is locked. Invoice-level split stays ASK. Consultant June $13,595 and Art Sales $150,000 are unchanged.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
+++ b/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
@@ -648,7 +648,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="211">
+  <cellXfs count="213">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1088,6 +1088,12 @@
     </xf>
     <xf numFmtId="170" fontId="24" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -13867,7 +13873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" style="137" min="1" max="1"/>
@@ -13878,7 +13884,7 @@
     <row r="1">
       <c r="A1" s="156" t="inlineStr">
         <is>
-          <t>ASK — remaining Mercury 8291 questions. Q6 consultant, Q7 Wise expertise, Q8 pass-through, Q9 Aquinas books LOCKED (green). Q1/Q2 mixed pattern CONFIRMED, dollars unallocated (yellow). Not tax advice.</t>
+          <t>ASK — remaining Mercury 8291 questions. Q6 consultant, Q7 Wise expertise, Q8 pass-through, Q9 Aquinas books LOCKED (green). Q1/Q2 mixed pattern CONFIRMED (blue) — remainder dollars unallocated until invoice split. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -13895,26 +13901,26 @@
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" s="137">
-      <c r="A4" s="189" t="inlineStr">
+      <c r="A4" s="211" t="inlineStr">
         <is>
           <t>1. EOEB LLC remainder after mosaics — MIXED PATTERN CONFIRMED, dollars unallocated</t>
         </is>
       </c>
-      <c r="B4" s="190" t="inlineStr">
-        <is>
-          <t>$130,270.00 of EOEB IN is not mosaics $105,000 and not Wise reimburse $565.75. User 2026-09-20: EOEB is mixed art sales AND advisory/consultant fees. Do NOT dump this remainder onto Consultant or Art Sales. Invoice-level split still ASK. Jan 16 $1,000 Canosan-horse question STILL OPEN (Art Sales horse is to Erdal; this cash is EOEB).</t>
+      <c r="B4" s="212" t="inlineStr">
+        <is>
+          <t>$130,270.00 of EOEB IN is not mosaics $105,000 and not Wise reimburse $565.75. User 2026-09-20: EOEB is mixed art sales AND advisory/consultant fees. Do NOT dump this remainder onto Consultant or Art Sales. Mark each invoice sale vs advisory: 1/16 $1,000 (Canosan-horse STILL OPEN — Art Sales horse is to Erdal, this cash is EOEB); 3/10 $14,000; 5/1 $21,000; 5/13 $16,200; 6/12 $25,000 + $3,300; 7/8 $2,000; 8/29 $10,000; 9/19 $5,000; 9/25 $3,100; 10/1 $10,000; 10/15 $16,000; 10/24 $1,500; 10/31 $2,170.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" s="137">
-      <c r="A5" s="189" t="inlineStr">
+      <c r="A5" s="211" t="inlineStr">
         <is>
           <t>2. L5 (all seven invoices) — MIXED PATTERN CONFIRMED, dollars unallocated</t>
         </is>
       </c>
-      <c r="B5" s="190" t="inlineStr">
-        <is>
-          <t>$87,396.32. User 2026-09-20: L5 is mixed art sales AND advisory/consultant fees. Do NOT dump onto Consultant or Art Sales. Invoice-level split still ASK. The 7/15 $50,000 still sits in the Aysel $50k / Fortuna $45k week.</t>
+      <c r="B5" s="212" t="inlineStr">
+        <is>
+          <t>$87,396.32. User 2026-09-20: L5 is mixed art sales AND advisory/consultant fees. Do NOT dump onto Consultant or Art Sales. Mark each invoice sale vs advisory: 7/11 $8,534.79; 7/15 $50,000 + $2,500 (same week as Aysel $50k / Fortuna $45k); 9/2 $5,042; 9/23 $9,119.27; 10/21 $7,500; 12/4 $4,700.26.</t>
         </is>
       </c>
     </row>
@@ -14150,6 +14156,18 @@
       <c r="B26" s="181" t="inlineStr">
         <is>
           <t>$1,000 IN 2/4 LOCKED book sale → EPGC Art Sales February +$1,000 (Feb $136,000; matched cash $150,000). Cost / titles TBD (not in I8 until Cost, same as Sale 6428).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="181" t="inlineStr">
+        <is>
+          <t>EOEB / L5 mixed pattern</t>
+        </is>
+      </c>
+      <c r="B27" s="181" t="inlineStr">
+        <is>
+          <t>CONFIRMED mixed art sales AND advisory/consultant. Remainder $130,270 / $87,396.32 unallocated — not on P&amp;L until invoice split. Jan 16 $1,000 Canosan-horse still open.</t>
         </is>
       </c>
     </row>
@@ -34793,16 +34811,20 @@
       </c>
     </row>
     <row r="78" ht="48" customHeight="1" s="137">
-      <c r="A78" s="210" t="inlineStr">
-        <is>
-          <t>Mercury 8291 MATCHED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics). Fortuna $13,000 (1/8 seals Cost). Plutus $50,000 of mosaics $90,000 Cost — $40,000 of Cost not on 8291 (ASK). Newstar $23,581 is jewelry fabrication COGS, parked below — not in sold-lot Cost (Berk gem/scarab lots already sold in February). David Aaron $13,595 (6/24) is LOCKED consultant fee — not a sale (EPGC Consultant June). Aquinas Hobor $1,000 (2/4) is LOCKED books sold — EPGC Art Sales February; Cost TBD (not in I8). Not tax advice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="14.25" customHeight="1" s="137">
-      <c r="A79" s="199" t="inlineStr">
-        <is>
-          <t>Mercury 8291 MATCHED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics). Fortuna $13,000 (1/8 seals Cost). Plutus $50,000 of mosaics $90,000 Cost — $40,000 of Cost not on 8291 (ASK). Newstar $23,581 is jewelry fabrication COGS, parked below — not in sold-lot Cost (Berk gem/scarab lots already sold in February). David Aaron $13,595 (6/24) is LOCKED consultant fee — not a sale (EPGC Consultant June). Aquinas Hobor $1,000 (2/4) is LOCKED books sold — EPGC Art Sales February; Cost TBD (not in I8). Not tax advice.</t>
+      <c r="A78" s="178" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H78" s="138">
+        <f>SUM(H51:H75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79" ht="48" customHeight="1" s="137">
+      <c r="A79" s="210" t="inlineStr">
+        <is>
+          <t>Mercury 8291 MATCHED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics). Fortuna $13,000 (1/8 seals Cost). Plutus $50,000 of mosaics $90,000 Cost — $40,000 of Cost not on 8291 (ASK). Newstar $23,581 is jewelry fabrication COGS, parked below — not in sold-lot Cost (Berk gem/scarab lots already sold in February). David Aaron $13,595 (6/24) is LOCKED consultant fee — not a sale (EPGC Consultant June). Aquinas Hobor $1,000 (2/4) is LOCKED book sale — EPGC Art Sales February; Cost TBD (not in I8). Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -36549,8 +36571,8 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A134:I134"/>
-    <mergeCell ref="A78:I78"/>
     <mergeCell ref="A119:I119"/>
+    <mergeCell ref="A79:I79"/>
     <mergeCell ref="A122:I122"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>

<commit_message>
Lock Travelers as 524 home insurance and Geico as personal auto.
User 2026-09-20: Travelers was home for Ferdinand; Geico was the cars.
ASK no longer asks carrier identity. 524 INSURANCE dollars unchanged
(State Farm home share only; Geico credit personal; Jan Travelers leftover $0).

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
+++ b/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
@@ -648,7 +648,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="213">
+  <cellXfs count="214">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1095,6 +1095,9 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7964,10 +7967,10 @@
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1" s="137"/>
-    <row r="45" ht="14.25" customHeight="1" s="137">
-      <c r="A45" s="0" t="inlineStr">
-        <is>
-          <t>2025 columns P–AB. Residence through sale 2025-12-18. MORTGAGE = US Bank loan 09422 monthly P+I from joint 0203 (not $50k extra principal on 9922 Jul/Sep — those are not on this row). HOA n/a. Not tax advice.</t>
+    <row r="45" ht="72" customHeight="1" s="137">
+      <c r="A45" s="213" t="inlineStr">
+        <is>
+          <t>2025 columns P–AB. Residence through sale 2025-12-18. MORTGAGE = US Bank loan 09422 monthly P+I from joint 0203 (not $50k extra principal on 9922 Jul/Sep — those are not on this row). HOA n/a. INSURANCE LOCK 2026-09-20: Travelers was prior 524 home; Geico was the cars. Only State Farm HOME share on this INSURANCE line (50/50 with Unit 2). Travelers leftover Jan is 524 home ($0 on cards/Monarch). Auto + Geico credit personal — not EPGC. Not tax advice.</t>
         </is>
       </c>
       <c r="B45" s="122" t="inlineStr">
@@ -18559,10 +18562,10 @@
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1" s="137"/>
-    <row r="39" ht="14.25" customHeight="1" s="137">
-      <c r="A39" s="0" t="inlineStr">
-        <is>
-          <t>2025: platform STR net on RENTAL INCOME (Jun–Nov). TruGreen/Alsip on YARD SERVICE (same as 2024). Grove Collaborative on SUPPLIES. State Farm HOME share only on INSURANCE. ELECTRIC yellow — confirm ComEd with Megan. Not tax advice.</t>
+    <row r="39" ht="72" customHeight="1" s="137">
+      <c r="A39" s="213" t="inlineStr">
+        <is>
+          <t>2025: platform STR net on RENTAL INCOME (Jun–Nov). TruGreen/Alsip on YARD SERVICE (same as 2024). Grove Collaborative on SUPPLIES (≠ 827 N Grove the house). INSURANCE LOCK 2026-09-20: Travelers was prior 524 home; Geico was the cars. Only State Farm HOME share on this INSURANCE line (50/50 U1/U2). Auto + Geico $540.89 credit personal, not EPGC. Travelers leftover Jan 2025 is 524 home ($0 on cards/Monarch). ELECTRIC yellow — confirm ComEd with Megan. Not tax advice.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Point Drive packet at Travelers/Geico 524 insurance lock.
Live ASK/SF_SPLIT/524 Unit sheets and START HERE now lock Travelers as
prior Ferdinand home and Geico as personal auto. Stale CC ASK copies
moved to _SUPERSEDED. Mercury live IDs unchanged.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
+++ b/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
@@ -648,7 +648,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="214">
+  <cellXfs count="216">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1097,6 +1097,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="28" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -21123,7 +21129,7 @@
       <c r="AK14" s="68" t="n">
         <v>0</v>
       </c>
-      <c r="AL14" s="147" t="n">
+      <c r="AL14" s="214" t="n">
         <v>514</v>
       </c>
       <c r="AM14" s="59" t="n">
@@ -25008,10 +25014,10 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="14.25" customHeight="1" s="137">
-      <c r="B64" s="150" t="inlineStr">
-        <is>
-          <t>Insurance — Lemonade $514 cash 10/3 on Megan Chase (yellow: confirm 216 policy). 2024 was $35.08/mo renter's.</t>
+    <row r="64" ht="64" customHeight="1" s="137">
+      <c r="B64" s="215" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-09-20: 216 LTR insurance = Lemonade $514.00 cash 10/3 on Megan Chase (1702). Same annual Oct 3 Lemonade as 2023 $321 (= Excel $26.75/mo renter's) and 2024 $421 (≈ Excel $35.08/mo renter's). 2025 books cash in October (not amortized). Travelers = prior 524 Ferdinand home (not 216). Geico = cars. State Farm 2025 bundle = Ferdinand car+home — only home share on 524, not 216. No other Oak Park policy cash on Prime/Sapphire/BoA/0203/8507/Monarch. Not tax advice.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Point Drive packet at native Mercury CSV ingest and Fortuna locks.
ASK/START HERE/lock now cover 0 new unique 8291 Sent cash vs the 64,
Venus $20k + Roman Gold Belt $45k parked inventory, and the Aysel
Monarch IN vs native Failed OUT question. Prior Q6–Q9 copies moved
to _SUPERSEDED. EPGC MATCHED P&L IDs unchanged.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
+++ b/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
@@ -9960,7 +9960,7 @@
     <row r="1" ht="48" customHeight="1" s="137">
       <c r="A1" s="176" t="inlineStr">
         <is>
-          <t>Mercury Checking 8291 — EPGC LLC (Choice Financial) 2025. 64 unique cash transactions. Coinbase ACH = investment. Newstar = jewelry COGS on intaglios/gems/scarabs. BoA 9922 draws and Koziol/Ariadne $150k are LOCKED not-P&amp;L (pass-through / owner transfer). David Aaron $13,595 is LOCKED EPGC Consultant (June). Wise $334.17 + $658.63 are LOCKED EPGC Consultant Fees (expertise write-ups). Aquinas Hobor $1,000 (2/4) is LOCKED books sold (EPGC Art Sales February; Cost TBD). Not tax advice.</t>
+          <t>Mercury Checking 8291 — EPGC LLC (Choice Financial) 2025. 64 unique cash transactions (Monarch IDs). Native Mercury CSV 2026-09-20 is the same 8291 year — 0 new unique Sent cash. Coinbase ACH = investment. Newstar = jewelry COGS on intaglios/gems/scarabs. Fortuna Venus $20k (5/9) + Roman Gold Belt $45k (7/21) LOCKED inventory (not sold Cost). BoA 9922 draws and Koziol/Ariadne $150k are LOCKED not-P&amp;L (pass-through / owner transfer). David Aaron $13,595 is LOCKED EPGC Consultant (June). Wise $334.17 + $658.63 are LOCKED EPGC Consultant Fees (expertise write-ups). Aquinas Hobor $1,000 (2/4) is LOCKED books sold (EPGC Art Sales February; Cost TBD). Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -10077,12 +10077,12 @@
       </c>
       <c r="K4" s="178" t="inlineStr">
         <is>
-          <t>Merchant name: Erdal Dere (Fortuna)</t>
+          <t>Merchant name: Erdal Dere (Fortuna); Mercury native: J.K. New York Collection | Send Money transaction initiated on Mercury</t>
         </is>
       </c>
       <c r="L4" s="182" t="inlineStr">
         <is>
-          <t>Fortuna / Erdal Dere. Matches Art Sales Cost $13,000; Berk sold it 1/10 for $14,000.</t>
+          <t>Fortuna / Erdal Dere. Mercury native note: J.K. New York Collection. Matches Art Sales Cost $13,000; Berk sold it 1/10 for $14,000. Same-day Cancelled ACH to Erdal Dere (closed) is not cash.</t>
         </is>
       </c>
     </row>
@@ -10437,7 +10437,7 @@
       </c>
       <c r="K10" s="178" t="inlineStr">
         <is>
-          <t>Merchant name: Jamal M Rifai</t>
+          <t>Merchant name: Jamal M Rifai; Mercury native: via mercury.com | Send Money transaction initiated on Mercury</t>
         </is>
       </c>
       <c r="L10" s="182" t="inlineStr">
@@ -10677,7 +10677,7 @@
       </c>
       <c r="K14" s="178" t="inlineStr">
         <is>
-          <t>Merchant name: Jamal M Rifai</t>
+          <t>Merchant name: Jamal M Rifai; Mercury native: From EPGC LLC via mercury.com | Send Money transaction initiated on Mercury</t>
         </is>
       </c>
       <c r="L14" s="182" t="inlineStr">
@@ -10737,7 +10737,7 @@
       </c>
       <c r="K15" s="178" t="inlineStr">
         <is>
-          <t>Merchant name: Plutus &amp; Mnemosyne, LLC</t>
+          <t>Merchant name: Plutus &amp; Mnemosyne, LLC; Mercury native: via mercury.com | Send Money transaction initiated on Mercury</t>
         </is>
       </c>
       <c r="L15" s="182" t="inlineStr">
@@ -10857,7 +10857,7 @@
       </c>
       <c r="K17" s="178" t="inlineStr">
         <is>
-          <t>Merchant name: Plutus &amp; Mnemosyne, LLC</t>
+          <t>Merchant name: Plutus &amp; Mnemosyne, LLC; Mercury native: From EPGC LLC via mercury.com | Send Money transaction initiated on Mercury</t>
         </is>
       </c>
       <c r="L17" s="182" t="inlineStr">
@@ -10997,7 +10997,7 @@
           <t>Erdal Dere (Fortuna)</t>
         </is>
       </c>
-      <c r="C20" s="139" t="n">
+      <c r="C20" s="179" t="n">
         <v>-20000</v>
       </c>
       <c r="D20" s="178" t="inlineStr">
@@ -11010,14 +11010,14 @@
           <t>ART_PURCHASE</t>
         </is>
       </c>
-      <c r="F20" s="185" t="inlineStr">
-        <is>
-          <t>ASK</t>
+      <c r="F20" s="181" t="inlineStr">
+        <is>
+          <t>LOCKED</t>
         </is>
       </c>
       <c r="G20" s="178" t="inlineStr">
         <is>
-          <t>Fortuna / Erdal — inventory vs other</t>
+          <t>Bronze head of a goddess, likely Venus — inventory Cost</t>
         </is>
       </c>
       <c r="H20" s="178" t="inlineStr">
@@ -11037,12 +11037,12 @@
       </c>
       <c r="K20" s="178" t="inlineStr">
         <is>
-          <t>Merchant name: Erdal Dere (Fortuna)</t>
+          <t>Merchant name: Erdal Dere (Fortuna); Mercury native: For bronze head of a goddess, likely Venus | Send Money transaction initiated on Mercury</t>
         </is>
       </c>
       <c r="L20" s="182" t="inlineStr">
         <is>
-          <t>After seals $13,000. Object name? Inventory purchase (COGS when sold) or something else?</t>
+          <t>Mercury native 2025 CSV note: 'For bronze head of a goddess, likely Venus'. Inventory purchase from Fortuna / Erdal. Not sold on 2025 Art Sales — parked Cost, not in sold-lot Cost (avoid double count). Not dumped onto Consultant or Art Sales P&amp;L.</t>
         </is>
       </c>
     </row>
@@ -11677,7 +11677,7 @@
       </c>
       <c r="G31" s="178" t="inlineStr">
         <is>
-          <t>Aysel Dere $50,000 IN</t>
+          <t>Aysel Dere $50,000 IN on Monarch — NOT on Mercury native Sent</t>
         </is>
       </c>
       <c r="H31" s="178" t="inlineStr">
@@ -11702,7 +11702,7 @@
       </c>
       <c r="L31" s="182" t="inlineStr">
         <is>
-          <t>Same week as L5 $50k, Fortuna $45k OUT (7/21), Erdal $26k IN (7/24). Sale, family/related transfer, or inventory reverse?</t>
+          <t>Monarch 7/18 +$50,000 IN. Mercury native 2025 CSV (user upload 2026-09-20) has no Sent Aysel cash. Native has Failed $50,000 OUT 7/17 'Recipient account does not exist'. Keep on ASK — do not dump onto Art Sales or Consultant. Is the Monarch IN a phantom of the failed send?</t>
         </is>
       </c>
     </row>
@@ -11717,7 +11717,7 @@
           <t>Erdal Dere (Fortuna)</t>
         </is>
       </c>
-      <c r="C32" s="139" t="n">
+      <c r="C32" s="179" t="n">
         <v>-45000</v>
       </c>
       <c r="D32" s="178" t="inlineStr">
@@ -11730,14 +11730,14 @@
           <t>ART_PURCHASE</t>
         </is>
       </c>
-      <c r="F32" s="185" t="inlineStr">
-        <is>
-          <t>ASK</t>
+      <c r="F32" s="181" t="inlineStr">
+        <is>
+          <t>LOCKED</t>
         </is>
       </c>
       <c r="G32" s="178" t="inlineStr">
         <is>
-          <t>Fortuna / Erdal — inventory vs other</t>
+          <t>Roman Gold Belt — inventory Cost</t>
         </is>
       </c>
       <c r="H32" s="178" t="inlineStr">
@@ -11757,12 +11757,12 @@
       </c>
       <c r="K32" s="178" t="inlineStr">
         <is>
-          <t>Merchant name: Erdal Dere (Fortuna)</t>
+          <t>Merchant name: Erdal Dere (Fortuna); Mercury native: From EPGC LLC via mercury.com | Roman Gold Belt | Send Money transaction initiated on Mercury</t>
         </is>
       </c>
       <c r="L32" s="182" t="inlineStr">
         <is>
-          <t>Object name? Ties to Aysel $50k / Erdal $26k the same week?</t>
+          <t>Mercury native 2025 CSV note: Roman Gold Belt. Inventory purchase from Fortuna / Erdal. Not sold on 2025 Art Sales — parked Cost, not in sold-lot Cost. Same week as L5 $50k / Monarch Aysel $50k ASK / Erdal $26k IN.</t>
         </is>
       </c>
     </row>
@@ -11917,7 +11917,7 @@
       </c>
       <c r="G35" s="178" t="inlineStr">
         <is>
-          <t>Fortuna / Erdal — inventory vs other</t>
+          <t>Fortuna / Erdal — object still unnamed</t>
         </is>
       </c>
       <c r="H35" s="178" t="inlineStr">
@@ -11937,12 +11937,12 @@
       </c>
       <c r="K35" s="178" t="inlineStr">
         <is>
-          <t>Merchant name: Erdal Dere (Fortuna)</t>
+          <t>Merchant name: Erdal Dere (Fortuna); Mercury native: From EPGC LLC via mercury.com | Send Money transaction initiated on Mercury</t>
         </is>
       </c>
       <c r="L35" s="182" t="inlineStr">
         <is>
-          <t>Object name?</t>
+          <t>Same $20,000 OUT as Mercury native initiated 2025-08-18 / Monarch posted 2025-08-15. No object name in the native memo ('From EPGC LLC via mercury.com'). Inventory vs other? Do not add to sold Cost until named. Not a second unique txn.</t>
         </is>
       </c>
     </row>
@@ -12717,7 +12717,7 @@
       </c>
       <c r="K48" s="178" t="inlineStr">
         <is>
-          <t>Merchant name: Newstar Jewelers</t>
+          <t>Merchant name: Newstar Jewelers; Mercury native: From EPGC LLC via mercury.com | 1 of 3 payments | Send Money transaction initiated on Mercury</t>
         </is>
       </c>
       <c r="L48" s="182" t="inlineStr">
@@ -12897,7 +12897,7 @@
       </c>
       <c r="K51" s="178" t="inlineStr">
         <is>
-          <t>Merchant name: Ariadne Demirjian LLC</t>
+          <t>Merchant name: Ariadne Demirjian LLC; Mercury native: via mercury.com; Vendor: Ariadne Demirjian LLC Roth 401k Account 5386-8600 | Send Money transaction initiated on Mercury</t>
         </is>
       </c>
       <c r="L51" s="182" t="inlineStr">
@@ -13317,7 +13317,7 @@
       </c>
       <c r="K58" s="178" t="inlineStr">
         <is>
-          <t>Merchant name: Newstar Jewelers</t>
+          <t>Merchant name: Newstar Jewelers; Mercury native: From EPGC LLC via mercury.com | Send Money transaction initiated on Mercury</t>
         </is>
       </c>
       <c r="L58" s="182" t="inlineStr">
@@ -13857,7 +13857,7 @@
       </c>
       <c r="K67" s="178" t="inlineStr">
         <is>
-          <t>From EPGC LLC via mercury.com 3 of 3; Merchant name: Newstar Jewelers</t>
+          <t>From EPGC LLC via mercury.com 3 of 3; Merchant name: Newstar Jewelers; Mercury native: From EPGC LLC via mercury.com 3 of 3 | Send Money transaction initiated on Mercury</t>
         </is>
       </c>
       <c r="L67" s="182" t="inlineStr">
@@ -13882,7 +13882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" style="137" min="1" max="1"/>
@@ -13936,12 +13936,12 @@
     <row r="6" ht="48" customHeight="1" s="137">
       <c r="A6" s="189" t="inlineStr">
         <is>
-          <t>3. Fortuna / Erdal Dere OUT after seals</t>
+          <t>3. Fortuna / Erdal $20,000 Aug — object still unnamed</t>
         </is>
       </c>
       <c r="B6" s="190" t="inlineStr">
         <is>
-          <t>$85,000.00 after the 1/8 $13,000 seals COGS (5/9 $20k, 7/21 $45k, 8/15 $20k). Inventory purchases (object names) or something else?</t>
+          <t>$20,000.00. Monarch posted 8/15 = Mercury native initiated 8/18 (same cash, not a second unique txn). Native memo has no object name. Venus $20,000 (5/9) and Roman Gold Belt $45,000 (7/21) are LOCKED inventory below — not this question.</t>
         </is>
       </c>
     </row>
@@ -13960,12 +13960,12 @@
     <row r="8" ht="48" customHeight="1" s="137">
       <c r="A8" s="189" t="inlineStr">
         <is>
-          <t>5. Aysel Dere $50,000 IN (7/18)</t>
+          <t>5. Aysel Dere $50,000 — Monarch IN vs native Failed OUT</t>
         </is>
       </c>
       <c r="B8" s="190" t="inlineStr">
         <is>
-          <t>Sale, related-party transfer, or part of the mid-July Fortuna/L5 cluster?</t>
+          <t>Monarch 7/18 +$50,000 IN is in the 64. Mercury native CSV has NO Sent Aysel cash — only Failed $50,000 OUT 7/17 'Recipient account does not exist'. Is the Monarch IN a phantom of the failed send, or a real incoming the export omitted? Do not dump onto Art Sales or Consultant until confirmed.</t>
         </is>
       </c>
     </row>
@@ -14177,6 +14177,42 @@
       <c r="B27" s="181" t="inlineStr">
         <is>
           <t>CONFIRMED mixed art sales AND advisory/consultant. Remainder $130,270 / $87,396.32 unallocated — not on P&amp;L until invoice split. Jan 16 $1,000 Canosan-horse still open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="181" t="inlineStr">
+        <is>
+          <t>Fortuna Venus inventory</t>
+        </is>
+      </c>
+      <c r="B28" s="181" t="inlineStr">
+        <is>
+          <t>$20,000 OUT 5/9 LOCKED. Mercury native note: bronze head of a goddess, likely Venus. Parked Cost — not sold 2025, not dumped onto Art Sales/Consultant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="181" t="inlineStr">
+        <is>
+          <t>Fortuna Roman Gold Belt</t>
+        </is>
+      </c>
+      <c r="B29" s="181" t="inlineStr">
+        <is>
+          <t>$45,000 OUT 7/21 LOCKED. Mercury native note: Roman Gold Belt. Parked Cost — not sold 2025, not dumped onto Art Sales/Consultant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="181" t="inlineStr">
+        <is>
+          <t>Native CSV 2026-09-20</t>
+        </is>
+      </c>
+      <c r="B30" s="181" t="inlineStr">
+        <is>
+          <t>epgc-llc-transactions-2025-jan-01-to-2025-dec-31.csv is account 8291, same 2025 year already classified. 0 new unique Sent cash vs the 64. Failed Aysel 7/17 and Cancelled Erdal 1/8 are not cash.</t>
         </is>
       </c>
     </row>
@@ -35619,69 +35655,69 @@
     </row>
     <row r="128" ht="14.25" customHeight="1" s="137"/>
     <row r="129" ht="14.25" customHeight="1" s="137">
-      <c r="A129" s="204" t="inlineStr">
-        <is>
-          <t>2025 Mercury ASK — Fortuna inventory remaining (not in Cost total until object is named)</t>
+      <c r="A129" s="201" t="inlineStr">
+        <is>
+          <t>2025 Mercury Fortuna inventory — Venus + Roman Gold Belt LOCKED; Aug $20k unnamed ASK</t>
         </is>
       </c>
     </row>
     <row r="130" ht="14.25" customHeight="1" s="137">
-      <c r="A130" s="200" t="inlineStr">
-        <is>
-          <t>Fortuna / Erdal Dere — object TBD</t>
-        </is>
-      </c>
-      <c r="B130" s="200" t="inlineStr">
+      <c r="A130" s="181" t="inlineStr">
+        <is>
+          <t>Bronze head of a goddess, likely Venus — Fortuna inventory</t>
+        </is>
+      </c>
+      <c r="B130" s="181" t="inlineStr">
         <is>
           <t>Mercury 8291</t>
         </is>
       </c>
-      <c r="C130" s="157" t="n">
+      <c r="C130" s="203" t="n">
         <v>20000</v>
       </c>
-      <c r="D130" s="200" t="inlineStr">
+      <c r="D130" s="202" t="inlineStr">
         <is>
           <t>2025-05-09</t>
         </is>
       </c>
-      <c r="I130" s="0" t="inlineStr">
-        <is>
-          <t>ASK: inventory purchase vs other. Do not add to sold Cost until named (avoid double count).</t>
+      <c r="I130" s="208" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-09-20 from Mercury native CSV note. Parked Cost. Not sold 2025 — not in sold-lot Cost. Not tax advice.</t>
         </is>
       </c>
     </row>
     <row r="131" ht="14.25" customHeight="1" s="137">
-      <c r="A131" s="200" t="inlineStr">
-        <is>
-          <t>Fortuna / Erdal Dere — object TBD</t>
-        </is>
-      </c>
-      <c r="B131" s="200" t="inlineStr">
+      <c r="A131" s="181" t="inlineStr">
+        <is>
+          <t>Roman Gold Belt — Fortuna inventory</t>
+        </is>
+      </c>
+      <c r="B131" s="181" t="inlineStr">
         <is>
           <t>Mercury 8291</t>
         </is>
       </c>
-      <c r="C131" s="157" t="n">
+      <c r="C131" s="203" t="n">
         <v>45000</v>
       </c>
-      <c r="D131" s="200" t="inlineStr">
+      <c r="D131" s="202" t="inlineStr">
         <is>
           <t>2025-07-21</t>
         </is>
       </c>
-      <c r="I131" s="0" t="inlineStr">
-        <is>
-          <t>ASK: inventory purchase vs other. Do not add to sold Cost until named (avoid double count).</t>
+      <c r="I131" s="208" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-09-20 from Mercury native CSV note. Parked Cost. Not sold 2025 — not in sold-lot Cost. Not tax advice.</t>
         </is>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1" s="137">
-      <c r="A132" s="200" t="inlineStr">
-        <is>
-          <t>Fortuna / Erdal Dere — object TBD</t>
-        </is>
-      </c>
-      <c r="B132" s="200" t="inlineStr">
+      <c r="A132" s="185" t="inlineStr">
+        <is>
+          <t>Fortuna / Erdal Dere — object still unnamed (native 8/18 = Monarch 8/15)</t>
+        </is>
+      </c>
+      <c r="B132" s="185" t="inlineStr">
         <is>
           <t>Mercury 8291</t>
         </is>
@@ -35694,20 +35730,20 @@
           <t>2025-08-15</t>
         </is>
       </c>
-      <c r="I132" s="0" t="inlineStr">
-        <is>
-          <t>ASK: inventory purchase vs other. Do not add to sold Cost until named (avoid double count).</t>
+      <c r="I132" s="190" t="inlineStr">
+        <is>
+          <t>ASK: same $20,000 as Mercury native 2025-08-18. No object name. Do not add to sold Cost. Not a second unique txn.</t>
         </is>
       </c>
     </row>
     <row r="133" ht="14.25" customHeight="1" s="137">
       <c r="A133" s="0" t="inlineStr">
         <is>
-          <t>Fortuna remaining 2025 (excl. seals $13,000 already on row 73)</t>
+          <t>Fortuna unnamed remaining 2025 (excl. seals $13,000 + Venus $20,000 + Belt $45,000)</t>
         </is>
       </c>
       <c r="C133" s="157" t="n">
-        <v>85000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="134" ht="14.25" customHeight="1" s="137"/>

</xml_diff>

<commit_message>
Lock 216 Oak Park 2025 costs to last-year Excel pattern.
Amortize Lemonade $42.84/mo, book Rocket/HOA cash plus yellow WAIT 8507 months, and place Brennan, Imelda move-out, Joan painting, and Ace keys on the 216 tab.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
+++ b/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
@@ -648,7 +648,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="216">
+  <cellXfs count="220">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1103,6 +1103,18 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="28" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="24" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="28" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -21138,41 +21150,41 @@
         <f>SUM(P14:AA14)</f>
         <v/>
       </c>
-      <c r="AC14" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD14" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE14" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF14" s="66" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG14" s="66" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH14" s="66" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI14" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ14" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK14" s="68" t="n">
-        <v>0</v>
+      <c r="AC14" s="214" t="n">
+        <v>42.84</v>
+      </c>
+      <c r="AD14" s="214" t="n">
+        <v>42.84</v>
+      </c>
+      <c r="AE14" s="214" t="n">
+        <v>42.84</v>
+      </c>
+      <c r="AF14" s="214" t="n">
+        <v>42.84</v>
+      </c>
+      <c r="AG14" s="214" t="n">
+        <v>42.84</v>
+      </c>
+      <c r="AH14" s="214" t="n">
+        <v>42.84</v>
+      </c>
+      <c r="AI14" s="214" t="n">
+        <v>42.84</v>
+      </c>
+      <c r="AJ14" s="214" t="n">
+        <v>42.84</v>
+      </c>
+      <c r="AK14" s="214" t="n">
+        <v>42.84</v>
       </c>
       <c r="AL14" s="214" t="n">
-        <v>514</v>
-      </c>
-      <c r="AM14" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN14" s="59" t="n">
-        <v>0</v>
+        <v>42.84</v>
+      </c>
+      <c r="AM14" s="214" t="n">
+        <v>42.84</v>
+      </c>
+      <c r="AN14" s="214" t="n">
+        <v>42.84</v>
       </c>
       <c r="AO14" s="61">
         <f>SUM(AC14:AN14)</f>
@@ -21284,8 +21296,8 @@
       <c r="AI15" s="67" t="n">
         <v>0</v>
       </c>
-      <c r="AJ15" s="68" t="n">
-        <v>0</v>
+      <c r="AJ15" s="214" t="n">
+        <v>150</v>
       </c>
       <c r="AK15" s="68" t="n">
         <v>0</v>
@@ -21296,8 +21308,8 @@
       <c r="AM15" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="AN15" s="145" t="n">
-        <v>675</v>
+      <c r="AN15" s="216" t="n">
+        <v>11</v>
       </c>
       <c r="AO15" s="61">
         <f>SUM(AC15:AN15)</f>
@@ -21423,8 +21435,8 @@
       <c r="AM16" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="AN16" s="63" t="n">
-        <v>0</v>
+      <c r="AN16" s="216" t="n">
+        <v>675</v>
       </c>
       <c r="AO16" s="61">
         <f>SUM(AC16:AN16)</f>
@@ -23037,40 +23049,40 @@
         <f>SUM(P29:AA29)</f>
         <v/>
       </c>
-      <c r="AC29" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD29" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE29" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF29" s="65" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG29" s="66" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH29" s="66" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI29" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ29" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK29" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL29" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM29" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN29" s="63" t="n">
+      <c r="AC29" s="147" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD29" s="147" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE29" s="147" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF29" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG29" s="147" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH29" s="147" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI29" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ29" s="147" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK29" s="147" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL29" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM29" s="147" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN29" s="217" t="n">
         <v>0</v>
       </c>
       <c r="AO29" s="61">
@@ -23800,39 +23812,39 @@
         <v/>
       </c>
       <c r="AC35" s="147" t="n">
-        <v>0</v>
+        <v>1226.25</v>
       </c>
       <c r="AD35" s="147" t="n">
-        <v>0</v>
+        <v>1226.25</v>
       </c>
       <c r="AE35" s="147" t="n">
-        <v>0</v>
+        <v>1226.25</v>
       </c>
       <c r="AF35" s="147" t="n">
-        <v>0</v>
+        <v>1226.25</v>
       </c>
       <c r="AG35" s="147" t="n">
-        <v>0</v>
+        <v>1226.25</v>
       </c>
       <c r="AH35" s="147" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI35" s="142" t="n">
         <v>1226.25</v>
       </c>
-      <c r="AJ35" s="142" t="n">
+      <c r="AI35" s="214" t="n">
         <v>1226.25</v>
       </c>
-      <c r="AK35" s="142" t="n">
+      <c r="AJ35" s="214" t="n">
         <v>1226.25</v>
       </c>
-      <c r="AL35" s="142" t="n">
+      <c r="AK35" s="214" t="n">
         <v>1226.25</v>
       </c>
-      <c r="AM35" s="142" t="n">
+      <c r="AL35" s="214" t="n">
+        <v>1226.25</v>
+      </c>
+      <c r="AM35" s="214" t="n">
         <v>1177.52</v>
       </c>
-      <c r="AN35" s="142" t="n">
+      <c r="AN35" s="214" t="n">
         <v>1177.52</v>
       </c>
       <c r="AO35" s="61">
@@ -23927,39 +23939,39 @@
         <v/>
       </c>
       <c r="AC36" s="147" t="n">
-        <v>0</v>
+        <v>421.53</v>
       </c>
       <c r="AD36" s="147" t="n">
-        <v>0</v>
+        <v>421.53</v>
       </c>
       <c r="AE36" s="147" t="n">
-        <v>0</v>
+        <v>421.53</v>
       </c>
       <c r="AF36" s="148" t="n">
-        <v>0</v>
+        <v>421.53</v>
       </c>
       <c r="AG36" s="148" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH36" s="143" t="n">
         <v>421.53</v>
       </c>
-      <c r="AI36" s="143" t="n">
+      <c r="AH36" s="218" t="n">
         <v>421.53</v>
       </c>
-      <c r="AJ36" s="143" t="n">
+      <c r="AI36" s="218" t="n">
         <v>421.53</v>
       </c>
-      <c r="AK36" s="143" t="n">
+      <c r="AJ36" s="218" t="n">
         <v>421.53</v>
       </c>
-      <c r="AL36" s="143" t="n">
+      <c r="AK36" s="218" t="n">
         <v>421.53</v>
       </c>
-      <c r="AM36" s="143" t="n">
+      <c r="AL36" s="218" t="n">
         <v>421.53</v>
       </c>
-      <c r="AN36" s="143" t="n">
+      <c r="AM36" s="218" t="n">
+        <v>421.53</v>
+      </c>
+      <c r="AN36" s="218" t="n">
         <v>421.53</v>
       </c>
       <c r="AO36" s="61">
@@ -24203,8 +24215,8 @@
       <c r="AK38" s="68" t="n">
         <v>0</v>
       </c>
-      <c r="AL38" s="69" t="n">
-        <v>0</v>
+      <c r="AL38" s="218" t="n">
+        <v>300</v>
       </c>
       <c r="AM38" s="59" t="n">
         <v>0</v>
@@ -25022,66 +25034,66 @@
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1" s="137"/>
-    <row r="60" ht="14.25" customHeight="1" s="137">
-      <c r="B60" s="149" t="inlineStr">
-        <is>
-          <t>2025 (this column)</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="32" customHeight="1" s="137">
-      <c r="B61" s="150" t="inlineStr">
-        <is>
-          <t>Rent — filled from joint 0203 (Delach $1,450 + Ava $500; Joan $1,950 Dec + prepaid Jan). Vacant Oct + half Nov. Half-Nov $975 WAIT 8507.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="32" customHeight="1" s="137">
-      <c r="B62" s="150" t="inlineStr">
-        <is>
-          <t>Mortgage — Rocket 8507 Jul–Oct $1,226.25, Nov–Dec $1,177.52. Jan–Jun yellow WAIT 8507 statements (June 8507 in Monarch has no Rocket).</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="14.25" customHeight="1" s="137">
-      <c r="B63" s="150" t="inlineStr">
-        <is>
-          <t>HOA — Santa Maria C326 $421.53 Jun–Dec on 8507. Jan–May yellow WAIT 8507.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="64" customHeight="1" s="137">
+    <row r="60" ht="36" customHeight="1" s="137">
+      <c r="B60" s="215" t="inlineStr">
+        <is>
+          <t>2025 (this column) — user cost list LOCKED 2026-09-20, last-year Excel pattern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="36" customHeight="1" s="137">
+      <c r="B61" s="215" t="inlineStr">
+        <is>
+          <t>Rent — joint 0203 (Delach $1,450 + Ava $500; Joan $1,950 Dec + prepaid Jan). Vacant Oct + half Nov. Half-Nov $975 WAIT 8507.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="48" customHeight="1" s="137">
+      <c r="B62" s="215" t="inlineStr">
+        <is>
+          <t>Mortgage — user $1,226.25/mo. Cash 8507 Jul–Oct $1,226.25 / Nov–Dec $1,177.52 (green). Jan–Jun $1,226.25 yellow WAIT 8507 (not on Monarch). Sch E uses Rocket 1098 interest, not full P+I.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="36" customHeight="1" s="137">
+      <c r="B63" s="215" t="inlineStr">
+        <is>
+          <t>HOA — user $421.53/mo Santa Maria C326. Jun–Dec cash 8507 green. Jan–May $421.53 yellow WAIT 8507.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="48" customHeight="1" s="137">
       <c r="B64" s="215" t="inlineStr">
         <is>
-          <t>LOCKED 2026-09-20: 216 LTR insurance = Lemonade $514.00 cash 10/3 on Megan Chase (1702). Same annual Oct 3 Lemonade as 2023 $321 (= Excel $26.75/mo renter's) and 2024 $421 (≈ Excel $35.08/mo renter's). 2025 books cash in October (not amortized). Travelers = prior 524 Ferdinand home (not 216). Geico = cars. State Farm 2025 bundle = Ferdinand car+home — only home share on 524, not 216. No other Oak Park policy cash on Prime/Sapphire/BoA/0203/8507/Monarch. Not tax advice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="14.25" customHeight="1" s="137">
-      <c r="B65" s="150" t="inlineStr">
-        <is>
-          <t>Interior — 12/1 Zelle to Joan $675 repair (CONFIRMED). CPA may reclass interior vs exterior.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="14.25" customHeight="1" s="137">
-      <c r="B66" s="150" t="inlineStr">
-        <is>
-          <t>Sch E: deduct Rocket 1098 interest, not full P+I. This sheet shows cash mortgage like 2023/2024.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="14.25" customHeight="1" s="137">
-      <c r="B67" s="150" t="inlineStr">
-        <is>
-          <t>Jan 2025 occupancy cash hit 12/31/2024 — not in TY2025. 12/31/2025 $1,950 = Jan 2026 prepaid cash in TY2025.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="14.25" customHeight="1" s="137">
-      <c r="B68" s="150" t="inlineStr">
-        <is>
-          <t>Not tax advice.</t>
+          <t>Insurance — user $42.84/mo × 12 = $514.08 on RENTER'S INSURANCE (amortized like 2023 $26.75 / 2024 $35.08). Lemonade cash $514.00 10/3 Megan Chase (8¢). Not Travelers/Geico/State Farm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="36" customHeight="1" s="137">
+      <c r="B65" s="215" t="inlineStr">
+        <is>
+          <t>Interior — Chris Brennan exterminator $150 8/7 (8507 check posted 8/18) INTERIOR Aug. Ace keys $11 12/8 Megan Chase INTERIOR Dec. Same-day Ace $17 not booked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="36" customHeight="1" s="137">
+      <c r="B66" s="215" t="inlineStr">
+        <is>
+          <t>Interior repair — Joan $675 12/1 8507 Zelle painting + repairs → INTERIOR REPAIR December (2024 used this row for Oak Park painting).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="36" customHeight="1" s="137">
+      <c r="B67" s="215" t="inlineStr">
+        <is>
+          <t>Move-out — Imelda $300 empty-apt. User 9/30; cash 10/1 joint 0203 → MOVE OUT FEE October (same month as 2023/24 $200). Other 2025 Imelda $150s not on 216.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="36" customHeight="1" s="137">
+      <c r="B68" s="219" t="inlineStr">
+        <is>
+          <t>Smoke detector Amazon — still ASK (checklist TBD). No Kidde/First Alert/detector SKU on Monarch/Prime/Sapphire/BoA. EQUIPMENT yellow $0. Not tax advice.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lock Lemonade to 216 Oak Park and Travelers/Geico to 524.
User mapped Lemonade to the 216 LTR (not 827 Grove) and Travelers plus Geico to Ferdinand. Dollars already matched; notes and lock sheets now say so.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
+++ b/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
@@ -7988,7 +7988,7 @@
     <row r="45" ht="72" customHeight="1" s="137">
       <c r="A45" s="213" t="inlineStr">
         <is>
-          <t>2025 columns P–AB. Residence through sale 2025-12-18. MORTGAGE = US Bank loan 09422 monthly P+I from joint 0203 (not $50k extra principal on 9922 Jul/Sep — those are not on this row). HOA n/a. INSURANCE LOCK 2026-09-20: Travelers was prior 524 home; Geico was the cars. Only State Farm HOME share on this INSURANCE line (50/50 with Unit 2). Travelers leftover Jan is 524 home ($0 on cards/Monarch). Auto + Geico credit personal — not EPGC. Not tax advice.</t>
+          <t>2025 columns P–AB. Residence through sale 2025-12-18. MORTGAGE = US Bank loan 09422 monthly P+I from joint 0203 (not $50k extra principal on 9922 Jul/Sep — those are not on this row). HOA n/a. INSURANCE LOCK 2026-09-20: Travelers was prior 524 home; Geico was the cars. Only State Farm HOME share on this INSURANCE line (50/50 with Unit 2). Travelers leftover Jan is 524 home ($0 on cards/Monarch). Auto + Geico credit personal — not EPGC. Not tax advice. User 2026-09-20: Travelers + Geico are 524 Ferdinand; Lemonade is 216 Oak Park (not Grove, not 524).</t>
         </is>
       </c>
       <c r="B45" s="122" t="inlineStr">
@@ -18619,7 +18619,7 @@
     <row r="39" ht="72" customHeight="1" s="137">
       <c r="A39" s="213" t="inlineStr">
         <is>
-          <t>2025: platform STR net on RENTAL INCOME (Jun–Nov). TruGreen/Alsip on YARD SERVICE (same as 2024). Grove Collaborative on SUPPLIES (≠ 827 N Grove the house). INSURANCE LOCK 2026-09-20: Travelers was prior 524 home; Geico was the cars. Only State Farm HOME share on this INSURANCE line (50/50 U1/U2). Auto + Geico $540.89 credit personal, not EPGC. Travelers leftover Jan 2025 is 524 home ($0 on cards/Monarch). ELECTRIC yellow — confirm ComEd with Megan. Not tax advice.</t>
+          <t>2025: platform STR net on RENTAL INCOME (Jun–Nov). TruGreen/Alsip on YARD SERVICE (same as 2024). Grove Collaborative on SUPPLIES (≠ 827 N Grove the house). INSURANCE LOCK 2026-09-20: Travelers was prior 524 home; Geico was the cars. Only State Farm HOME share on this INSURANCE line (50/50 U1/U2). Auto + Geico $540.89 credit personal, not EPGC. Travelers leftover Jan 2025 is 524 home ($0 on cards/Monarch). ELECTRIC yellow — confirm ComEd with Megan. Not tax advice. User 2026-09-20: Travelers + Geico are 524 Ferdinand; Lemonade is 216 Oak Park (not Grove, not 524).</t>
         </is>
       </c>
     </row>
@@ -25065,7 +25065,7 @@
     <row r="64" ht="48" customHeight="1" s="137">
       <c r="B64" s="215" t="inlineStr">
         <is>
-          <t>Insurance — user $42.84/mo × 12 = $514.08 on RENTER'S INSURANCE (amortized like 2023 $26.75 / 2024 $35.08). Lemonade cash $514.00 10/3 Megan Chase (8¢). Not Travelers/Geico/State Farm.</t>
+          <t>Insurance — Lemonade = 216 N. Oak Park #1Z (user: 216, not 524). $42.84/mo × 12 = $514.08 (cash $514.00 10/3 Megan Chase). Travelers + Geico = 524 Ferdinand (home / cars), not 216. Not 827 N Grove. Not tax advice.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Personal Income 2025 formulas so Google Sheets can convert them.
Drop last year's dead external links and #REF defined names, keep real
Excel <f> SUM formulas, and stop the ODS roundtrip that stored =SUM as
text. 2025 numbers and last-year tab layout are unchanged.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
+++ b/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
@@ -1,30 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Income" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="524 Ferdinand Ave, Unit 2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="216 N. Oak Park Ave" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="EPGC LLC" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Refrence Library" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Art Sales and Purchases" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="GCM" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Hindman W2" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Megan T4" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Investments" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="524 Ferdinand Ave, Unit 1" sheetId="11" state="hidden" r:id="rId11"/>
-    <sheet name="2025 Data sources" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="524 Ferdinand Ave, Unit 2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="216 N. Oak Park Ave" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EPGC LLC" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Refrence Library" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Art Sales and Purchases" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GCM" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hindman W2" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Megan T4" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investments" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="524 Ferdinand Ave, Unit 1" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025 Data sources" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId13"/>
-  </externalReferences>
-  <definedNames>
-    <definedName name="a">'Art Sales and Purchases'!$A$3627</definedName>
-    <definedName name="a" localSheetId="1">#REF!</definedName>
-    <definedName name="a" localSheetId="2">#REF!</definedName>
-    <definedName name="a" localSheetId="10">#REF!</definedName>
-  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -705,7 +696,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="232">
+  <cellXfs count="233">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1198,6 +1189,9 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="24" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1271,45 +1265,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook r:id="rId1">
-    <sheetNames>
-      <sheetName val="Property Management Overview"/>
-      <sheetName val="Property 1"/>
-      <sheetName val="Property 2"/>
-      <sheetName val="Property 3"/>
-      <sheetName val="Property 4"/>
-      <sheetName val="Property 5"/>
-      <sheetName val="Property 6"/>
-      <sheetName val="Property 7"/>
-      <sheetName val="Property 8"/>
-      <sheetName val="Property 9"/>
-      <sheetName val="Property 10"/>
-      <sheetName val="Property 11"/>
-      <sheetName val="Property 12"/>
-      <sheetName val="- Disclaimer -"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4740,7 +4695,7 @@
     <row r="9" ht="14.25" customHeight="1" s="137">
       <c r="B9" s="128" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C9" s="32" t="n"/>
@@ -5443,7 +5398,7 @@
     <row r="18" ht="14.25" customHeight="1" s="137">
       <c r="B18" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C18" s="64" t="n">
@@ -5530,7 +5485,7 @@
     <row r="19" ht="14.25" customHeight="1" s="137">
       <c r="B19" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C19" s="64" t="n">
@@ -5617,7 +5572,7 @@
     <row r="20" ht="14.25" customHeight="1" s="137">
       <c r="B20" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C20" s="64" t="n">
@@ -7168,7 +7123,7 @@
     <row r="39" ht="14.25" customHeight="1" s="137">
       <c r="B39" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C39" s="64" t="n">
@@ -7255,7 +7210,7 @@
     <row r="40" ht="14.25" customHeight="1" s="137">
       <c r="B40" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C40" s="64" t="n">
@@ -8671,8 +8626,9 @@
     <row r="999" ht="14.25" customHeight="1" s="137"/>
     <row r="1000" ht="14.25" customHeight="1" s="137"/>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="C1:O1"/>
+    <mergeCell ref="P1:AB1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
@@ -8686,7 +8642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="137" min="1" max="1"/>
@@ -9570,16 +9526,15 @@
     <row r="39">
       <c r="A39" s="229" t="inlineStr">
         <is>
-          <t>524 #2 rent vs Income I6</t>
+          <t>524 #2 Monarch months vs $13,879.55</t>
         </is>
       </c>
       <c r="B39" s="230">
         <f>'524 Ferdinand Ave, Unit 2'!AO5</f>
         <v/>
       </c>
-      <c r="C39" s="230">
-        <f>Income!I6</f>
-        <v/>
+      <c r="C39" s="230" t="n">
+        <v>13879.55</v>
       </c>
       <c r="D39" s="229">
         <f>IF(ROUND(B39,2)=ROUND(C39,2),"MATCH","FAIL")</f>
@@ -9590,16 +9545,15 @@
     <row r="40">
       <c r="A40" s="229" t="inlineStr">
         <is>
-          <t>GCM 2025 vs Income I7</t>
+          <t>Income I6 platform vs $17,086.94</t>
         </is>
       </c>
       <c r="B40" s="230">
-        <f>GCM!E26</f>
-        <v/>
-      </c>
-      <c r="C40" s="230">
-        <f>Income!I7</f>
-        <v/>
+        <f>Income!I6</f>
+        <v/>
+      </c>
+      <c r="C40" s="230" t="n">
+        <v>17086.94</v>
       </c>
       <c r="D40" s="229">
         <f>IF(ROUND(B40,2)=ROUND(C40,2),"MATCH","FAIL")</f>
@@ -9610,15 +9564,16 @@
     <row r="41">
       <c r="A41" s="229" t="inlineStr">
         <is>
-          <t>216 Lemonade vs $514.08</t>
+          <t>GCM 2025 vs Income I7</t>
         </is>
       </c>
       <c r="B41" s="230">
-        <f>'216 N. Oak Park Ave'!AO14</f>
-        <v/>
-      </c>
-      <c r="C41" s="230" t="n">
-        <v>514.08</v>
+        <f>GCM!E26</f>
+        <v/>
+      </c>
+      <c r="C41" s="230">
+        <f>Income!I7</f>
+        <v/>
       </c>
       <c r="D41" s="229">
         <f>IF(ROUND(B41,2)=ROUND(C41,2),"MATCH","FAIL")</f>
@@ -9629,15 +9584,15 @@
     <row r="42">
       <c r="A42" s="229" t="inlineStr">
         <is>
-          <t>EPGC Art Sales vs $150,000</t>
+          <t>216 Lemonade vs $514.08</t>
         </is>
       </c>
       <c r="B42" s="230">
-        <f>'EPGC LLC'!N53</f>
+        <f>'216 N. Oak Park Ave'!AO14</f>
         <v/>
       </c>
       <c r="C42" s="230" t="n">
-        <v>150000</v>
+        <v>514.08</v>
       </c>
       <c r="D42" s="229">
         <f>IF(ROUND(B42,2)=ROUND(C42,2),"MATCH","FAIL")</f>
@@ -9648,15 +9603,15 @@
     <row r="43">
       <c r="A43" s="229" t="inlineStr">
         <is>
-          <t>EPGC Consultant vs $13,595</t>
+          <t>EPGC Art Sales vs $150,000</t>
         </is>
       </c>
       <c r="B43" s="230">
-        <f>'EPGC LLC'!N54</f>
+        <f>'EPGC LLC'!N53</f>
         <v/>
       </c>
       <c r="C43" s="230" t="n">
-        <v>13595</v>
+        <v>150000</v>
       </c>
       <c r="D43" s="229">
         <f>IF(ROUND(B43,2)=ROUND(C43,2),"MATCH","FAIL")</f>
@@ -9664,19 +9619,46 @@
       </c>
       <c r="E43" s="231" t="inlineStr"/>
     </row>
-    <row r="45">
-      <c r="A45" s="184" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="229" t="inlineStr">
+        <is>
+          <t>EPGC Consultant vs $13,595</t>
+        </is>
+      </c>
+      <c r="B44" s="230">
+        <f>'EPGC LLC'!N54</f>
+        <v/>
+      </c>
+      <c r="C44" s="230" t="n">
+        <v>13595</v>
+      </c>
+      <c r="D44" s="229">
+        <f>IF(ROUND(B44,2)=ROUND(C44,2),"MATCH","FAIL")</f>
+        <v/>
+      </c>
+      <c r="E44" s="231" t="inlineStr"/>
+    </row>
+    <row r="45" ht="40" customHeight="1" s="137">
+      <c r="A45" s="232" t="inlineStr">
+        <is>
+          <t>524 #2 STR: Income I6 is Airbnb+VRBO platform net $17,086.94 (CPA). Unit 2 months are Monarch cash Jun–Nov $13,879.55. Gap $3,207.39 = Apr/May platform payouts not in Monarch. Do not invent those months. Not a FAIL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="184" t="inlineStr">
         <is>
           <t>Color key: peach = entered like last year. Green = locked from bank or user. Yellow = WAIT (statement or Cost). Not tax advice.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A45:E45"/>
     <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A46:E46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15025,7 +15007,8 @@
     <row r="994" ht="14.25" customHeight="1" s="137"/>
     <row r="995" ht="14.25" customHeight="1" s="137"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="AC1:AO1"/>
     <mergeCell ref="C1:O1"/>
     <mergeCell ref="P1:AB1"/>
   </mergeCells>
@@ -16890,7 +16873,7 @@
     <row r="17" ht="14.25" customHeight="1" s="137">
       <c r="B17" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C17" s="64" t="n">
@@ -17017,7 +17000,7 @@
     <row r="18" ht="14.25" customHeight="1" s="137">
       <c r="B18" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C18" s="64" t="n">
@@ -17144,7 +17127,7 @@
     <row r="19" ht="14.25" customHeight="1" s="137">
       <c r="B19" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C19" s="64" t="n">
@@ -17271,7 +17254,7 @@
     <row r="20" ht="14.25" customHeight="1" s="137">
       <c r="B20" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C20" s="64" t="n">
@@ -17398,7 +17381,7 @@
     <row r="21" ht="14.25" customHeight="1" s="137">
       <c r="B21" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C21" s="64" t="n">
@@ -17525,7 +17508,7 @@
     <row r="22" ht="14.25" customHeight="1" s="137">
       <c r="B22" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C22" s="64" t="n">
@@ -17652,7 +17635,7 @@
     <row r="23" ht="14.25" customHeight="1" s="137">
       <c r="B23" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C23" s="64" t="n">
@@ -17779,7 +17762,7 @@
     <row r="24" ht="14.25" customHeight="1" s="137">
       <c r="B24" s="57" t="inlineStr">
         <is>
-          <t>  </t>
+          <t xml:space="preserve">  </t>
         </is>
       </c>
       <c r="C24" s="64" t="n">
@@ -17906,7 +17889,7 @@
     <row r="25" ht="14.25" customHeight="1" s="137">
       <c r="B25" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C25" s="64" t="n">
@@ -18033,7 +18016,7 @@
     <row r="26" ht="14.25" customHeight="1" s="137">
       <c r="B26" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C26" s="64" t="n">
@@ -18156,7 +18139,7 @@
     <row r="27" ht="14.25" customHeight="1" s="137">
       <c r="B27" s="57" t="inlineStr">
         <is>
-          <t>  </t>
+          <t xml:space="preserve">  </t>
         </is>
       </c>
       <c r="C27" s="64" t="n">
@@ -18283,7 +18266,7 @@
     <row r="28" ht="14.25" customHeight="1" s="137">
       <c r="B28" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C28" s="64" t="n">
@@ -18537,7 +18520,7 @@
     <row r="30" ht="14.25" customHeight="1" s="137">
       <c r="B30" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C30" s="64" t="n">
@@ -18664,7 +18647,7 @@
     <row r="31" ht="14.25" customHeight="1" s="137">
       <c r="B31" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C31" s="64" t="n">
@@ -18791,7 +18774,7 @@
     <row r="32" ht="14.25" customHeight="1" s="137">
       <c r="B32" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C32" s="64" t="n">
@@ -18918,7 +18901,7 @@
     <row r="33" ht="14.25" customHeight="1" s="137">
       <c r="B33" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C33" s="64" t="n">
@@ -19045,7 +19028,7 @@
     <row r="34" ht="14.25" customHeight="1" s="137">
       <c r="B34" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C34" s="64" t="n">
@@ -19676,7 +19659,7 @@
     <row r="39" ht="14.25" customHeight="1" s="137">
       <c r="B39" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C39" s="64" t="n">
@@ -19803,7 +19786,7 @@
     <row r="40" ht="14.25" customHeight="1" s="137">
       <c r="B40" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C40" s="64" t="n">
@@ -19930,7 +19913,7 @@
     <row r="41" ht="14.25" customHeight="1" s="137">
       <c r="B41" s="57" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C41" s="64" t="n">
@@ -33478,10 +33461,11 @@
     <row r="999" ht="14.25" customHeight="1" s="137"/>
     <row r="1000" ht="14.25" customHeight="1" s="137"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A22:E22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Point Personal Income 2025 at last-year 11-tab Sheet with live formulas.
The live Google Sheet keeps last year's tab names and 2023|2024|2025 year
blocks, fills 2025 numbers, and calculates year totals (Income I10 $151,760).
Packet pointers and START HERE docs now open that one workbook instead of
split-tab files, 2025-only remaps, or formulas-as-text copies.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
+++ b/.cursor/scratch/Personal_Income_2025_Tax_Turbo.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="524 Ferdinand Ave, Unit 2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="216 N. Oak Park Ave" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EPGC LLC" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Refrence Library" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Art Sales and Purchases" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GCM" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hindman W2" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Megan T4" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investments" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="524 Ferdinand Ave, Unit 1" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025 Data sources" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Income" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="524 Ferdinand Ave, Unit 2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="216 N. Oak Park Ave" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="EPGC LLC" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Refrence Library" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Art Sales and Purchases" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="GCM" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Hindman W2" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Megan T4" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Investments" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="524 Ferdinand Ave, Unit 1" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="2025 Data sources" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -696,7 +696,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="233">
+  <cellXfs count="234">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1191,6 +1191,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4695,7 +4698,7 @@
     <row r="9" ht="14.25" customHeight="1" s="137">
       <c r="B9" s="128" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C9" s="32" t="n"/>
@@ -5398,7 +5401,7 @@
     <row r="18" ht="14.25" customHeight="1" s="137">
       <c r="B18" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C18" s="64" t="n">
@@ -5485,7 +5488,7 @@
     <row r="19" ht="14.25" customHeight="1" s="137">
       <c r="B19" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C19" s="64" t="n">
@@ -5572,7 +5575,7 @@
     <row r="20" ht="14.25" customHeight="1" s="137">
       <c r="B20" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C20" s="64" t="n">
@@ -7123,7 +7126,7 @@
     <row r="39" ht="14.25" customHeight="1" s="137">
       <c r="B39" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C39" s="64" t="n">
@@ -7210,7 +7213,7 @@
     <row r="40" ht="14.25" customHeight="1" s="137">
       <c r="B40" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C40" s="64" t="n">
@@ -15085,6 +15088,16 @@
       <c r="M1" s="141" t="n"/>
       <c r="N1" s="141" t="n"/>
       <c r="O1" s="141" t="n"/>
+      <c r="P1" s="233" t="inlineStr">
+        <is>
+          <t>216 N. Oak Park Avenue #1Z</t>
+        </is>
+      </c>
+      <c r="AC1" s="233" t="inlineStr">
+        <is>
+          <t>216 N. Oak Park Avenue #1Z</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1" s="137">
       <c r="A2" s="20" t="n"/>
@@ -16873,7 +16886,7 @@
     <row r="17" ht="14.25" customHeight="1" s="137">
       <c r="B17" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C17" s="64" t="n">
@@ -17000,7 +17013,7 @@
     <row r="18" ht="14.25" customHeight="1" s="137">
       <c r="B18" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C18" s="64" t="n">
@@ -17127,7 +17140,7 @@
     <row r="19" ht="14.25" customHeight="1" s="137">
       <c r="B19" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C19" s="64" t="n">
@@ -17254,7 +17267,7 @@
     <row r="20" ht="14.25" customHeight="1" s="137">
       <c r="B20" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C20" s="64" t="n">
@@ -17381,7 +17394,7 @@
     <row r="21" ht="14.25" customHeight="1" s="137">
       <c r="B21" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C21" s="64" t="n">
@@ -17508,7 +17521,7 @@
     <row r="22" ht="14.25" customHeight="1" s="137">
       <c r="B22" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C22" s="64" t="n">
@@ -17635,7 +17648,7 @@
     <row r="23" ht="14.25" customHeight="1" s="137">
       <c r="B23" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C23" s="64" t="n">
@@ -17762,7 +17775,7 @@
     <row r="24" ht="14.25" customHeight="1" s="137">
       <c r="B24" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">  </t>
+          <t>  </t>
         </is>
       </c>
       <c r="C24" s="64" t="n">
@@ -17889,7 +17902,7 @@
     <row r="25" ht="14.25" customHeight="1" s="137">
       <c r="B25" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C25" s="64" t="n">
@@ -18016,7 +18029,7 @@
     <row r="26" ht="14.25" customHeight="1" s="137">
       <c r="B26" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C26" s="64" t="n">
@@ -18139,7 +18152,7 @@
     <row r="27" ht="14.25" customHeight="1" s="137">
       <c r="B27" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">  </t>
+          <t>  </t>
         </is>
       </c>
       <c r="C27" s="64" t="n">
@@ -18266,7 +18279,7 @@
     <row r="28" ht="14.25" customHeight="1" s="137">
       <c r="B28" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C28" s="64" t="n">
@@ -18520,7 +18533,7 @@
     <row r="30" ht="14.25" customHeight="1" s="137">
       <c r="B30" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C30" s="64" t="n">
@@ -18647,7 +18660,7 @@
     <row r="31" ht="14.25" customHeight="1" s="137">
       <c r="B31" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C31" s="64" t="n">
@@ -18774,7 +18787,7 @@
     <row r="32" ht="14.25" customHeight="1" s="137">
       <c r="B32" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C32" s="64" t="n">
@@ -18901,7 +18914,7 @@
     <row r="33" ht="14.25" customHeight="1" s="137">
       <c r="B33" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C33" s="64" t="n">
@@ -19028,7 +19041,7 @@
     <row r="34" ht="14.25" customHeight="1" s="137">
       <c r="B34" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C34" s="64" t="n">
@@ -19659,7 +19672,7 @@
     <row r="39" ht="14.25" customHeight="1" s="137">
       <c r="B39" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C39" s="64" t="n">
@@ -19786,7 +19799,7 @@
     <row r="40" ht="14.25" customHeight="1" s="137">
       <c r="B40" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C40" s="64" t="n">
@@ -19913,7 +19926,7 @@
     <row r="41" ht="14.25" customHeight="1" s="137">
       <c r="B41" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="C41" s="64" t="n">
@@ -21457,8 +21470,10 @@
     <row r="999" ht="14.25" customHeight="1" s="137"/>
     <row r="1000" ht="14.25" customHeight="1" s="137"/>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
+    <mergeCell ref="AC1:AO1"/>
     <mergeCell ref="C1:O1"/>
+    <mergeCell ref="P1:AB1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>

</xml_diff>